<commit_message>
Lower river unlock cost to 150 so the tutorial reward opens it right away
Update the tutorial finish message, README and balance spreadsheet.
</commit_message>
<xml_diff>
--- a/bukangi-fishing-balance.xlsx
+++ b/bukangi-fishing-balance.xlsx
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B10" s="6" t="n">
         <f aca="false">낚시터!G5</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>12</v>
@@ -4754,7 +4754,7 @@
       </c>
       <c r="G5" s="24" t="n">
         <f aca="false">ROUNDUP((C6-가정!$B$12)/F5,0)</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H5" s="14" t="n">
         <f aca="false">COUNTIFS($A$14:$A$44,B5,$I$14:$I$44,"전설")</f>
@@ -4769,7 +4769,7 @@
         <v>221</v>
       </c>
       <c r="C6" s="12" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>156</v>

</xml_diff>

<commit_message>
Rebalance mid-game, add sound, catch animation and dex rewards
- Boat unlock 6000 -> 4000; 우럭 120 -> 150, 감성돔 380 -> 450 so pier -> boat
  takes about as many fish as river -> pier (53 -> 33 expected catches)
- Synthesized sound effects and phone vibration for cast, bite, hook, reel,
  tension warning, line snap, catch, sell and upgrade, with a sound toggle
- Catch animation: the fish leaps out of the water with grade-based glow,
  light rays, sparkles and a flash for legendary catches (skippable)
- Dex completion rewards: small permanent conveniences per stage
- Spreadsheet: new dex reward sheet; README updated
</commit_message>
<xml_diff>
--- a/bukangi-fishing-balance.xlsx
+++ b/bukangi-fishing-balance.xlsx
@@ -14,6 +14,7 @@
     <sheet name="장비" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="물고기" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="낚시터" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="도감 보상" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -201,7 +202,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="258">
   <si>
     <t xml:space="preserve">부캉이 낚시터 밸런스 요약</t>
   </si>
@@ -264,6 +265,12 @@
   </si>
   <si>
     <t xml:space="preserve">부산 이용권 1장 시간 (초)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">부산 도감 완성 시 +30초</t>
+  </si>
+  <si>
+    <t xml:space="preserve">살림망 칸 수 (실내 도감 완성 시)</t>
   </si>
   <si>
     <t xml:space="preserve">기본 대 적정 구간 (가장 쉬운 붕어)</t>
@@ -924,6 +931,69 @@
   <si>
     <t xml:space="preserve">기대 판매가 기여
 (확률×기대가, 원)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">도감 완성 보상</t>
+  </si>
+  <si>
+    <t xml:space="preserve">낚시터의 물고기를 모두 한 번 이상 잡으면 받는 작은 편의 효과입니다. 부산은 부산 전용 어종 기준입니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">채워야 할 종 수</t>
+  </si>
+  <si>
+    <t xml:space="preserve">보상</t>
+  </si>
+  <si>
+    <t xml:space="preserve">효과 종류</t>
+  </si>
+  <si>
+    <t xml:space="preserve">게임에서 쓰이는 곳</t>
+  </si>
+  <si>
+    <t xml:space="preserve">살림망 +2칸</t>
+  </si>
+  <si>
+    <t xml:space="preserve">net</t>
+  </si>
+  <si>
+    <t xml:space="preserve">살림망 칸 수에 더함</t>
+  </si>
+  <si>
+    <t xml:space="preserve">챔질 판정 10% 넓어짐</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hook</t>
+  </si>
+  <si>
+    <t xml:space="preserve">챔질 게이지 구간·찌 반응 시간에 (1+수치)를 곱함</t>
+  </si>
+  <si>
+    <t xml:space="preserve">느슨함 허용 +0.3초</t>
+  </si>
+  <si>
+    <t xml:space="preserve">slack</t>
+  </si>
+  <si>
+    <t xml:space="preserve">느슨함 허용 시간에 더함</t>
+  </si>
+  <si>
+    <t xml:space="preserve">입질 대기 10% 단축</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wait</t>
+  </si>
+  <si>
+    <t xml:space="preserve">입질 대기 시간에 (1−수치)를 곱함</t>
+  </si>
+  <si>
+    <t xml:space="preserve">부산 이용 시간 +30초</t>
+  </si>
+  <si>
+    <t xml:space="preserve">busan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">부산 이용권 1장 시간에 더함</t>
   </si>
 </sst>
 </file>
@@ -1163,7 +1233,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1293,6 +1363,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="173" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1548,7 +1622,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -1607,7 +1681,7 @@
       </c>
       <c r="B7" s="5" t="n">
         <f aca="false">낚시터!F7</f>
-        <v>114.47175718879</v>
+        <v>122.221537481253</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>6</v>
@@ -1667,7 +1741,7 @@
       </c>
       <c r="B12" s="6" t="n">
         <f aca="false">낚시터!G7</f>
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>12</v>
@@ -1723,39 +1797,51 @@
         <f aca="false">가정!$B$11</f>
         <v>150</v>
       </c>
-      <c r="C17" s="4"/>
+      <c r="C17" s="4" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B18" s="8" t="n">
-        <f aca="false">물고기!R5</f>
-        <v>0.24495</v>
-      </c>
-      <c r="C18" s="4" t="s">
         <v>22</v>
       </c>
+      <c r="B18" s="7" t="n">
+        <f aca="false">가정!$B$4+'도감 보상'!E5</f>
+        <v>17</v>
+      </c>
+      <c r="C18" s="4"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
         <v>23</v>
       </c>
       <c r="B19" s="8" t="n">
+        <f aca="false">물고기!R5</f>
+        <v>0.24495</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" s="8" t="n">
         <f aca="false">물고기!R30</f>
         <v>0.138</v>
       </c>
-      <c r="C19" s="4"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B20" s="8" t="n">
+      <c r="C20" s="4"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21" s="8" t="n">
         <f aca="false">물고기!S30</f>
         <v>0.23575</v>
       </c>
-      <c r="C20" s="4"/>
+      <c r="C21" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1783,12 +1869,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="20.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1799,84 +1885,84 @@
         <v>3</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B4" s="9" t="n">
         <v>15</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B5" s="9" t="n">
         <v>1.8</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B6" s="9" t="n">
         <v>0.6</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B7" s="9" t="n">
         <v>0.35</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B8" s="9" t="n">
         <v>1.5</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B9" s="10" t="n">
         <v>0.004</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B10" s="9" t="n">
         <v>2</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1887,172 +1973,172 @@
         <v>150</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B12" s="9" t="n">
         <v>150</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B13" s="9" t="n">
         <v>30</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B14" s="9" t="n">
         <v>0.5</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B15" s="9" t="n">
         <v>1.15</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B16" s="9" t="n">
         <v>0.88</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B17" s="9" t="n">
         <v>0.88</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B18" s="9" t="n">
         <v>1.12</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B19" s="9" t="n">
         <v>0.24</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B20" s="9" t="n">
         <v>0.36</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B21" s="9" t="n">
         <v>0.75</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B22" s="9" t="n">
         <v>0.9</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B23" s="9" t="n">
         <v>2.2</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B24" s="9" t="n">
         <v>0.7</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B25" s="9" t="n">
         <v>0.05</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B26" s="9" t="n">
         <v>0.12</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -2082,37 +2168,37 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B4" s="12" t="n">
         <v>0</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D4" s="14" t="n">
         <f aca="false">COUNTIF(물고기!$O$5:$O$40,A4)</f>
@@ -2121,13 +2207,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B5" s="12" t="n">
         <v>60</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D5" s="14" t="n">
         <f aca="false">COUNTIF(물고기!$O$5:$O$40,A5)</f>
@@ -2136,13 +2222,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B6" s="12" t="n">
         <v>200</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D6" s="14" t="n">
         <f aca="false">COUNTIF(물고기!$O$5:$O$40,A6)</f>
@@ -2151,13 +2237,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B7" s="12" t="n">
         <v>700</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D7" s="14" t="n">
         <f aca="false">COUNTIF(물고기!$O$5:$O$40,A7)</f>
@@ -2166,13 +2252,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B8" s="12" t="n">
         <v>2500</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D8" s="14" t="n">
         <f aca="false">COUNTIF(물고기!$O$5:$O$40,A8)</f>
@@ -2181,13 +2267,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -2220,52 +2306,52 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B5" s="14" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D5" s="12" t="n">
         <v>0</v>
@@ -2278,18 +2364,18 @@
         <v>0.24</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B6" s="14" t="n">
         <v>2</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D6" s="12" t="n">
         <v>200</v>
@@ -2302,18 +2388,18 @@
         <v>0.28</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B7" s="14" t="n">
         <v>3</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D7" s="12" t="n">
         <v>1200</v>
@@ -2326,18 +2412,18 @@
         <v>0.32</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B8" s="14" t="n">
         <v>4</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D8" s="12" t="n">
         <v>6000</v>
@@ -2350,18 +2436,18 @@
         <v>0.36</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B9" s="14" t="n">
         <v>5</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D9" s="12" t="n">
         <v>25000</v>
@@ -2374,18 +2460,18 @@
         <v>0.41</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B10" s="14" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D10" s="12" t="n">
         <v>0</v>
@@ -2398,18 +2484,18 @@
         <v>0.16</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B11" s="14" t="n">
         <v>2</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D11" s="12" t="n">
         <v>250</v>
@@ -2422,18 +2508,18 @@
         <v>0.21</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B12" s="14" t="n">
         <v>3</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D12" s="12" t="n">
         <v>1500</v>
@@ -2446,18 +2532,18 @@
         <v>0.27</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B13" s="14" t="n">
         <v>4</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D13" s="12" t="n">
         <v>7000</v>
@@ -2470,18 +2556,18 @@
         <v>0.34</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B14" s="14" t="n">
         <v>5</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D14" s="12" t="n">
         <v>30000</v>
@@ -2494,18 +2580,18 @@
         <v>0.42</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B15" s="14" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D15" s="12" t="n">
         <v>0</v>
@@ -2518,18 +2604,18 @@
         <v>1.2</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B16" s="14" t="n">
         <v>2</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D16" s="12" t="n">
         <v>150</v>
@@ -2542,18 +2628,18 @@
         <v>1.7</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B17" s="14" t="n">
         <v>3</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D17" s="12" t="n">
         <v>1000</v>
@@ -2566,18 +2652,18 @@
         <v>2.4</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B18" s="14" t="n">
         <v>4</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D18" s="12" t="n">
         <v>5000</v>
@@ -2590,18 +2676,18 @@
         <v>3.3</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B19" s="14" t="n">
         <v>5</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D19" s="12" t="n">
         <v>22000</v>
@@ -2614,18 +2700,18 @@
         <v>4.5</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B20" s="14" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D20" s="12" t="n">
         <v>0</v>
@@ -2638,7 +2724,7 @@
         <v>0</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="H20" s="23" t="n">
         <f aca="false">가정!$B$9*(1+F20*가정!$B$10)</f>
@@ -2651,13 +2737,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B21" s="14" t="n">
         <v>2</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D21" s="12" t="n">
         <v>100</v>
@@ -2670,7 +2756,7 @@
         <v>0.15</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="H21" s="23" t="n">
         <f aca="false">가정!$B$9*(1+F21*가정!$B$10)</f>
@@ -2683,13 +2769,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B22" s="14" t="n">
         <v>3</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D22" s="12" t="n">
         <v>800</v>
@@ -2702,7 +2788,7 @@
         <v>0.3</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="H22" s="23" t="n">
         <f aca="false">가정!$B$9*(1+F22*가정!$B$10)</f>
@@ -2715,13 +2801,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B23" s="14" t="n">
         <v>4</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D23" s="12" t="n">
         <v>4500</v>
@@ -2734,7 +2820,7 @@
         <v>0.5</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="H23" s="23" t="n">
         <f aca="false">가정!$B$9*(1+F23*가정!$B$10)</f>
@@ -2747,13 +2833,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B24" s="14" t="n">
         <v>5</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D24" s="12" t="n">
         <v>20000</v>
@@ -2766,7 +2852,7 @@
         <v>0.8</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="H24" s="23" t="n">
         <f aca="false">가정!$B$9*(1+F24*가정!$B$10)</f>
@@ -2779,7 +2865,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C25" s="25" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D25" s="26" t="n">
         <f aca="false">SUM(D5:D24)</f>
@@ -2822,82 +2908,82 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="Q4" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="S4" s="3" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="9" t="n">
@@ -2959,13 +3045,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B6" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="C6" s="11" t="s">
         <v>158</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>156</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="9" t="n">
@@ -3027,13 +3113,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D7" s="4"/>
       <c r="E7" s="9" t="n">
@@ -3095,13 +3181,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D8" s="4"/>
       <c r="E8" s="9" t="n">
@@ -3163,13 +3249,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D9" s="4"/>
       <c r="E9" s="9" t="n">
@@ -3231,13 +3317,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B10" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="C10" s="11" t="s">
         <v>167</v>
-      </c>
-      <c r="C10" s="11" t="s">
-        <v>165</v>
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="9" t="n">
@@ -3299,13 +3385,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D11" s="4"/>
       <c r="E11" s="9" t="n">
@@ -3367,13 +3453,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D12" s="4"/>
       <c r="E12" s="9" t="n">
@@ -3435,13 +3521,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D13" s="4"/>
       <c r="E13" s="9" t="n">
@@ -3503,13 +3589,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D14" s="4"/>
       <c r="E14" s="9" t="n">
@@ -3571,13 +3657,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D15" s="4"/>
       <c r="E15" s="9" t="n">
@@ -3639,13 +3725,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D16" s="4"/>
       <c r="E16" s="9" t="n">
@@ -3655,7 +3741,7 @@
         <v>50</v>
       </c>
       <c r="G16" s="12" t="n">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="H16" s="22" t="n">
         <v>0.45</v>
@@ -3666,15 +3752,15 @@
       </c>
       <c r="J16" s="20" t="n">
         <f aca="false">MAX(1,ROUND(G16*(E16/I16)^2,0))</f>
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="K16" s="20" t="n">
         <f aca="false">MAX(1,ROUND(G16*(F16/I16)^2,0))</f>
-        <v>245</v>
+        <v>306</v>
       </c>
       <c r="L16" s="20" t="n">
         <f aca="false">G16*(E16^2+2*E16*(F16-E16)/(1+가정!$B$5)+(F16-E16)^2/(1+2*가정!$B$5))/I16^2</f>
-        <v>100.332107998479</v>
+        <v>125.415134998099</v>
       </c>
       <c r="M16" s="4" t="str">
         <f aca="false">INDEX(등급!$A$4:$A$8,MATCH(J16,등급!$B$4:$B$8,1))</f>
@@ -3707,13 +3793,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D17" s="4"/>
       <c r="E17" s="9" t="n">
@@ -3723,7 +3809,7 @@
         <v>60</v>
       </c>
       <c r="G17" s="12" t="n">
-        <v>380</v>
+        <v>450</v>
       </c>
       <c r="H17" s="22" t="n">
         <v>0.6</v>
@@ -3734,15 +3820,15 @@
       </c>
       <c r="J17" s="20" t="n">
         <f aca="false">MAX(1,ROUND(G17*(E17/I17)^2,0))</f>
-        <v>131</v>
+        <v>156</v>
       </c>
       <c r="K17" s="20" t="n">
         <f aca="false">MAX(1,ROUND(G17*(F17/I17)^2,0))</f>
-        <v>757</v>
+        <v>897</v>
       </c>
       <c r="L17" s="20" t="n">
         <f aca="false">G17*(E17^2+2*E17*(F17-E17)/(1+가정!$B$5)+(F17-E17)^2/(1+2*가정!$B$5))/I17^2</f>
-        <v>319.001053106665</v>
+        <v>377.764404994735</v>
       </c>
       <c r="M17" s="4" t="str">
         <f aca="false">INDEX(등급!$A$4:$A$8,MATCH(J17,등급!$B$4:$B$8,1))</f>
@@ -3775,13 +3861,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D18" s="4"/>
       <c r="E18" s="9" t="n">
@@ -3843,13 +3929,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D19" s="4"/>
       <c r="E19" s="9" t="n">
@@ -3911,13 +3997,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D20" s="4"/>
       <c r="E20" s="9" t="n">
@@ -3979,13 +4065,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D21" s="4"/>
       <c r="E21" s="9" t="n">
@@ -4047,13 +4133,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D22" s="4"/>
       <c r="E22" s="9" t="n">
@@ -4115,13 +4201,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D23" s="4"/>
       <c r="E23" s="9" t="n">
@@ -4183,13 +4269,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D24" s="4"/>
       <c r="E24" s="9" t="n">
@@ -4251,13 +4337,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D25" s="4"/>
       <c r="E25" s="9" t="n">
@@ -4319,13 +4405,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D26" s="4"/>
       <c r="E26" s="9" t="n">
@@ -4387,16 +4473,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="E27" s="9" t="n">
         <v>30</v>
@@ -4457,16 +4543,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B28" s="11" t="s">
+        <v>206</v>
+      </c>
+      <c r="C28" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="D28" s="4" t="s">
         <v>204</v>
-      </c>
-      <c r="C28" s="11" t="s">
-        <v>165</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>202</v>
       </c>
       <c r="E28" s="9" t="n">
         <v>90</v>
@@ -4527,16 +4613,16 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="E29" s="9" t="n">
         <v>50</v>
@@ -4597,16 +4683,16 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="E30" s="9" t="n">
         <v>100</v>
@@ -4697,52 +4783,52 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C5" s="12" t="n">
         <v>0</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E5" s="14" t="n">
         <f aca="false">COUNTIF($A$14:$A$44,B5)</f>
@@ -4763,16 +4849,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C6" s="12" t="n">
         <v>150</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E6" s="14" t="n">
         <f aca="false">COUNTIF($A$14:$A$44,B6)</f>
@@ -4793,16 +4879,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C7" s="12" t="n">
         <v>1500</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E7" s="14" t="n">
         <f aca="false">COUNTIF($A$14:$A$44,B7)</f>
@@ -4810,11 +4896,11 @@
       </c>
       <c r="F7" s="20" t="n">
         <f aca="false">SUMIF($A$14:$A$44,B7,$G$14:$G$44)</f>
-        <v>114.47175718879</v>
+        <v>122.221537481253</v>
       </c>
       <c r="G7" s="24" t="n">
         <f aca="false">ROUNDUP(C8/F7,0)</f>
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="H7" s="14" t="n">
         <f aca="false">COUNTIFS($A$14:$A$44,B7,$I$14:$I$44,"전설")</f>
@@ -4823,16 +4909,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C8" s="12" t="n">
-        <v>6000</v>
+        <v>4000</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="E8" s="14" t="n">
         <f aca="false">COUNTIF($A$14:$A$44,B8)</f>
@@ -4843,7 +4929,7 @@
         <v>758.269279988315</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="H8" s="14" t="n">
         <f aca="false">COUNTIFS($A$14:$A$44,B8,$I$14:$I$44,"전설")</f>
@@ -4852,16 +4938,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="E9" s="14" t="n">
         <f aca="false">COUNTIF($A$14:$A$44,B9)</f>
@@ -4872,7 +4958,7 @@
         <v>1944.80772047492</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="H9" s="14" t="n">
         <f aca="false">COUNTIFS($A$14:$A$44,B9,$I$14:$I$44,"전설")</f>
@@ -4881,44 +4967,44 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="30" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C14" s="31" t="str">
         <f aca="false">물고기!B5</f>
@@ -4950,10 +5036,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C15" s="31" t="str">
         <f aca="false">물고기!B6</f>
@@ -4985,10 +5071,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C16" s="31" t="str">
         <f aca="false">물고기!B7</f>
@@ -5020,10 +5106,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C17" s="31" t="str">
         <f aca="false">물고기!B8</f>
@@ -5055,10 +5141,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C18" s="31" t="str">
         <f aca="false">물고기!B5</f>
@@ -5090,10 +5176,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C19" s="31" t="str">
         <f aca="false">물고기!B7</f>
@@ -5125,10 +5211,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C20" s="31" t="str">
         <f aca="false">물고기!B9</f>
@@ -5160,10 +5246,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C21" s="31" t="str">
         <f aca="false">물고기!B10</f>
@@ -5195,10 +5281,10 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C22" s="31" t="str">
         <f aca="false">물고기!B11</f>
@@ -5230,10 +5316,10 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C23" s="31" t="str">
         <f aca="false">물고기!B12</f>
@@ -5265,10 +5351,10 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C24" s="31" t="str">
         <f aca="false">물고기!B13</f>
@@ -5300,10 +5386,10 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C25" s="31" t="str">
         <f aca="false">물고기!B14</f>
@@ -5335,10 +5421,10 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C26" s="31" t="str">
         <f aca="false">물고기!B15</f>
@@ -5370,10 +5456,10 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C27" s="31" t="str">
         <f aca="false">물고기!B16</f>
@@ -5392,11 +5478,11 @@
       </c>
       <c r="G27" s="20" t="n">
         <f aca="false">F27*H27</f>
-        <v>12.1003547334849</v>
+        <v>15.1254434168561</v>
       </c>
       <c r="H27" s="5" t="n">
         <f aca="false">물고기!L16</f>
-        <v>100.332107998479</v>
+        <v>125.415134998099</v>
       </c>
       <c r="I27" s="31" t="str">
         <f aca="false">물고기!O16</f>
@@ -5405,10 +5491,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C28" s="31" t="str">
         <f aca="false">물고기!B17</f>
@@ -5427,11 +5513,11 @@
       </c>
       <c r="G28" s="20" t="n">
         <f aca="false">F28*H28</f>
-        <v>25.6483258779228</v>
+        <v>30.3730174870138</v>
       </c>
       <c r="H28" s="5" t="n">
         <f aca="false">물고기!L17</f>
-        <v>319.001053106665</v>
+        <v>377.764404994735</v>
       </c>
       <c r="I28" s="31" t="str">
         <f aca="false">물고기!O17</f>
@@ -5440,10 +5526,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C29" s="31" t="str">
         <f aca="false">물고기!B18</f>
@@ -5475,10 +5561,10 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C30" s="31" t="str">
         <f aca="false">물고기!B19</f>
@@ -5510,10 +5596,10 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C31" s="31" t="str">
         <f aca="false">물고기!B20</f>
@@ -5545,10 +5631,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C32" s="31" t="str">
         <f aca="false">물고기!B21</f>
@@ -5580,10 +5666,10 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C33" s="31" t="str">
         <f aca="false">물고기!B22</f>
@@ -5615,10 +5701,10 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C34" s="31" t="str">
         <f aca="false">물고기!B23</f>
@@ -5650,10 +5736,10 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C35" s="31" t="str">
         <f aca="false">물고기!B24</f>
@@ -5685,10 +5771,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C36" s="31" t="str">
         <f aca="false">물고기!B25</f>
@@ -5720,10 +5806,10 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C37" s="31" t="str">
         <f aca="false">물고기!B26</f>
@@ -5755,10 +5841,10 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C38" s="31" t="str">
         <f aca="false">물고기!B23</f>
@@ -5790,10 +5876,10 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C39" s="31" t="str">
         <f aca="false">물고기!B24</f>
@@ -5825,10 +5911,10 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C40" s="31" t="str">
         <f aca="false">물고기!B25</f>
@@ -5860,10 +5946,10 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C41" s="31" t="str">
         <f aca="false">물고기!B28</f>
@@ -5895,10 +5981,10 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C42" s="31" t="str">
         <f aca="false">물고기!B27</f>
@@ -5930,10 +6016,10 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C43" s="31" t="str">
         <f aca="false">물고기!B29</f>
@@ -5965,10 +6051,10 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C44" s="31" t="str">
         <f aca="false">물고기!B30</f>
@@ -6008,4 +6094,161 @@
   </headerFooter>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="48"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="B5" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>243</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="E5" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="B6" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>246</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="B7" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="E7" s="32" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="B8" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>252</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="E8" s="21" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>255</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="E9" s="33" t="n">
+        <v>30</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>257</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add timed casting with distance-based rarity, and quick sell
- Casting: first press starts a distance gauge, second press casts (12-40 m).
  Far casts raise the weight of pricier fish, near casts lower it
  (boat expected price ~590 / 760 / 960 for near / middle / far), and far
  casts start the fight farther away (x1.15) for more risk
- Quick sell button on the catch result
- Spreadsheet: casting assumptions and near/far expected prices; README
</commit_message>
<xml_diff>
--- a/bukangi-fishing-balance.xlsx
+++ b/bukangi-fishing-balance.xlsx
@@ -202,7 +202,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="258">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="279">
   <si>
     <t xml:space="preserve">부캉이 낚시터 밸런스 요약</t>
   </si>
@@ -264,6 +264,18 @@
     <t xml:space="preserve">부캉이까지 기대 입질 수 (황금 미끼)</t>
   </si>
   <si>
+    <t xml:space="preserve">배낚시 기대 판매가: 가장 가까이 (원)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">캐스팅 게이지 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">배낚시 기대 판매가: 가장 멀리 (원)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">캐스팅 게이지 끝</t>
+  </si>
+  <si>
     <t xml:space="preserve">부산 이용권 1장 시간 (초)</t>
   </si>
   <si>
@@ -421,6 +433,36 @@
   </si>
   <si>
     <t xml:space="preserve">난이도: 크기 가중</t>
+  </si>
+  <si>
+    <t xml:space="preserve">캐스팅 등급 배율</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONFIG.cast.gradeBias — 가중치 × (1+배율)^((파워−0.5)×2×기준등급번호). 파워 0.5면 변화 없음</t>
+  </si>
+  <si>
+    <t xml:space="preserve">가장 가까이 표시 거리 (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONFIG.cast.nearM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">가장 멀리 표시 거리 (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONFIG.cast.farM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">가까이 던졌을 때 시작 거리 배수</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONFIG.cast.startDistNear — 걸린 뒤 끌어올 거리</t>
+  </si>
+  <si>
+    <t xml:space="preserve">멀리 던졌을 때 시작 거리 배수</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONFIG.cast.startDistFar — 도망 거리(1.3)에 더 가까워 위험↑</t>
   </si>
   <si>
     <t xml:space="preserve">등급 기준</t>
@@ -687,6 +729,10 @@
 최고 대·최대 난이도</t>
   </si>
   <si>
+    <t xml:space="preserve">기준가 등급
+번호 (출현 가중)</t>
+  </si>
+  <si>
     <t xml:space="preserve">bungeo</t>
   </si>
   <si>
@@ -881,6 +927,14 @@
 나올 수 있는 종</t>
   </si>
   <si>
+    <t xml:space="preserve">기대 판매가
+가장 가까이 (원)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">기대 판매가
+가장 멀리 (원)</t>
+  </si>
+  <si>
     <t xml:space="preserve">0</t>
   </si>
   <si>
@@ -931,6 +985,22 @@
   <si>
     <t xml:space="preserve">기대 판매가 기여
 (확률×기대가, 원)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">가중치
+가장 가까이</t>
+  </si>
+  <si>
+    <t xml:space="preserve">가중치
+가장 멀리</t>
+  </si>
+  <si>
+    <t xml:space="preserve">기여
+가장 가까이 (원)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">기여
+가장 멀리 (원)</t>
   </si>
   <si>
     <t xml:space="preserve">도감 완성 보상</t>
@@ -1622,7 +1692,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -1793,9 +1863,9 @@
       <c r="A17" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="7" t="n">
-        <f aca="false">가정!$B$11</f>
-        <v>150</v>
+      <c r="B17" s="5" t="n">
+        <f aca="false">낚시터!I8</f>
+        <v>588.258441092311</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>21</v>
@@ -1805,43 +1875,67 @@
       <c r="A18" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="7" t="n">
+      <c r="B18" s="5" t="n">
+        <f aca="false">낚시터!J8</f>
+        <v>959.735272708961</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" s="7" t="n">
+        <f aca="false">가정!$B$11</f>
+        <v>150</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="7" t="n">
         <f aca="false">가정!$B$4+'도감 보상'!E5</f>
         <v>17</v>
       </c>
-      <c r="C18" s="4"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B19" s="8" t="n">
+      <c r="C20" s="4"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B21" s="8" t="n">
         <f aca="false">물고기!R5</f>
         <v>0.24495</v>
       </c>
-      <c r="C19" s="4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B20" s="8" t="n">
+      <c r="C21" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B22" s="8" t="n">
         <f aca="false">물고기!R30</f>
         <v>0.138</v>
       </c>
-      <c r="C20" s="4"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B21" s="8" t="n">
+      <c r="C22" s="4"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23" s="8" t="n">
         <f aca="false">물고기!S30</f>
         <v>0.23575</v>
       </c>
-      <c r="C21" s="4"/>
+      <c r="C23" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1859,7 +1953,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -1869,12 +1963,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="20.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1885,260 +1979,315 @@
         <v>3</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B4" s="9" t="n">
         <v>15</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B5" s="9" t="n">
         <v>1.8</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B6" s="9" t="n">
         <v>0.6</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B7" s="9" t="n">
         <v>0.35</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B8" s="9" t="n">
         <v>1.5</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B9" s="10" t="n">
         <v>0.004</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="B10" s="9" t="n">
         <v>2</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B11" s="9" t="n">
         <v>150</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B12" s="9" t="n">
         <v>150</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B13" s="9" t="n">
         <v>30</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B14" s="9" t="n">
         <v>0.5</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B15" s="9" t="n">
         <v>1.15</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B16" s="9" t="n">
         <v>0.88</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B17" s="9" t="n">
         <v>0.88</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B18" s="9" t="n">
         <v>1.12</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B19" s="9" t="n">
         <v>0.24</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B20" s="9" t="n">
         <v>0.36</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B21" s="9" t="n">
         <v>0.75</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B22" s="9" t="n">
         <v>0.9</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B23" s="9" t="n">
         <v>2.2</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B24" s="9" t="n">
         <v>0.7</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B25" s="9" t="n">
         <v>0.05</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B26" s="9" t="n">
         <v>0.12</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>66</v>
+        <v>70</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B27" s="9" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B28" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B29" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B30" s="9" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B31" s="9" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -2168,37 +2317,37 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>73</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>75</v>
+        <v>89</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>76</v>
+        <v>90</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>77</v>
+        <v>91</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>78</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>79</v>
+        <v>93</v>
       </c>
       <c r="B4" s="12" t="n">
         <v>0</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="D4" s="14" t="n">
         <f aca="false">COUNTIF(물고기!$O$5:$O$40,A4)</f>
@@ -2207,13 +2356,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="B5" s="12" t="n">
         <v>60</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="D5" s="14" t="n">
         <f aca="false">COUNTIF(물고기!$O$5:$O$40,A5)</f>
@@ -2222,13 +2371,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>83</v>
+        <v>97</v>
       </c>
       <c r="B6" s="12" t="n">
         <v>200</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>84</v>
+        <v>98</v>
       </c>
       <c r="D6" s="14" t="n">
         <f aca="false">COUNTIF(물고기!$O$5:$O$40,A6)</f>
@@ -2237,13 +2386,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>85</v>
+        <v>99</v>
       </c>
       <c r="B7" s="12" t="n">
         <v>700</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>86</v>
+        <v>100</v>
       </c>
       <c r="D7" s="14" t="n">
         <f aca="false">COUNTIF(물고기!$O$5:$O$40,A7)</f>
@@ -2252,13 +2401,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="B8" s="12" t="n">
         <v>2500</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>88</v>
+        <v>102</v>
       </c>
       <c r="D8" s="14" t="n">
         <f aca="false">COUNTIF(물고기!$O$5:$O$40,A8)</f>
@@ -2267,13 +2416,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>89</v>
+        <v>103</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>91</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -2306,52 +2455,52 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>92</v>
+        <v>106</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>93</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>95</v>
+        <v>109</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>100</v>
+        <v>114</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>102</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="B5" s="14" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="D5" s="12" t="n">
         <v>0</v>
@@ -2364,18 +2513,18 @@
         <v>0.24</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="B6" s="14" t="n">
         <v>2</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="D6" s="12" t="n">
         <v>200</v>
@@ -2388,18 +2537,18 @@
         <v>0.28</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="B7" s="14" t="n">
         <v>3</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="D7" s="12" t="n">
         <v>1200</v>
@@ -2412,18 +2561,18 @@
         <v>0.32</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="B8" s="14" t="n">
         <v>4</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="D8" s="12" t="n">
         <v>6000</v>
@@ -2436,18 +2585,18 @@
         <v>0.36</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>111</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="B9" s="14" t="n">
         <v>5</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="D9" s="12" t="n">
         <v>25000</v>
@@ -2460,18 +2609,18 @@
         <v>0.41</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
       <c r="B10" s="14" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
       <c r="D10" s="12" t="n">
         <v>0</v>
@@ -2484,18 +2633,18 @@
         <v>0.16</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>116</v>
+        <v>130</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
       <c r="B11" s="14" t="n">
         <v>2</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="D11" s="12" t="n">
         <v>250</v>
@@ -2508,18 +2657,18 @@
         <v>0.21</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>116</v>
+        <v>130</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
       <c r="B12" s="14" t="n">
         <v>3</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="D12" s="12" t="n">
         <v>1500</v>
@@ -2532,18 +2681,18 @@
         <v>0.27</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>116</v>
+        <v>130</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
       <c r="B13" s="14" t="n">
         <v>4</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="D13" s="12" t="n">
         <v>7000</v>
@@ -2556,18 +2705,18 @@
         <v>0.34</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>116</v>
+        <v>130</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
       <c r="B14" s="14" t="n">
         <v>5</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="D14" s="12" t="n">
         <v>30000</v>
@@ -2580,18 +2729,18 @@
         <v>0.42</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>116</v>
+        <v>130</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="B15" s="14" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
       <c r="D15" s="12" t="n">
         <v>0</v>
@@ -2604,18 +2753,18 @@
         <v>1.2</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="B16" s="14" t="n">
         <v>2</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="D16" s="12" t="n">
         <v>150</v>
@@ -2628,18 +2777,18 @@
         <v>1.7</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="B17" s="14" t="n">
         <v>3</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="D17" s="12" t="n">
         <v>1000</v>
@@ -2652,18 +2801,18 @@
         <v>2.4</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="B18" s="14" t="n">
         <v>4</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="D18" s="12" t="n">
         <v>5000</v>
@@ -2676,18 +2825,18 @@
         <v>3.3</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="B19" s="14" t="n">
         <v>5</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>127</v>
+        <v>141</v>
       </c>
       <c r="D19" s="12" t="n">
         <v>22000</v>
@@ -2700,18 +2849,18 @@
         <v>4.5</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="B20" s="14" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="D20" s="12" t="n">
         <v>0</v>
@@ -2724,7 +2873,7 @@
         <v>0</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="H20" s="23" t="n">
         <f aca="false">가정!$B$9*(1+F20*가정!$B$10)</f>
@@ -2737,13 +2886,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="B21" s="14" t="n">
         <v>2</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>131</v>
+        <v>145</v>
       </c>
       <c r="D21" s="12" t="n">
         <v>100</v>
@@ -2756,7 +2905,7 @@
         <v>0.15</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="H21" s="23" t="n">
         <f aca="false">가정!$B$9*(1+F21*가정!$B$10)</f>
@@ -2769,13 +2918,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="B22" s="14" t="n">
         <v>3</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="D22" s="12" t="n">
         <v>800</v>
@@ -2788,7 +2937,7 @@
         <v>0.3</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="H22" s="23" t="n">
         <f aca="false">가정!$B$9*(1+F22*가정!$B$10)</f>
@@ -2801,13 +2950,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="B23" s="14" t="n">
         <v>4</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
       <c r="D23" s="12" t="n">
         <v>4500</v>
@@ -2820,7 +2969,7 @@
         <v>0.5</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="H23" s="23" t="n">
         <f aca="false">가정!$B$9*(1+F23*가정!$B$10)</f>
@@ -2833,13 +2982,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="B24" s="14" t="n">
         <v>5</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>134</v>
+        <v>148</v>
       </c>
       <c r="D24" s="12" t="n">
         <v>20000</v>
@@ -2852,7 +3001,7 @@
         <v>0.8</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="H24" s="23" t="n">
         <f aca="false">가정!$B$9*(1+F24*가정!$B$10)</f>
@@ -2865,7 +3014,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C25" s="25" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
       <c r="D25" s="26" t="n">
         <f aca="false">SUM(D5:D24)</f>
@@ -2888,7 +3037,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:S30"/>
+  <dimension ref="A1:T30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -2903,87 +3052,90 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="13" style="0" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="16" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="18" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="18" style="0" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>136</v>
+        <v>150</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>137</v>
+        <v>151</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>138</v>
+        <v>152</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>139</v>
+        <v>153</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>141</v>
+        <v>155</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>142</v>
+        <v>156</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>143</v>
+        <v>157</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>144</v>
+        <v>158</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>145</v>
+        <v>159</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>146</v>
+        <v>160</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>147</v>
+        <v>161</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>149</v>
+        <v>163</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>150</v>
+        <v>164</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="Q4" s="3" t="s">
-        <v>153</v>
+        <v>167</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>154</v>
+        <v>168</v>
       </c>
       <c r="S4" s="3" t="s">
-        <v>155</v>
+        <v>169</v>
+      </c>
+      <c r="T4" s="3" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>156</v>
+        <v>171</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>157</v>
+        <v>172</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>158</v>
+        <v>173</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="9" t="n">
@@ -3042,16 +3194,20 @@
         <f aca="false">장비!$F$9*(1-Q5*가정!$B$14)*가정!$B$15</f>
         <v>0.41845625</v>
       </c>
+      <c r="T5" s="14" t="n">
+        <f aca="false">MATCH(G5,등급!$B$4:$B$8,1)-1</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>159</v>
+        <v>174</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>160</v>
+        <v>175</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>158</v>
+        <v>173</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="9" t="n">
@@ -3110,16 +3266,20 @@
         <f aca="false">장비!$F$9*(1-Q6*가정!$B$14)*가정!$B$15</f>
         <v>0.3937025</v>
       </c>
+      <c r="T6" s="14" t="n">
+        <f aca="false">MATCH(G6,등급!$B$4:$B$8,1)-1</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>161</v>
+        <v>176</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>162</v>
+        <v>177</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>158</v>
+        <v>173</v>
       </c>
       <c r="D7" s="4"/>
       <c r="E7" s="9" t="n">
@@ -3178,16 +3338,20 @@
         <f aca="false">장비!$F$9*(1-Q7*가정!$B$14)*가정!$B$15</f>
         <v>0.35716125</v>
       </c>
+      <c r="T7" s="14" t="n">
+        <f aca="false">MATCH(G7,등급!$B$4:$B$8,1)-1</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>163</v>
+        <v>178</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>164</v>
+        <v>179</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>158</v>
+        <v>173</v>
       </c>
       <c r="D8" s="4"/>
       <c r="E8" s="9" t="n">
@@ -3246,16 +3410,20 @@
         <f aca="false">장비!$F$9*(1-Q8*가정!$B$14)*가정!$B$15</f>
         <v>0.4267075</v>
       </c>
+      <c r="T8" s="14" t="n">
+        <f aca="false">MATCH(G8,등급!$B$4:$B$8,1)-1</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>165</v>
+        <v>180</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>166</v>
+        <v>181</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>167</v>
+        <v>182</v>
       </c>
       <c r="D9" s="4"/>
       <c r="E9" s="9" t="n">
@@ -3314,16 +3482,20 @@
         <f aca="false">장비!$F$9*(1-Q9*가정!$B$14)*가정!$B$15</f>
         <v>0.34891</v>
       </c>
+      <c r="T9" s="14" t="n">
+        <f aca="false">MATCH(G9,등급!$B$4:$B$8,1)-1</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>168</v>
+        <v>183</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>169</v>
+        <v>184</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>167</v>
+        <v>182</v>
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="9" t="n">
@@ -3382,16 +3554,20 @@
         <f aca="false">장비!$F$9*(1-Q10*가정!$B$14)*가정!$B$15</f>
         <v>0.32887125</v>
       </c>
+      <c r="T10" s="14" t="n">
+        <f aca="false">MATCH(G10,등급!$B$4:$B$8,1)-1</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>167</v>
+        <v>182</v>
       </c>
       <c r="D11" s="4"/>
       <c r="E11" s="9" t="n">
@@ -3450,16 +3626,20 @@
         <f aca="false">장비!$F$9*(1-Q11*가정!$B$14)*가정!$B$15</f>
         <v>0.29233</v>
       </c>
+      <c r="T11" s="14" t="n">
+        <f aca="false">MATCH(G11,등급!$B$4:$B$8,1)-1</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>172</v>
+        <v>187</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>173</v>
+        <v>188</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>167</v>
+        <v>182</v>
       </c>
       <c r="D12" s="4"/>
       <c r="E12" s="9" t="n">
@@ -3518,16 +3698,20 @@
         <f aca="false">장비!$F$9*(1-Q12*가정!$B$14)*가정!$B$15</f>
         <v>0.2475375</v>
       </c>
+      <c r="T12" s="14" t="n">
+        <f aca="false">MATCH(G12,등급!$B$4:$B$8,1)-1</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>174</v>
+        <v>189</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>175</v>
+        <v>190</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>158</v>
+        <v>173</v>
       </c>
       <c r="D13" s="4"/>
       <c r="E13" s="9" t="n">
@@ -3586,16 +3770,20 @@
         <f aca="false">장비!$F$9*(1-Q13*가정!$B$14)*가정!$B$15</f>
         <v>0.41845625</v>
       </c>
+      <c r="T13" s="14" t="n">
+        <f aca="false">MATCH(G13,등급!$B$4:$B$8,1)-1</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>176</v>
+        <v>191</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>177</v>
+        <v>192</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>167</v>
+        <v>182</v>
       </c>
       <c r="D14" s="4"/>
       <c r="E14" s="9" t="n">
@@ -3654,16 +3842,20 @@
         <f aca="false">장비!$F$9*(1-Q14*가정!$B$14)*가정!$B$15</f>
         <v>0.381915</v>
       </c>
+      <c r="T14" s="14" t="n">
+        <f aca="false">MATCH(G14,등급!$B$4:$B$8,1)-1</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>178</v>
+        <v>193</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>179</v>
+        <v>194</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>167</v>
+        <v>182</v>
       </c>
       <c r="D15" s="4"/>
       <c r="E15" s="9" t="n">
@@ -3722,16 +3914,20 @@
         <f aca="false">장비!$F$9*(1-Q15*가정!$B$14)*가정!$B$15</f>
         <v>0.3654125</v>
       </c>
+      <c r="T15" s="14" t="n">
+        <f aca="false">MATCH(G15,등급!$B$4:$B$8,1)-1</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>180</v>
+        <v>195</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>181</v>
+        <v>196</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>158</v>
+        <v>173</v>
       </c>
       <c r="D16" s="4"/>
       <c r="E16" s="9" t="n">
@@ -3790,16 +3986,20 @@
         <f aca="false">장비!$F$9*(1-Q16*가정!$B$14)*가정!$B$15</f>
         <v>0.34537375</v>
       </c>
+      <c r="T16" s="14" t="n">
+        <f aca="false">MATCH(G16,등급!$B$4:$B$8,1)-1</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>182</v>
+        <v>197</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>183</v>
+        <v>198</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>158</v>
+        <v>173</v>
       </c>
       <c r="D17" s="4"/>
       <c r="E17" s="9" t="n">
@@ -3858,16 +4058,20 @@
         <f aca="false">장비!$F$9*(1-Q17*가정!$B$14)*가정!$B$15</f>
         <v>0.3088325</v>
       </c>
+      <c r="T17" s="14" t="n">
+        <f aca="false">MATCH(G17,등급!$B$4:$B$8,1)-1</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>184</v>
+        <v>199</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>185</v>
+        <v>200</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>167</v>
+        <v>182</v>
       </c>
       <c r="D18" s="4"/>
       <c r="E18" s="9" t="n">
@@ -3926,16 +4130,20 @@
         <f aca="false">장비!$F$9*(1-Q18*가정!$B$14)*가정!$B$15</f>
         <v>0.29233</v>
       </c>
+      <c r="T18" s="14" t="n">
+        <f aca="false">MATCH(G18,등급!$B$4:$B$8,1)-1</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>186</v>
+        <v>201</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>187</v>
+        <v>202</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>158</v>
+        <v>173</v>
       </c>
       <c r="D19" s="4"/>
       <c r="E19" s="9" t="n">
@@ -3994,16 +4202,20 @@
         <f aca="false">장비!$F$9*(1-Q19*가정!$B$14)*가정!$B$15</f>
         <v>0.28407875</v>
       </c>
+      <c r="T19" s="14" t="n">
+        <f aca="false">MATCH(G19,등급!$B$4:$B$8,1)-1</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>188</v>
+        <v>203</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>189</v>
+        <v>204</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>158</v>
+        <v>173</v>
       </c>
       <c r="D20" s="4"/>
       <c r="E20" s="9" t="n">
@@ -4062,16 +4274,20 @@
         <f aca="false">장비!$F$9*(1-Q20*가정!$B$14)*가정!$B$15</f>
         <v>0.25578875</v>
       </c>
+      <c r="T20" s="14" t="n">
+        <f aca="false">MATCH(G20,등급!$B$4:$B$8,1)-1</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>190</v>
+        <v>205</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>191</v>
+        <v>206</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>167</v>
+        <v>182</v>
       </c>
       <c r="D21" s="4"/>
       <c r="E21" s="9" t="n">
@@ -4130,16 +4346,20 @@
         <f aca="false">장비!$F$9*(1-Q21*가정!$B$14)*가정!$B$15</f>
         <v>0.353625</v>
       </c>
+      <c r="T21" s="14" t="n">
+        <f aca="false">MATCH(G21,등급!$B$4:$B$8,1)-1</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>192</v>
+        <v>207</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>193</v>
+        <v>208</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>167</v>
+        <v>182</v>
       </c>
       <c r="D22" s="4"/>
       <c r="E22" s="9" t="n">
@@ -4198,16 +4418,20 @@
         <f aca="false">장비!$F$9*(1-Q22*가정!$B$14)*가정!$B$15</f>
         <v>0.325335</v>
       </c>
+      <c r="T22" s="14" t="n">
+        <f aca="false">MATCH(G22,등급!$B$4:$B$8,1)-1</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>194</v>
+        <v>209</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>195</v>
+        <v>210</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>167</v>
+        <v>182</v>
       </c>
       <c r="D23" s="4"/>
       <c r="E23" s="9" t="n">
@@ -4266,16 +4490,20 @@
         <f aca="false">장비!$F$9*(1-Q23*가정!$B$14)*가정!$B$15</f>
         <v>0.30058125</v>
       </c>
+      <c r="T23" s="14" t="n">
+        <f aca="false">MATCH(G23,등급!$B$4:$B$8,1)-1</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>196</v>
+        <v>211</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>167</v>
+        <v>182</v>
       </c>
       <c r="D24" s="4"/>
       <c r="E24" s="9" t="n">
@@ -4334,16 +4562,20 @@
         <f aca="false">장비!$F$9*(1-Q24*가정!$B$14)*가정!$B$15</f>
         <v>0.27229125</v>
       </c>
+      <c r="T24" s="14" t="n">
+        <f aca="false">MATCH(G24,등급!$B$4:$B$8,1)-1</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>198</v>
+        <v>213</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>199</v>
+        <v>214</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>167</v>
+        <v>182</v>
       </c>
       <c r="D25" s="4"/>
       <c r="E25" s="9" t="n">
@@ -4402,16 +4634,20 @@
         <f aca="false">장비!$F$9*(1-Q25*가정!$B$14)*가정!$B$15</f>
         <v>0.25578875</v>
       </c>
+      <c r="T25" s="14" t="n">
+        <f aca="false">MATCH(G25,등급!$B$4:$B$8,1)-1</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>201</v>
+        <v>216</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>167</v>
+        <v>182</v>
       </c>
       <c r="D26" s="4"/>
       <c r="E26" s="9" t="n">
@@ -4470,19 +4706,23 @@
         <f aca="false">장비!$F$9*(1-Q26*가정!$B$14)*가정!$B$15</f>
         <v>0.23598575</v>
       </c>
+      <c r="T26" s="14" t="n">
+        <f aca="false">MATCH(G26,등급!$B$4:$B$8,1)-1</f>
+        <v>4</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>202</v>
+        <v>217</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>203</v>
+        <v>218</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>167</v>
+        <v>182</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>204</v>
+        <v>219</v>
       </c>
       <c r="E27" s="9" t="n">
         <v>30</v>
@@ -4540,19 +4780,23 @@
         <f aca="false">장비!$F$9*(1-Q27*가정!$B$14)*가정!$B$15</f>
         <v>0.297045</v>
       </c>
+      <c r="T27" s="14" t="n">
+        <f aca="false">MATCH(G27,등급!$B$4:$B$8,1)-1</f>
+        <v>4</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>206</v>
+        <v>221</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>167</v>
+        <v>182</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>204</v>
+        <v>219</v>
       </c>
       <c r="E28" s="9" t="n">
         <v>90</v>
@@ -4610,19 +4854,23 @@
         <f aca="false">장비!$F$9*(1-Q28*가정!$B$14)*가정!$B$15</f>
         <v>0.30529625</v>
       </c>
+      <c r="T28" s="14" t="n">
+        <f aca="false">MATCH(G28,등급!$B$4:$B$8,1)-1</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>207</v>
+        <v>222</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>208</v>
+        <v>223</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>158</v>
+        <v>173</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>204</v>
+        <v>219</v>
       </c>
       <c r="E29" s="9" t="n">
         <v>50</v>
@@ -4680,19 +4928,23 @@
         <f aca="false">장비!$F$9*(1-Q29*가정!$B$14)*가정!$B$15</f>
         <v>0.25578875</v>
       </c>
+      <c r="T29" s="14" t="n">
+        <f aca="false">MATCH(G29,등급!$B$4:$B$8,1)-1</f>
+        <v>4</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>209</v>
+        <v>224</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>210</v>
+        <v>225</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>167</v>
+        <v>182</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>204</v>
+        <v>219</v>
       </c>
       <c r="E30" s="9" t="n">
         <v>100</v>
@@ -4749,6 +5001,10 @@
       <c r="S30" s="29" t="n">
         <f aca="false">장비!$F$9*(1-Q30*가정!$B$14)*가정!$B$15</f>
         <v>0.23575</v>
+      </c>
+      <c r="T30" s="14" t="n">
+        <f aca="false">MATCH(G30,등급!$B$4:$B$8,1)-1</f>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -4768,7 +5024,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:N44"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="14"/>
@@ -4777,58 +5033,66 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="0" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>211</v>
+        <v>226</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>212</v>
+        <v>227</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>213</v>
+        <v>228</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>214</v>
+        <v>229</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>215</v>
+        <v>230</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>216</v>
+        <v>231</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>217</v>
+        <v>232</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>218</v>
+        <v>233</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>219</v>
+        <v>234</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>220</v>
+        <v>237</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>221</v>
+        <v>238</v>
       </c>
       <c r="C5" s="12" t="n">
         <v>0</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>158</v>
+        <v>173</v>
       </c>
       <c r="E5" s="14" t="n">
         <f aca="false">COUNTIF($A$14:$A$44,B5)</f>
@@ -4846,19 +5110,27 @@
         <f aca="false">COUNTIFS($A$14:$A$44,B5,$I$14:$I$44,"전설")</f>
         <v>0</v>
       </c>
+      <c r="I5" s="20" t="n">
+        <f aca="false">SUMIF($A$14:$A$44,B5,$M$14:$M$44)</f>
+        <v>15.5107341598645</v>
+      </c>
+      <c r="J5" s="20" t="n">
+        <f aca="false">SUMIF($A$14:$A$44,B5,$N$14:$N$44)</f>
+        <v>16.5397899764719</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>222</v>
+        <v>239</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>223</v>
+        <v>240</v>
       </c>
       <c r="C6" s="12" t="n">
         <v>150</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>158</v>
+        <v>173</v>
       </c>
       <c r="E6" s="14" t="n">
         <f aca="false">COUNTIF($A$14:$A$44,B6)</f>
@@ -4876,19 +5148,27 @@
         <f aca="false">COUNTIFS($A$14:$A$44,B6,$I$14:$I$44,"전설")</f>
         <v>1</v>
       </c>
+      <c r="I6" s="20" t="n">
+        <f aca="false">SUMIF($A$14:$A$44,B6,$M$14:$M$44)</f>
+        <v>34.6166477771951</v>
+      </c>
+      <c r="J6" s="20" t="n">
+        <f aca="false">SUMIF($A$14:$A$44,B6,$N$14:$N$44)</f>
+        <v>66.7160206581735</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>224</v>
+        <v>241</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>225</v>
+        <v>242</v>
       </c>
       <c r="C7" s="12" t="n">
         <v>1500</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>158</v>
+        <v>173</v>
       </c>
       <c r="E7" s="14" t="n">
         <f aca="false">COUNTIF($A$14:$A$44,B7)</f>
@@ -4906,19 +5186,27 @@
         <f aca="false">COUNTIFS($A$14:$A$44,B7,$I$14:$I$44,"전설")</f>
         <v>1</v>
       </c>
+      <c r="I7" s="20" t="n">
+        <f aca="false">SUMIF($A$14:$A$44,B7,$M$14:$M$44)</f>
+        <v>88.4793821300199</v>
+      </c>
+      <c r="J7" s="20" t="n">
+        <f aca="false">SUMIF($A$14:$A$44,B7,$N$14:$N$44)</f>
+        <v>168.298288084171</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>226</v>
+        <v>243</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>227</v>
+        <v>244</v>
       </c>
       <c r="C8" s="12" t="n">
         <v>4000</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>167</v>
+        <v>182</v>
       </c>
       <c r="E8" s="14" t="n">
         <f aca="false">COUNTIF($A$14:$A$44,B8)</f>
@@ -4929,25 +5217,33 @@
         <v>758.269279988315</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>228</v>
+        <v>245</v>
       </c>
       <c r="H8" s="14" t="n">
         <f aca="false">COUNTIFS($A$14:$A$44,B8,$I$14:$I$44,"전설")</f>
         <v>3</v>
       </c>
+      <c r="I8" s="20" t="n">
+        <f aca="false">SUMIF($A$14:$A$44,B8,$M$14:$M$44)</f>
+        <v>588.258441092311</v>
+      </c>
+      <c r="J8" s="20" t="n">
+        <f aca="false">SUMIF($A$14:$A$44,B8,$N$14:$N$44)</f>
+        <v>959.735272708961</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>229</v>
+        <v>246</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>230</v>
+        <v>247</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>231</v>
+        <v>248</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>167</v>
+        <v>182</v>
       </c>
       <c r="E9" s="14" t="n">
         <f aca="false">COUNTIF($A$14:$A$44,B9)</f>
@@ -4958,53 +5254,73 @@
         <v>1944.80772047492</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>228</v>
+        <v>245</v>
       </c>
       <c r="H9" s="14" t="n">
         <f aca="false">COUNTIFS($A$14:$A$44,B9,$I$14:$I$44,"전설")</f>
         <v>6</v>
       </c>
+      <c r="I9" s="20" t="n">
+        <f aca="false">SUMIF($A$14:$A$44,B9,$M$14:$M$44)</f>
+        <v>1806.84392337803</v>
+      </c>
+      <c r="J9" s="20" t="n">
+        <f aca="false">SUMIF($A$14:$A$44,B9,$N$14:$N$44)</f>
+        <v>2104.83864095855</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="30" t="s">
-        <v>232</v>
+        <v>249</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>214</v>
+        <v>229</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>233</v>
+        <v>250</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>139</v>
+        <v>153</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>234</v>
+        <v>251</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>235</v>
+        <v>252</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>236</v>
+        <v>253</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>151</v>
+        <v>165</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="K13" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="L13" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="M13" s="3" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>221</v>
+        <v>238</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>156</v>
+        <v>171</v>
       </c>
       <c r="C14" s="31" t="str">
         <f aca="false">물고기!B5</f>
@@ -5033,13 +5349,29 @@
         <f aca="false">물고기!O5</f>
         <v>일반</v>
       </c>
+      <c r="J14" s="28" t="n">
+        <f aca="false">E14*(1+가정!$B$27)^(-물고기!T5)</f>
+        <v>70</v>
+      </c>
+      <c r="K14" s="28" t="n">
+        <f aca="false">E14*(1+가정!$B$27)^(물고기!T5)</f>
+        <v>70</v>
+      </c>
+      <c r="M14" s="20" t="n">
+        <f aca="false">J14/SUMIF($A$14:$A$44,A14,$J$14:$J$44)*H14</f>
+        <v>7.11548533272514</v>
+      </c>
+      <c r="N14" s="20" t="n">
+        <f aca="false">K14/SUMIF($A$14:$A$44,A14,$K$14:$K$44)*H14</f>
+        <v>6.90245460431796</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>221</v>
+        <v>238</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>159</v>
+        <v>174</v>
       </c>
       <c r="C15" s="31" t="str">
         <f aca="false">물고기!B6</f>
@@ -5068,13 +5400,29 @@
         <f aca="false">물고기!O6</f>
         <v>일반</v>
       </c>
+      <c r="J15" s="28" t="n">
+        <f aca="false">E15*(1+가정!$B$27)^(-물고기!T6)</f>
+        <v>25</v>
+      </c>
+      <c r="K15" s="28" t="n">
+        <f aca="false">E15*(1+가정!$B$27)^(물고기!T6)</f>
+        <v>25</v>
+      </c>
+      <c r="M15" s="20" t="n">
+        <f aca="false">J15/SUMIF($A$14:$A$44,A15,$J$14:$J$44)*H15</f>
+        <v>6.52348711733653</v>
+      </c>
+      <c r="N15" s="20" t="n">
+        <f aca="false">K15/SUMIF($A$14:$A$44,A15,$K$14:$K$44)*H15</f>
+        <v>6.32818024122372</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>221</v>
+        <v>238</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>161</v>
+        <v>176</v>
       </c>
       <c r="C16" s="31" t="str">
         <f aca="false">물고기!B7</f>
@@ -5103,13 +5451,29 @@
         <f aca="false">물고기!O7</f>
         <v>고급</v>
       </c>
+      <c r="J16" s="28" t="n">
+        <f aca="false">E16*(1+가정!$B$27)^(-물고기!T7)</f>
+        <v>3.7037037037037</v>
+      </c>
+      <c r="K16" s="28" t="n">
+        <f aca="false">E16*(1+가정!$B$27)^(물고기!T7)</f>
+        <v>6.75</v>
+      </c>
+      <c r="M16" s="20" t="n">
+        <f aca="false">J16/SUMIF($A$14:$A$44,A16,$J$14:$J$44)*H16</f>
+        <v>1.87176170980278</v>
+      </c>
+      <c r="N16" s="20" t="n">
+        <f aca="false">K16/SUMIF($A$14:$A$44,A16,$K$14:$K$44)*H16</f>
+        <v>3.30915513093019</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>223</v>
+        <v>240</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>163</v>
+        <v>178</v>
       </c>
       <c r="C17" s="31" t="str">
         <f aca="false">물고기!B8</f>
@@ -5138,13 +5502,29 @@
         <f aca="false">물고기!O8</f>
         <v>일반</v>
       </c>
+      <c r="J17" s="28" t="n">
+        <f aca="false">E17*(1+가정!$B$27)^(-물고기!T8)</f>
+        <v>35</v>
+      </c>
+      <c r="K17" s="28" t="n">
+        <f aca="false">E17*(1+가정!$B$27)^(물고기!T8)</f>
+        <v>35</v>
+      </c>
+      <c r="M17" s="20" t="n">
+        <f aca="false">J17/SUMIF($A$14:$A$44,A17,$J$14:$J$44)*H17</f>
+        <v>1.96543759758879</v>
+      </c>
+      <c r="N17" s="20" t="n">
+        <f aca="false">K17/SUMIF($A$14:$A$44,A17,$K$14:$K$44)*H17</f>
+        <v>1.53354420949566</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>223</v>
+        <v>240</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>156</v>
+        <v>171</v>
       </c>
       <c r="C18" s="31" t="str">
         <f aca="false">물고기!B5</f>
@@ -5173,13 +5553,29 @@
         <f aca="false">물고기!O5</f>
         <v>일반</v>
       </c>
+      <c r="J18" s="28" t="n">
+        <f aca="false">E18*(1+가정!$B$27)^(-물고기!T5)</f>
+        <v>28</v>
+      </c>
+      <c r="K18" s="28" t="n">
+        <f aca="false">E18*(1+가정!$B$27)^(물고기!T5)</f>
+        <v>28</v>
+      </c>
+      <c r="M18" s="20" t="n">
+        <f aca="false">J18/SUMIF($A$14:$A$44,A18,$J$14:$J$44)*H18</f>
+        <v>3.14470015614207</v>
+      </c>
+      <c r="N18" s="20" t="n">
+        <f aca="false">K18/SUMIF($A$14:$A$44,A18,$K$14:$K$44)*H18</f>
+        <v>2.45367073519305</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>223</v>
+        <v>240</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>161</v>
+        <v>176</v>
       </c>
       <c r="C19" s="31" t="str">
         <f aca="false">물고기!B7</f>
@@ -5208,13 +5604,29 @@
         <f aca="false">물고기!O7</f>
         <v>고급</v>
       </c>
+      <c r="J19" s="28" t="n">
+        <f aca="false">E19*(1+가정!$B$27)^(-물고기!T7)</f>
+        <v>10.3703703703704</v>
+      </c>
+      <c r="K19" s="28" t="n">
+        <f aca="false">E19*(1+가정!$B$27)^(물고기!T7)</f>
+        <v>18.9</v>
+      </c>
+      <c r="M19" s="20" t="n">
+        <f aca="false">J19/SUMIF($A$14:$A$44,A19,$J$14:$J$44)*H19</f>
+        <v>5.7905966298665</v>
+      </c>
+      <c r="N19" s="20" t="n">
+        <f aca="false">K19/SUMIF($A$14:$A$44,A19,$K$14:$K$44)*H19</f>
+        <v>8.23432285744928</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>223</v>
+        <v>240</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>165</v>
+        <v>180</v>
       </c>
       <c r="C20" s="31" t="str">
         <f aca="false">물고기!B9</f>
@@ -5243,13 +5655,29 @@
         <f aca="false">물고기!O9</f>
         <v>고급</v>
       </c>
+      <c r="J20" s="28" t="n">
+        <f aca="false">E20*(1+가정!$B$27)^(-물고기!T9)</f>
+        <v>8.88888888888889</v>
+      </c>
+      <c r="K20" s="28" t="n">
+        <f aca="false">E20*(1+가정!$B$27)^(물고기!T9)</f>
+        <v>16.2</v>
+      </c>
+      <c r="M20" s="20" t="n">
+        <f aca="false">J20/SUMIF($A$14:$A$44,A20,$J$14:$J$44)*H20</f>
+        <v>5.74295542210349</v>
+      </c>
+      <c r="N20" s="20" t="n">
+        <f aca="false">K20/SUMIF($A$14:$A$44,A20,$K$14:$K$44)*H20</f>
+        <v>8.16657628293983</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>223</v>
+        <v>240</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>168</v>
+        <v>183</v>
       </c>
       <c r="C21" s="31" t="str">
         <f aca="false">물고기!B10</f>
@@ -5278,13 +5706,29 @@
         <f aca="false">물고기!O10</f>
         <v>희귀</v>
       </c>
+      <c r="J21" s="28" t="n">
+        <f aca="false">E21*(1+가정!$B$27)^(-물고기!T10)</f>
+        <v>5.18518518518519</v>
+      </c>
+      <c r="K21" s="28" t="n">
+        <f aca="false">E21*(1+가정!$B$27)^(물고기!T10)</f>
+        <v>9.45</v>
+      </c>
+      <c r="M21" s="20" t="n">
+        <f aca="false">J21/SUMIF($A$14:$A$44,A21,$J$14:$J$44)*H21</f>
+        <v>7.70220169694312</v>
+      </c>
+      <c r="N21" s="20" t="n">
+        <f aca="false">K21/SUMIF($A$14:$A$44,A21,$K$14:$K$44)*H21</f>
+        <v>10.9526564428104</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>223</v>
+        <v>240</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="C22" s="31" t="str">
         <f aca="false">물고기!B11</f>
@@ -5313,13 +5757,29 @@
         <f aca="false">물고기!O11</f>
         <v>영웅</v>
       </c>
+      <c r="J22" s="28" t="n">
+        <f aca="false">E22*(1+가정!$B$27)^(-물고기!T11)</f>
+        <v>1.64609053497942</v>
+      </c>
+      <c r="K22" s="28" t="n">
+        <f aca="false">E22*(1+가정!$B$27)^(물고기!T11)</f>
+        <v>5.4675</v>
+      </c>
+      <c r="M22" s="20" t="n">
+        <f aca="false">J22/SUMIF($A$14:$A$44,A22,$J$14:$J$44)*H22</f>
+        <v>6.16245376473068</v>
+      </c>
+      <c r="N22" s="20" t="n">
+        <f aca="false">K22/SUMIF($A$14:$A$44,A22,$K$14:$K$44)*H22</f>
+        <v>15.9707675531762</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>223</v>
+        <v>240</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>172</v>
+        <v>187</v>
       </c>
       <c r="C23" s="31" t="str">
         <f aca="false">물고기!B12</f>
@@ -5348,13 +5808,29 @@
         <f aca="false">물고기!O12</f>
         <v>전설</v>
       </c>
+      <c r="J23" s="28" t="n">
+        <f aca="false">E23*(1+가정!$B$27)^(-물고기!T12)</f>
+        <v>0.243865264441396</v>
+      </c>
+      <c r="K23" s="28" t="n">
+        <f aca="false">E23*(1+가정!$B$27)^(물고기!T12)</f>
+        <v>1.476225</v>
+      </c>
+      <c r="M23" s="20" t="n">
+        <f aca="false">J23/SUMIF($A$14:$A$44,A23,$J$14:$J$44)*H23</f>
+        <v>4.10830250982045</v>
+      </c>
+      <c r="N23" s="20" t="n">
+        <f aca="false">K23/SUMIF($A$14:$A$44,A23,$K$14:$K$44)*H23</f>
+        <v>19.4044825771091</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>225</v>
+        <v>242</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>174</v>
+        <v>189</v>
       </c>
       <c r="C24" s="31" t="str">
         <f aca="false">물고기!B13</f>
@@ -5383,13 +5859,29 @@
         <f aca="false">물고기!O13</f>
         <v>일반</v>
       </c>
+      <c r="J24" s="28" t="n">
+        <f aca="false">E24*(1+가정!$B$27)^(-물고기!T13)</f>
+        <v>30</v>
+      </c>
+      <c r="K24" s="28" t="n">
+        <f aca="false">E24*(1+가정!$B$27)^(물고기!T13)</f>
+        <v>30</v>
+      </c>
+      <c r="M24" s="20" t="n">
+        <f aca="false">J24/SUMIF($A$14:$A$44,A24,$J$14:$J$44)*H24</f>
+        <v>4.42384125560499</v>
+      </c>
+      <c r="N24" s="20" t="n">
+        <f aca="false">K24/SUMIF($A$14:$A$44,A24,$K$14:$K$44)*H24</f>
+        <v>2.96082372613453</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>225</v>
+        <v>242</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>176</v>
+        <v>191</v>
       </c>
       <c r="C25" s="31" t="str">
         <f aca="false">물고기!B14</f>
@@ -5418,13 +5910,29 @@
         <f aca="false">물고기!O14</f>
         <v>고급</v>
       </c>
+      <c r="J25" s="28" t="n">
+        <f aca="false">E25*(1+가정!$B$27)^(-물고기!T14)</f>
+        <v>22</v>
+      </c>
+      <c r="K25" s="28" t="n">
+        <f aca="false">E25*(1+가정!$B$27)^(물고기!T14)</f>
+        <v>22</v>
+      </c>
+      <c r="M25" s="20" t="n">
+        <f aca="false">J25/SUMIF($A$14:$A$44,A25,$J$14:$J$44)*H25</f>
+        <v>7.64987525879106</v>
+      </c>
+      <c r="N25" s="20" t="n">
+        <f aca="false">K25/SUMIF($A$14:$A$44,A25,$K$14:$K$44)*H25</f>
+        <v>5.11996946985851</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>225</v>
+        <v>242</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>178</v>
+        <v>193</v>
       </c>
       <c r="C26" s="31" t="str">
         <f aca="false">물고기!B15</f>
@@ -5453,13 +5961,29 @@
         <f aca="false">물고기!O15</f>
         <v>고급</v>
       </c>
+      <c r="J26" s="28" t="n">
+        <f aca="false">E26*(1+가정!$B$27)^(-물고기!T15)</f>
+        <v>13.3333333333333</v>
+      </c>
+      <c r="K26" s="28" t="n">
+        <f aca="false">E26*(1+가정!$B$27)^(물고기!T15)</f>
+        <v>24.3</v>
+      </c>
+      <c r="M26" s="20" t="n">
+        <f aca="false">J26/SUMIF($A$14:$A$44,A26,$J$14:$J$44)*H26</f>
+        <v>8.20746592662871</v>
+      </c>
+      <c r="N26" s="20" t="n">
+        <f aca="false">K26/SUMIF($A$14:$A$44,A26,$K$14:$K$44)*H26</f>
+        <v>10.0112808105512</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>225</v>
+        <v>242</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>180</v>
+        <v>195</v>
       </c>
       <c r="C27" s="31" t="str">
         <f aca="false">물고기!B16</f>
@@ -5488,13 +6012,29 @@
         <f aca="false">물고기!O16</f>
         <v>희귀</v>
       </c>
+      <c r="J27" s="28" t="n">
+        <f aca="false">E27*(1+가정!$B$27)^(-물고기!T16)</f>
+        <v>8.88888888888889</v>
+      </c>
+      <c r="K27" s="28" t="n">
+        <f aca="false">E27*(1+가정!$B$27)^(물고기!T16)</f>
+        <v>16.2</v>
+      </c>
+      <c r="M27" s="20" t="n">
+        <f aca="false">J27/SUMIF($A$14:$A$44,A27,$J$14:$J$44)*H27</f>
+        <v>13.3218498389108</v>
+      </c>
+      <c r="N27" s="20" t="n">
+        <f aca="false">K27/SUMIF($A$14:$A$44,A27,$K$14:$K$44)*H27</f>
+        <v>16.2496903241016</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>225</v>
+        <v>242</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>182</v>
+        <v>197</v>
       </c>
       <c r="C28" s="31" t="str">
         <f aca="false">물고기!B17</f>
@@ -5523,13 +6063,29 @@
         <f aca="false">물고기!O17</f>
         <v>영웅</v>
       </c>
+      <c r="J28" s="28" t="n">
+        <f aca="false">E28*(1+가정!$B$27)^(-물고기!T17)</f>
+        <v>4.38957475994513</v>
+      </c>
+      <c r="K28" s="28" t="n">
+        <f aca="false">E28*(1+가정!$B$27)^(물고기!T17)</f>
+        <v>14.58</v>
+      </c>
+      <c r="M28" s="20" t="n">
+        <f aca="false">J28/SUMIF($A$14:$A$44,A28,$J$14:$J$44)*H28</f>
+        <v>19.8157534694248</v>
+      </c>
+      <c r="N28" s="20" t="n">
+        <f aca="false">K28/SUMIF($A$14:$A$44,A28,$K$14:$K$44)*H28</f>
+        <v>44.051295220895</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>225</v>
+        <v>242</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>184</v>
+        <v>199</v>
       </c>
       <c r="C29" s="31" t="str">
         <f aca="false">물고기!B18</f>
@@ -5558,13 +6114,29 @@
         <f aca="false">물고기!O18</f>
         <v>영웅</v>
       </c>
+      <c r="J29" s="28" t="n">
+        <f aca="false">E29*(1+가정!$B$27)^(-물고기!T18)</f>
+        <v>2.74348422496571</v>
+      </c>
+      <c r="K29" s="28" t="n">
+        <f aca="false">E29*(1+가정!$B$27)^(물고기!T18)</f>
+        <v>9.1125</v>
+      </c>
+      <c r="M29" s="20" t="n">
+        <f aca="false">J29/SUMIF($A$14:$A$44,A29,$J$14:$J$44)*H29</f>
+        <v>17.8172888792016</v>
+      </c>
+      <c r="N29" s="20" t="n">
+        <f aca="false">K29/SUMIF($A$14:$A$44,A29,$K$14:$K$44)*H29</f>
+        <v>39.6086201649976</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>225</v>
+        <v>242</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>186</v>
+        <v>201</v>
       </c>
       <c r="C30" s="31" t="str">
         <f aca="false">물고기!B19</f>
@@ -5593,13 +6165,29 @@
         <f aca="false">물고기!O19</f>
         <v>영웅</v>
       </c>
+      <c r="J30" s="28" t="n">
+        <f aca="false">E30*(1+가정!$B$27)^(-물고기!T19)</f>
+        <v>1.92043895747599</v>
+      </c>
+      <c r="K30" s="28" t="n">
+        <f aca="false">E30*(1+가정!$B$27)^(물고기!T19)</f>
+        <v>6.37875</v>
+      </c>
+      <c r="M30" s="20" t="n">
+        <f aca="false">J30/SUMIF($A$14:$A$44,A30,$J$14:$J$44)*H30</f>
+        <v>10.7000883269804</v>
+      </c>
+      <c r="N30" s="20" t="n">
+        <f aca="false">K30/SUMIF($A$14:$A$44,A30,$K$14:$K$44)*H30</f>
+        <v>23.7867689719066</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>225</v>
+        <v>242</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>188</v>
+        <v>203</v>
       </c>
       <c r="C31" s="31" t="str">
         <f aca="false">물고기!B20</f>
@@ -5628,13 +6216,29 @@
         <f aca="false">물고기!O20</f>
         <v>전설</v>
       </c>
+      <c r="J31" s="28" t="n">
+        <f aca="false">E31*(1+가정!$B$27)^(-물고기!T20)</f>
+        <v>0.406442107402327</v>
+      </c>
+      <c r="K31" s="28" t="n">
+        <f aca="false">E31*(1+가정!$B$27)^(물고기!T20)</f>
+        <v>2.460375</v>
+      </c>
+      <c r="M31" s="20" t="n">
+        <f aca="false">J31/SUMIF($A$14:$A$44,A31,$J$14:$J$44)*H31</f>
+        <v>6.54321917447758</v>
+      </c>
+      <c r="N31" s="20" t="n">
+        <f aca="false">K31/SUMIF($A$14:$A$44,A31,$K$14:$K$44)*H31</f>
+        <v>26.5098393957261</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>227</v>
+        <v>244</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>190</v>
+        <v>205</v>
       </c>
       <c r="C32" s="31" t="str">
         <f aca="false">물고기!B21</f>
@@ -5663,13 +6267,29 @@
         <f aca="false">물고기!O21</f>
         <v>희귀</v>
       </c>
+      <c r="J32" s="28" t="n">
+        <f aca="false">E32*(1+가정!$B$27)^(-물고기!T21)</f>
+        <v>22.2222222222222</v>
+      </c>
+      <c r="K32" s="28" t="n">
+        <f aca="false">E32*(1+가정!$B$27)^(물고기!T21)</f>
+        <v>40.5</v>
+      </c>
+      <c r="M32" s="20" t="n">
+        <f aca="false">J32/SUMIF($A$14:$A$44,A32,$J$14:$J$44)*H32</f>
+        <v>64.5085762139014</v>
+      </c>
+      <c r="N32" s="20" t="n">
+        <f aca="false">K32/SUMIF($A$14:$A$44,A32,$K$14:$K$44)*H32</f>
+        <v>32.6228464589079</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>227</v>
+        <v>244</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>192</v>
+        <v>207</v>
       </c>
       <c r="C33" s="31" t="str">
         <f aca="false">물고기!B22</f>
@@ -5698,13 +6318,29 @@
         <f aca="false">물고기!O22</f>
         <v>영웅</v>
       </c>
+      <c r="J33" s="28" t="n">
+        <f aca="false">E33*(1+가정!$B$27)^(-물고기!T22)</f>
+        <v>13.1687242798354</v>
+      </c>
+      <c r="K33" s="28" t="n">
+        <f aca="false">E33*(1+가정!$B$27)^(물고기!T22)</f>
+        <v>43.74</v>
+      </c>
+      <c r="M33" s="20" t="n">
+        <f aca="false">J33/SUMIF($A$14:$A$44,A33,$J$14:$J$44)*H33</f>
+        <v>95.3221597454697</v>
+      </c>
+      <c r="N33" s="20" t="n">
+        <f aca="false">K33/SUMIF($A$14:$A$44,A33,$K$14:$K$44)*H33</f>
+        <v>87.854863080623</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>227</v>
+        <v>244</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>194</v>
+        <v>209</v>
       </c>
       <c r="C34" s="31" t="str">
         <f aca="false">물고기!B23</f>
@@ -5733,13 +6369,29 @@
         <f aca="false">물고기!O23</f>
         <v>영웅</v>
       </c>
+      <c r="J34" s="28" t="n">
+        <f aca="false">E34*(1+가정!$B$27)^(-물고기!T23)</f>
+        <v>7.31595793324188</v>
+      </c>
+      <c r="K34" s="28" t="n">
+        <f aca="false">E34*(1+가정!$B$27)^(물고기!T23)</f>
+        <v>44.28675</v>
+      </c>
+      <c r="M34" s="20" t="n">
+        <f aca="false">J34/SUMIF($A$14:$A$44,A34,$J$14:$J$44)*H34</f>
+        <v>104.717951302916</v>
+      </c>
+      <c r="N34" s="20" t="n">
+        <f aca="false">K34/SUMIF($A$14:$A$44,A34,$K$14:$K$44)*H34</f>
+        <v>175.897880579644</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>227</v>
+        <v>244</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>196</v>
+        <v>211</v>
       </c>
       <c r="C35" s="31" t="str">
         <f aca="false">물고기!B24</f>
@@ -5768,13 +6420,29 @@
         <f aca="false">물고기!O24</f>
         <v>전설</v>
       </c>
+      <c r="J35" s="28" t="n">
+        <f aca="false">E35*(1+가정!$B$27)^(-물고기!T24)</f>
+        <v>5.28374739623025</v>
+      </c>
+      <c r="K35" s="28" t="n">
+        <f aca="false">E35*(1+가정!$B$27)^(물고기!T24)</f>
+        <v>31.984875</v>
+      </c>
+      <c r="M35" s="20" t="n">
+        <f aca="false">J35/SUMIF($A$14:$A$44,A35,$J$14:$J$44)*H35</f>
+        <v>120.955582178713</v>
+      </c>
+      <c r="N35" s="20" t="n">
+        <f aca="false">K35/SUMIF($A$14:$A$44,A35,$K$14:$K$44)*H35</f>
+        <v>203.172715707247</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>227</v>
+        <v>244</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>198</v>
+        <v>213</v>
       </c>
       <c r="C36" s="31" t="str">
         <f aca="false">물고기!B25</f>
@@ -5803,13 +6471,29 @@
         <f aca="false">물고기!O25</f>
         <v>전설</v>
       </c>
+      <c r="J36" s="28" t="n">
+        <f aca="false">E36*(1+가정!$B$27)^(-물고기!T25)</f>
+        <v>3.25153685921861</v>
+      </c>
+      <c r="K36" s="28" t="n">
+        <f aca="false">E36*(1+가정!$B$27)^(물고기!T25)</f>
+        <v>19.683</v>
+      </c>
+      <c r="M36" s="20" t="n">
+        <f aca="false">J36/SUMIF($A$14:$A$44,A36,$J$14:$J$44)*H36</f>
+        <v>116.175839865974</v>
+      </c>
+      <c r="N36" s="20" t="n">
+        <f aca="false">K36/SUMIF($A$14:$A$44,A36,$K$14:$K$44)*H36</f>
+        <v>195.144039323999</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>227</v>
+        <v>244</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="C37" s="31" t="str">
         <f aca="false">물고기!B26</f>
@@ -5838,13 +6522,29 @@
         <f aca="false">물고기!O26</f>
         <v>전설</v>
       </c>
+      <c r="J37" s="28" t="n">
+        <f aca="false">E37*(1+가정!$B$27)^(-물고기!T26)</f>
+        <v>0.602136455410855</v>
+      </c>
+      <c r="K37" s="28" t="n">
+        <f aca="false">E37*(1+가정!$B$27)^(물고기!T26)</f>
+        <v>6.6430125</v>
+      </c>
+      <c r="M37" s="20" t="n">
+        <f aca="false">J37/SUMIF($A$14:$A$44,A37,$J$14:$J$44)*H37</f>
+        <v>86.5783317853365</v>
+      </c>
+      <c r="N37" s="20" t="n">
+        <f aca="false">K37/SUMIF($A$14:$A$44,A37,$K$14:$K$44)*H37</f>
+        <v>265.042927558541</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>230</v>
+        <v>247</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>194</v>
+        <v>209</v>
       </c>
       <c r="C38" s="31" t="str">
         <f aca="false">물고기!B23</f>
@@ -5873,13 +6573,29 @@
         <f aca="false">물고기!O23</f>
         <v>영웅</v>
       </c>
+      <c r="J38" s="28" t="n">
+        <f aca="false">E38*(1+가정!$B$27)^(-물고기!T23)</f>
+        <v>8.12884214804654</v>
+      </c>
+      <c r="K38" s="28" t="n">
+        <f aca="false">E38*(1+가정!$B$27)^(물고기!T23)</f>
+        <v>49.2075</v>
+      </c>
+      <c r="M38" s="20" t="n">
+        <f aca="false">J38/SUMIF($A$14:$A$44,A38,$J$14:$J$44)*H38</f>
+        <v>177.389819603573</v>
+      </c>
+      <c r="N38" s="20" t="n">
+        <f aca="false">K38/SUMIF($A$14:$A$44,A38,$K$14:$K$44)*H38</f>
+        <v>152.41709788788</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>230</v>
+        <v>247</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>196</v>
+        <v>211</v>
       </c>
       <c r="C39" s="31" t="str">
         <f aca="false">물고기!B24</f>
@@ -5908,13 +6624,29 @@
         <f aca="false">물고기!O24</f>
         <v>전설</v>
       </c>
+      <c r="J39" s="28" t="n">
+        <f aca="false">E39*(1+가정!$B$27)^(-물고기!T24)</f>
+        <v>6.0966316110349</v>
+      </c>
+      <c r="K39" s="28" t="n">
+        <f aca="false">E39*(1+가정!$B$27)^(물고기!T24)</f>
+        <v>36.905625</v>
+      </c>
+      <c r="M39" s="20" t="n">
+        <f aca="false">J39/SUMIF($A$14:$A$44,A39,$J$14:$J$44)*H39</f>
+        <v>212.776610947514</v>
+      </c>
+      <c r="N39" s="20" t="n">
+        <f aca="false">K39/SUMIF($A$14:$A$44,A39,$K$14:$K$44)*H39</f>
+        <v>182.822180052464</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>230</v>
+        <v>247</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>198</v>
+        <v>213</v>
       </c>
       <c r="C40" s="31" t="str">
         <f aca="false">물고기!B25</f>
@@ -5943,13 +6675,29 @@
         <f aca="false">물고기!O25</f>
         <v>전설</v>
       </c>
+      <c r="J40" s="28" t="n">
+        <f aca="false">E40*(1+가정!$B$27)^(-물고기!T25)</f>
+        <v>4.87730528882792</v>
+      </c>
+      <c r="K40" s="28" t="n">
+        <f aca="false">E40*(1+가정!$B$27)^(물고기!T25)</f>
+        <v>29.5245</v>
+      </c>
+      <c r="M40" s="20" t="n">
+        <f aca="false">J40/SUMIF($A$14:$A$44,A40,$J$14:$J$44)*H40</f>
+        <v>265.678948801069</v>
+      </c>
+      <c r="N40" s="20" t="n">
+        <f aca="false">K40/SUMIF($A$14:$A$44,A40,$K$14:$K$44)*H40</f>
+        <v>228.27699152441</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>230</v>
+        <v>247</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="C41" s="31" t="str">
         <f aca="false">물고기!B28</f>
@@ -5978,13 +6726,29 @@
         <f aca="false">물고기!O28</f>
         <v>전설</v>
       </c>
+      <c r="J41" s="28" t="n">
+        <f aca="false">E41*(1+가정!$B$27)^(-물고기!T28)</f>
+        <v>8.12884214804654</v>
+      </c>
+      <c r="K41" s="28" t="n">
+        <f aca="false">E41*(1+가정!$B$27)^(물고기!T28)</f>
+        <v>49.2075</v>
+      </c>
+      <c r="M41" s="20" t="n">
+        <f aca="false">J41/SUMIF($A$14:$A$44,A41,$J$14:$J$44)*H41</f>
+        <v>369.404370097251</v>
+      </c>
+      <c r="N41" s="20" t="n">
+        <f aca="false">K41/SUMIF($A$14:$A$44,A41,$K$14:$K$44)*H41</f>
+        <v>317.400074948772</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>230</v>
+        <v>247</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>202</v>
+        <v>217</v>
       </c>
       <c r="C42" s="31" t="str">
         <f aca="false">물고기!B27</f>
@@ -6013,13 +6777,29 @@
         <f aca="false">물고기!O27</f>
         <v>전설</v>
       </c>
+      <c r="J42" s="28" t="n">
+        <f aca="false">E42*(1+가정!$B$27)^(-물고기!T27)</f>
+        <v>4.51602341558141</v>
+      </c>
+      <c r="K42" s="28" t="n">
+        <f aca="false">E42*(1+가정!$B$27)^(물고기!T27)</f>
+        <v>49.82259375</v>
+      </c>
+      <c r="M42" s="20" t="n">
+        <f aca="false">J42/SUMIF($A$14:$A$44,A42,$J$14:$J$44)*H42</f>
+        <v>288.871522157125</v>
+      </c>
+      <c r="N42" s="20" t="n">
+        <f aca="false">K42/SUMIF($A$14:$A$44,A42,$K$14:$K$44)*H42</f>
+        <v>452.352779227973</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
-        <v>230</v>
+        <v>247</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>207</v>
+        <v>222</v>
       </c>
       <c r="C43" s="31" t="str">
         <f aca="false">물고기!B29</f>
@@ -6048,13 +6828,29 @@
         <f aca="false">물고기!O29</f>
         <v>전설</v>
       </c>
+      <c r="J43" s="28" t="n">
+        <f aca="false">E43*(1+가정!$B$27)^(-물고기!T29)</f>
+        <v>1.80640936623256</v>
+      </c>
+      <c r="K43" s="28" t="n">
+        <f aca="false">E43*(1+가정!$B$27)^(물고기!T29)</f>
+        <v>19.9290375</v>
+      </c>
+      <c r="M43" s="20" t="n">
+        <f aca="false">J43/SUMIF($A$14:$A$44,A43,$J$14:$J$44)*H43</f>
+        <v>267.562216906408</v>
+      </c>
+      <c r="N43" s="20" t="n">
+        <f aca="false">K43/SUMIF($A$14:$A$44,A43,$K$14:$K$44)*H43</f>
+        <v>418.98388435873</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="s">
-        <v>230</v>
+        <v>247</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>209</v>
+        <v>224</v>
       </c>
       <c r="C44" s="31" t="str">
         <f aca="false">물고기!B30</f>
@@ -6082,6 +6878,22 @@
       <c r="I44" s="31" t="str">
         <f aca="false">물고기!O30</f>
         <v>전설</v>
+      </c>
+      <c r="J44" s="28" t="n">
+        <f aca="false">E44*(1+가정!$B$27)^(-물고기!T30)</f>
+        <v>0.451602341558141</v>
+      </c>
+      <c r="K44" s="28" t="n">
+        <f aca="false">E44*(1+가정!$B$27)^(물고기!T30)</f>
+        <v>4.982259375</v>
+      </c>
+      <c r="M44" s="20" t="n">
+        <f aca="false">J44/SUMIF($A$14:$A$44,A44,$J$14:$J$44)*H44</f>
+        <v>225.160434865095</v>
+      </c>
+      <c r="N44" s="20" t="n">
+        <f aca="false">K44/SUMIF($A$14:$A$44,A44,$K$14:$K$44)*H44</f>
+        <v>352.585632958324</v>
       </c>
     </row>
   </sheetData>
@@ -6114,132 +6926,132 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>237</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>238</v>
+        <v>259</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>214</v>
+        <v>229</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>239</v>
+        <v>260</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>240</v>
+        <v>261</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>241</v>
+        <v>262</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>242</v>
+        <v>263</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>221</v>
+        <v>238</v>
       </c>
       <c r="B5" s="14" t="n">
         <v>3</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>243</v>
+        <v>264</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>244</v>
+        <v>265</v>
       </c>
       <c r="E5" s="33" t="n">
         <v>2</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>245</v>
+        <v>266</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>223</v>
+        <v>240</v>
       </c>
       <c r="B6" s="14" t="n">
         <v>7</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>246</v>
+        <v>267</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>247</v>
+        <v>268</v>
       </c>
       <c r="E6" s="21" t="n">
         <v>0.1</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>248</v>
+        <v>269</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>225</v>
+        <v>242</v>
       </c>
       <c r="B7" s="14" t="n">
         <v>8</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>249</v>
+        <v>270</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>250</v>
+        <v>271</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>0.3</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>251</v>
+        <v>272</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>227</v>
+        <v>244</v>
       </c>
       <c r="B8" s="14" t="n">
         <v>6</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>252</v>
+        <v>273</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>253</v>
+        <v>274</v>
       </c>
       <c r="E8" s="21" t="n">
         <v>0.1</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>254</v>
+        <v>275</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="B9" s="14" t="n">
         <v>4</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>255</v>
+        <v>276</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>256</v>
+        <v>277</v>
       </c>
       <c r="E9" s="33" t="n">
         <v>30</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>257</v>
+        <v>278</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add auto-fishing net and redraw the pier stage
- Net (5 levels, 5,000 to 400,000): catches one fish from the current stage
  every 90 to 30 s, keeps up to 4 to 12, keeps working while the game is
  closed (up to 24 h). Higher levels catch better fish using the same
  grade bias as long casts. Net chip in the HUD opens a panel to sell all or
  move fish to the keep net; net catches count for the dex
- Pier: sun, drifting clouds, seagulls, layered islands, a passing ship, a
  far breakwater with a detailed red lighthouse, sun glints on the water,
  a concrete pier with joints, moss line, bollard, rope and cooler, and a
  pile of half-submerged tetrapods with breaking foam (also used in Busan)
- Spreadsheet: net sheet with expected price, income per minute and
  payback per stage; fix shifted headers in the stage detail table
</commit_message>
<xml_diff>
--- a/bukangi-fishing-balance.xlsx
+++ b/bukangi-fishing-balance.xlsx
@@ -14,7 +14,8 @@
     <sheet name="장비" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="물고기" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="낚시터" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="도감 보상" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="그물" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="도감 보상" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -201,8 +202,122 @@
 </comments>
 </file>
 
+<file path=xl/comments7.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>Unknown Author</author>
+  </authors>
+  <commentList>
+    <comment ref="K5" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Noto Sans CJK SC"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">반올림을 뺀 근사값</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">. </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Noto Sans CJK SC"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">게임 안에서 </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">2</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Noto Sans CJK SC"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">만 번 굴린 평균과 </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">1~3% </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Noto Sans CJK SC"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">안에서 맞습니다</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Q5" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Noto Sans CJK SC"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">그 레벨로 올리는 비용을 그 레벨의 분당 수입으로 나눈 값 </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">(</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Noto Sans CJK SC"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">게임을 켜 둔 채 칸이 안 찬다고 가정</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">)</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="310">
   <si>
     <t xml:space="preserve">부캉이 낚시터 밸런스 요약</t>
   </si>
@@ -276,6 +391,18 @@
     <t xml:space="preserve">캐스팅 게이지 끝</t>
   </si>
   <si>
+    <t xml:space="preserve">그물 전체 강화 비용 (원)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">작은 그물 ~ 황금 그물</t>
+  </si>
+  <si>
+    <t xml:space="preserve">작은 그물 배낚시 분당 수입 (원)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">황금 그물 배낚시 분당 수입 (원)</t>
+  </si>
+  <si>
     <t xml:space="preserve">부산 이용권 1장 시간 (초)</t>
   </si>
   <si>
@@ -457,6 +584,12 @@
   </si>
   <si>
     <t xml:space="preserve">CONFIG.cast.startDistNear — 걸린 뒤 끌어올 거리</t>
+  </si>
+  <si>
+    <t xml:space="preserve">그물: 꺼 둔 동안 최대 진행 시간 (시간)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONFIG.autoNet.maxOfflineHours</t>
   </si>
   <si>
     <t xml:space="preserve">멀리 던졌을 때 시작 거리 배수</t>
@@ -1001,6 +1134,91 @@
   <si>
     <t xml:space="preserve">기여
 가장 멀리 (원)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">기준가 등급
+번호</t>
+  </si>
+  <si>
+    <t xml:space="preserve">그물 (자동 낚시)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">그물은 일정 시간마다 지금 낚시터 물고기 1마리를 잡습니다(부캉이 제외). 그물 칸이 차면 멈추고, 게임을 꺼 둔 동안에도 진행됩니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">물고기 질은 캐스팅 거리 효과와 같은 식입니다: 가중치 × (1+캐스팅 등급 배율)^(질 × 기준가 등급 번호). 질 0 = 게이지 한가운데, 1 = 가장 멀리 던진 것과 같음. 행운은 미끼 행운 대신 쓰입니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">구입·강화 비용 (원)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">물고기 질</t>
+  </si>
+  <si>
+    <t xml:space="preserve">행운</t>
+  </si>
+  <si>
+    <t xml:space="preserve">크기 분포 지수</t>
+  </si>
+  <si>
+    <t xml:space="preserve">간격 (초)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">칸 수</t>
+  </si>
+  <si>
+    <t xml:space="preserve">가득 차는 시간 (분)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1마리 기대가
+강 (원)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1마리 기대가
+방파제 (원)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1마리 기대가
+배낚시 (원)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">분당 수입
+강 (원)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">분당 수입
+방파제 (원)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">분당 수입
+배낚시 (원)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">비용 회수
+강 (분)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">비용 회수
+방파제 (분)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">비용 회수
+배낚시 (분)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">작은 그물</t>
+  </si>
+  <si>
+    <t xml:space="preserve">자망</t>
+  </si>
+  <si>
+    <t xml:space="preserve">나일론 정치망</t>
+  </si>
+  <si>
+    <t xml:space="preserve">대형 정치망</t>
+  </si>
+  <si>
+    <t xml:space="preserve">황금 그물</t>
   </si>
   <si>
     <t xml:space="preserve">도감 완성 보상</t>
@@ -1303,7 +1521,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1433,6 +1651,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="173" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1692,7 +1914,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -1887,9 +2109,9 @@
       <c r="A19" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B19" s="7" t="n">
-        <f aca="false">가정!$B$11</f>
-        <v>150</v>
+      <c r="B19" s="5" t="n">
+        <f aca="false">그물!D10</f>
+        <v>635000</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>25</v>
@@ -1899,9 +2121,9 @@
       <c r="A20" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="7" t="n">
-        <f aca="false">가정!$B$4+'도감 보상'!E5</f>
-        <v>17</v>
+      <c r="B20" s="5" t="n">
+        <f aca="false">그물!P6</f>
+        <v>446.025217121152</v>
       </c>
       <c r="C20" s="4"/>
     </row>
@@ -1909,33 +2131,65 @@
       <c r="A21" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B21" s="8" t="n">
-        <f aca="false">물고기!R5</f>
-        <v>0.24495</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>28</v>
-      </c>
+      <c r="B21" s="5" t="n">
+        <f aca="false">그물!P10</f>
+        <v>2568.32699576596</v>
+      </c>
+      <c r="C21" s="4"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B22" s="7" t="n">
+        <f aca="false">가정!$B$11</f>
+        <v>150</v>
+      </c>
+      <c r="C22" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B22" s="8" t="n">
-        <f aca="false">물고기!R30</f>
-        <v>0.138</v>
-      </c>
-      <c r="C22" s="4"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B23" s="8" t="n">
+      <c r="B23" s="7" t="n">
+        <f aca="false">가정!$B$4+'도감 보상'!E5</f>
+        <v>17</v>
+      </c>
+      <c r="C23" s="4"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B24" s="8" t="n">
+        <f aca="false">물고기!R5</f>
+        <v>0.24495</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B25" s="8" t="n">
+        <f aca="false">물고기!R30</f>
+        <v>0.138</v>
+      </c>
+      <c r="C25" s="4"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B26" s="8" t="n">
         <f aca="false">물고기!S30</f>
         <v>0.23575</v>
       </c>
-      <c r="C23" s="4"/>
+      <c r="C26" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1953,7 +2207,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -1963,12 +2217,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="20.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1979,315 +2233,326 @@
         <v>3</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B4" s="9" t="n">
         <v>15</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B5" s="9" t="n">
         <v>1.8</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B6" s="9" t="n">
         <v>0.6</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B7" s="9" t="n">
         <v>0.35</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="B8" s="9" t="n">
         <v>1.5</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B9" s="10" t="n">
         <v>0.004</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B10" s="9" t="n">
         <v>2</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B11" s="9" t="n">
         <v>150</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B12" s="9" t="n">
         <v>150</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B13" s="9" t="n">
         <v>30</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B14" s="9" t="n">
         <v>0.5</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B15" s="9" t="n">
         <v>1.15</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B16" s="9" t="n">
         <v>0.88</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B17" s="9" t="n">
         <v>0.88</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B18" s="9" t="n">
         <v>1.12</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B19" s="9" t="n">
         <v>0.24</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B20" s="9" t="n">
         <v>0.36</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B21" s="9" t="n">
         <v>0.75</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B22" s="9" t="n">
         <v>0.9</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B23" s="9" t="n">
         <v>2.2</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B24" s="9" t="n">
         <v>0.7</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B25" s="9" t="n">
         <v>0.05</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B26" s="9" t="n">
         <v>0.12</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B27" s="9" t="n">
         <v>0.35</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B28" s="9" t="n">
         <v>12</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B29" s="9" t="n">
         <v>40</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B30" s="9" t="n">
         <v>0.85</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B31" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B32" s="9" t="n">
         <v>1.15</v>
       </c>
-      <c r="C31" s="4" t="s">
-        <v>86</v>
+      <c r="C32" s="4" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -2317,37 +2582,37 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="B4" s="12" t="n">
         <v>0</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="D4" s="14" t="n">
         <f aca="false">COUNTIF(물고기!$O$5:$O$40,A4)</f>
@@ -2356,13 +2621,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="B5" s="12" t="n">
         <v>60</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D5" s="14" t="n">
         <f aca="false">COUNTIF(물고기!$O$5:$O$40,A5)</f>
@@ -2371,13 +2636,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B6" s="12" t="n">
         <v>200</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="D6" s="14" t="n">
         <f aca="false">COUNTIF(물고기!$O$5:$O$40,A6)</f>
@@ -2386,13 +2651,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="B7" s="12" t="n">
         <v>700</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="D7" s="14" t="n">
         <f aca="false">COUNTIF(물고기!$O$5:$O$40,A7)</f>
@@ -2401,13 +2666,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="B8" s="12" t="n">
         <v>2500</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="D8" s="14" t="n">
         <f aca="false">COUNTIF(물고기!$O$5:$O$40,A8)</f>
@@ -2416,13 +2681,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -2455,52 +2720,52 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="B5" s="14" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="D5" s="12" t="n">
         <v>0</v>
@@ -2513,18 +2778,18 @@
         <v>0.24</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="B6" s="14" t="n">
         <v>2</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D6" s="12" t="n">
         <v>200</v>
@@ -2537,18 +2802,18 @@
         <v>0.28</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="B7" s="14" t="n">
         <v>3</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="D7" s="12" t="n">
         <v>1200</v>
@@ -2561,18 +2826,18 @@
         <v>0.32</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="B8" s="14" t="n">
         <v>4</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="D8" s="12" t="n">
         <v>6000</v>
@@ -2585,18 +2850,18 @@
         <v>0.36</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="B9" s="14" t="n">
         <v>5</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="D9" s="12" t="n">
         <v>25000</v>
@@ -2609,18 +2874,18 @@
         <v>0.41</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="B10" s="14" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="D10" s="12" t="n">
         <v>0</v>
@@ -2633,18 +2898,18 @@
         <v>0.16</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="B11" s="14" t="n">
         <v>2</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="D11" s="12" t="n">
         <v>250</v>
@@ -2657,18 +2922,18 @@
         <v>0.21</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="B12" s="14" t="n">
         <v>3</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="D12" s="12" t="n">
         <v>1500</v>
@@ -2681,18 +2946,18 @@
         <v>0.27</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="B13" s="14" t="n">
         <v>4</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="D13" s="12" t="n">
         <v>7000</v>
@@ -2705,18 +2970,18 @@
         <v>0.34</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="B14" s="14" t="n">
         <v>5</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="D14" s="12" t="n">
         <v>30000</v>
@@ -2729,18 +2994,18 @@
         <v>0.42</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="B15" s="14" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="D15" s="12" t="n">
         <v>0</v>
@@ -2753,18 +3018,18 @@
         <v>1.2</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="B16" s="14" t="n">
         <v>2</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D16" s="12" t="n">
         <v>150</v>
@@ -2777,18 +3042,18 @@
         <v>1.7</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="B17" s="14" t="n">
         <v>3</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="D17" s="12" t="n">
         <v>1000</v>
@@ -2801,18 +3066,18 @@
         <v>2.4</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="B18" s="14" t="n">
         <v>4</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="D18" s="12" t="n">
         <v>5000</v>
@@ -2825,18 +3090,18 @@
         <v>3.3</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="B19" s="14" t="n">
         <v>5</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="D19" s="12" t="n">
         <v>22000</v>
@@ -2849,18 +3114,18 @@
         <v>4.5</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="B20" s="14" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="D20" s="12" t="n">
         <v>0</v>
@@ -2873,7 +3138,7 @@
         <v>0</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="H20" s="23" t="n">
         <f aca="false">가정!$B$9*(1+F20*가정!$B$10)</f>
@@ -2886,13 +3151,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="B21" s="14" t="n">
         <v>2</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="D21" s="12" t="n">
         <v>100</v>
@@ -2905,7 +3170,7 @@
         <v>0.15</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="H21" s="23" t="n">
         <f aca="false">가정!$B$9*(1+F21*가정!$B$10)</f>
@@ -2918,13 +3183,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="B22" s="14" t="n">
         <v>3</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="D22" s="12" t="n">
         <v>800</v>
@@ -2937,7 +3202,7 @@
         <v>0.3</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="H22" s="23" t="n">
         <f aca="false">가정!$B$9*(1+F22*가정!$B$10)</f>
@@ -2950,13 +3215,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="B23" s="14" t="n">
         <v>4</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="D23" s="12" t="n">
         <v>4500</v>
@@ -2969,7 +3234,7 @@
         <v>0.5</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="H23" s="23" t="n">
         <f aca="false">가정!$B$9*(1+F23*가정!$B$10)</f>
@@ -2982,13 +3247,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="B24" s="14" t="n">
         <v>5</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="D24" s="12" t="n">
         <v>20000</v>
@@ -3001,7 +3266,7 @@
         <v>0.8</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="H24" s="23" t="n">
         <f aca="false">가정!$B$9*(1+F24*가정!$B$10)</f>
@@ -3014,7 +3279,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C25" s="25" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="D25" s="26" t="n">
         <f aca="false">SUM(D5:D24)</f>
@@ -3057,85 +3322,85 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="Q4" s="3" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="S4" s="3" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="T4" s="3" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="9" t="n">
@@ -3201,13 +3466,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="9" t="n">
@@ -3273,13 +3538,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D7" s="4"/>
       <c r="E7" s="9" t="n">
@@ -3345,13 +3610,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="B8" s="11" t="s">
+        <v>185</v>
+      </c>
+      <c r="C8" s="11" t="s">
         <v>179</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>173</v>
       </c>
       <c r="D8" s="4"/>
       <c r="E8" s="9" t="n">
@@ -3417,13 +3682,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="D9" s="4"/>
       <c r="E9" s="9" t="n">
@@ -3489,13 +3754,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="9" t="n">
@@ -3561,13 +3826,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="D11" s="4"/>
       <c r="E11" s="9" t="n">
@@ -3633,13 +3898,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="B12" s="11" t="s">
+        <v>194</v>
+      </c>
+      <c r="C12" s="11" t="s">
         <v>188</v>
-      </c>
-      <c r="C12" s="11" t="s">
-        <v>182</v>
       </c>
       <c r="D12" s="4"/>
       <c r="E12" s="9" t="n">
@@ -3705,13 +3970,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D13" s="4"/>
       <c r="E13" s="9" t="n">
@@ -3777,13 +4042,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="D14" s="4"/>
       <c r="E14" s="9" t="n">
@@ -3849,13 +4114,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="D15" s="4"/>
       <c r="E15" s="9" t="n">
@@ -3921,13 +4186,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D16" s="4"/>
       <c r="E16" s="9" t="n">
@@ -3993,13 +4258,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D17" s="4"/>
       <c r="E17" s="9" t="n">
@@ -4065,13 +4330,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="D18" s="4"/>
       <c r="E18" s="9" t="n">
@@ -4137,13 +4402,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D19" s="4"/>
       <c r="E19" s="9" t="n">
@@ -4209,13 +4474,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D20" s="4"/>
       <c r="E20" s="9" t="n">
@@ -4281,13 +4546,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="D21" s="4"/>
       <c r="E21" s="9" t="n">
@@ -4353,13 +4618,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="D22" s="4"/>
       <c r="E22" s="9" t="n">
@@ -4425,13 +4690,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="D23" s="4"/>
       <c r="E23" s="9" t="n">
@@ -4497,13 +4762,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="D24" s="4"/>
       <c r="E24" s="9" t="n">
@@ -4569,13 +4834,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="D25" s="4"/>
       <c r="E25" s="9" t="n">
@@ -4641,13 +4906,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="D26" s="4"/>
       <c r="E26" s="9" t="n">
@@ -4713,16 +4978,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="E27" s="9" t="n">
         <v>30</v>
@@ -4787,16 +5052,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="E28" s="9" t="n">
         <v>90</v>
@@ -4861,16 +5126,16 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="E29" s="9" t="n">
         <v>50</v>
@@ -4935,16 +5200,16 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="B30" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="C30" s="11" t="s">
+        <v>188</v>
+      </c>
+      <c r="D30" s="4" t="s">
         <v>225</v>
-      </c>
-      <c r="C30" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="D30" s="4" t="s">
-        <v>219</v>
       </c>
       <c r="E30" s="9" t="n">
         <v>100</v>
@@ -5024,7 +5289,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N44"/>
+  <dimension ref="A1:S44"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="14"/>
@@ -5037,62 +5302,63 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="15" style="0" width="10"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>227</v>
+        <v>233</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="C5" s="12" t="n">
         <v>0</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="E5" s="14" t="n">
         <f aca="false">COUNTIF($A$14:$A$44,B5)</f>
@@ -5121,16 +5387,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="C6" s="12" t="n">
         <v>150</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="E6" s="14" t="n">
         <f aca="false">COUNTIF($A$14:$A$44,B6)</f>
@@ -5159,16 +5425,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="C7" s="12" t="n">
         <v>1500</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="E7" s="14" t="n">
         <f aca="false">COUNTIF($A$14:$A$44,B7)</f>
@@ -5197,16 +5463,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="C8" s="12" t="n">
         <v>4000</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="E8" s="14" t="n">
         <f aca="false">COUNTIF($A$14:$A$44,B8)</f>
@@ -5217,7 +5483,7 @@
         <v>758.269279988315</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="H8" s="14" t="n">
         <f aca="false">COUNTIFS($A$14:$A$44,B8,$I$14:$I$44,"전설")</f>
@@ -5234,16 +5500,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="E9" s="14" t="n">
         <f aca="false">COUNTIF($A$14:$A$44,B9)</f>
@@ -5254,7 +5520,7 @@
         <v>1944.80772047492</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="H9" s="14" t="n">
         <f aca="false">COUNTIFS($A$14:$A$44,B9,$I$14:$I$44,"전설")</f>
@@ -5271,56 +5537,72 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="30" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="H13" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="K13" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="L13" s="3"/>
+      <c r="M13" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="N13" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="O13" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="P13" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="I13" s="3" t="s">
+      <c r="Q13" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="R13" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="J13" s="3" t="s">
-        <v>254</v>
-      </c>
-      <c r="K13" s="3" t="s">
-        <v>255</v>
-      </c>
-      <c r="L13" s="3" t="s">
-        <v>256</v>
-      </c>
-      <c r="M13" s="3" t="s">
-        <v>257</v>
+      <c r="S13" s="3" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C14" s="31" t="str">
         <f aca="false">물고기!B5</f>
@@ -5365,13 +5647,33 @@
         <f aca="false">K14/SUMIF($A$14:$A$44,A14,$K$14:$K$44)*H14</f>
         <v>6.90245460431796</v>
       </c>
+      <c r="O14" s="31" t="n">
+        <f aca="false">물고기!E5</f>
+        <v>12</v>
+      </c>
+      <c r="P14" s="31" t="n">
+        <f aca="false">물고기!F5</f>
+        <v>30</v>
+      </c>
+      <c r="Q14" s="5" t="n">
+        <f aca="false">물고기!G5</f>
+        <v>12</v>
+      </c>
+      <c r="R14" s="33" t="n">
+        <f aca="false">물고기!I5</f>
+        <v>21</v>
+      </c>
+      <c r="S14" s="31" t="n">
+        <f aca="false">물고기!T5</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="C15" s="31" t="str">
         <f aca="false">물고기!B6</f>
@@ -5416,13 +5718,33 @@
         <f aca="false">K15/SUMIF($A$14:$A$44,A15,$K$14:$K$44)*H15</f>
         <v>6.32818024122372</v>
       </c>
+      <c r="O15" s="31" t="n">
+        <f aca="false">물고기!E6</f>
+        <v>25</v>
+      </c>
+      <c r="P15" s="31" t="n">
+        <f aca="false">물고기!F6</f>
+        <v>50</v>
+      </c>
+      <c r="Q15" s="5" t="n">
+        <f aca="false">물고기!G6</f>
+        <v>30</v>
+      </c>
+      <c r="R15" s="33" t="n">
+        <f aca="false">물고기!I6</f>
+        <v>37.5</v>
+      </c>
+      <c r="S15" s="31" t="n">
+        <f aca="false">물고기!T6</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="C16" s="31" t="str">
         <f aca="false">물고기!B7</f>
@@ -5467,13 +5789,33 @@
         <f aca="false">K16/SUMIF($A$14:$A$44,A16,$K$14:$K$44)*H16</f>
         <v>3.30915513093019</v>
       </c>
+      <c r="O16" s="31" t="n">
+        <f aca="false">물고기!E7</f>
+        <v>30</v>
+      </c>
+      <c r="P16" s="31" t="n">
+        <f aca="false">물고기!F7</f>
+        <v>80</v>
+      </c>
+      <c r="Q16" s="5" t="n">
+        <f aca="false">물고기!G7</f>
+        <v>60</v>
+      </c>
+      <c r="R16" s="33" t="n">
+        <f aca="false">물고기!I7</f>
+        <v>55</v>
+      </c>
+      <c r="S16" s="31" t="n">
+        <f aca="false">물고기!T7</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="C17" s="31" t="str">
         <f aca="false">물고기!B8</f>
@@ -5518,13 +5860,33 @@
         <f aca="false">K17/SUMIF($A$14:$A$44,A17,$K$14:$K$44)*H17</f>
         <v>1.53354420949566</v>
       </c>
+      <c r="O17" s="31" t="n">
+        <f aca="false">물고기!E8</f>
+        <v>6</v>
+      </c>
+      <c r="P17" s="31" t="n">
+        <f aca="false">물고기!F8</f>
+        <v>15</v>
+      </c>
+      <c r="Q17" s="5" t="n">
+        <f aca="false">물고기!G8</f>
+        <v>6</v>
+      </c>
+      <c r="R17" s="33" t="n">
+        <f aca="false">물고기!I8</f>
+        <v>10.5</v>
+      </c>
+      <c r="S17" s="31" t="n">
+        <f aca="false">물고기!T8</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C18" s="31" t="str">
         <f aca="false">물고기!B5</f>
@@ -5569,13 +5931,33 @@
         <f aca="false">K18/SUMIF($A$14:$A$44,A18,$K$14:$K$44)*H18</f>
         <v>2.45367073519305</v>
       </c>
+      <c r="O18" s="31" t="n">
+        <f aca="false">물고기!E5</f>
+        <v>12</v>
+      </c>
+      <c r="P18" s="31" t="n">
+        <f aca="false">물고기!F5</f>
+        <v>30</v>
+      </c>
+      <c r="Q18" s="5" t="n">
+        <f aca="false">물고기!G5</f>
+        <v>12</v>
+      </c>
+      <c r="R18" s="33" t="n">
+        <f aca="false">물고기!I5</f>
+        <v>21</v>
+      </c>
+      <c r="S18" s="31" t="n">
+        <f aca="false">물고기!T5</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="C19" s="31" t="str">
         <f aca="false">물고기!B7</f>
@@ -5620,13 +6002,33 @@
         <f aca="false">K19/SUMIF($A$14:$A$44,A19,$K$14:$K$44)*H19</f>
         <v>8.23432285744928</v>
       </c>
+      <c r="O19" s="31" t="n">
+        <f aca="false">물고기!E7</f>
+        <v>30</v>
+      </c>
+      <c r="P19" s="31" t="n">
+        <f aca="false">물고기!F7</f>
+        <v>80</v>
+      </c>
+      <c r="Q19" s="5" t="n">
+        <f aca="false">물고기!G7</f>
+        <v>60</v>
+      </c>
+      <c r="R19" s="33" t="n">
+        <f aca="false">물고기!I7</f>
+        <v>55</v>
+      </c>
+      <c r="S19" s="31" t="n">
+        <f aca="false">물고기!T7</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="C20" s="31" t="str">
         <f aca="false">물고기!B9</f>
@@ -5671,13 +6073,33 @@
         <f aca="false">K20/SUMIF($A$14:$A$44,A20,$K$14:$K$44)*H20</f>
         <v>8.16657628293983</v>
       </c>
+      <c r="O20" s="31" t="n">
+        <f aca="false">물고기!E9</f>
+        <v>30</v>
+      </c>
+      <c r="P20" s="31" t="n">
+        <f aca="false">물고기!F9</f>
+        <v>90</v>
+      </c>
+      <c r="Q20" s="5" t="n">
+        <f aca="false">물고기!G9</f>
+        <v>70</v>
+      </c>
+      <c r="R20" s="33" t="n">
+        <f aca="false">물고기!I9</f>
+        <v>60</v>
+      </c>
+      <c r="S20" s="31" t="n">
+        <f aca="false">물고기!T9</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="C21" s="31" t="str">
         <f aca="false">물고기!B10</f>
@@ -5722,13 +6144,33 @@
         <f aca="false">K21/SUMIF($A$14:$A$44,A21,$K$14:$K$44)*H21</f>
         <v>10.9526564428104</v>
       </c>
+      <c r="O21" s="31" t="n">
+        <f aca="false">물고기!E10</f>
+        <v>20</v>
+      </c>
+      <c r="P21" s="31" t="n">
+        <f aca="false">물고기!F10</f>
+        <v>55</v>
+      </c>
+      <c r="Q21" s="5" t="n">
+        <f aca="false">물고기!G10</f>
+        <v>160</v>
+      </c>
+      <c r="R21" s="33" t="n">
+        <f aca="false">물고기!I10</f>
+        <v>37.5</v>
+      </c>
+      <c r="S21" s="31" t="n">
+        <f aca="false">물고기!T10</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="C22" s="31" t="str">
         <f aca="false">물고기!B11</f>
@@ -5773,13 +6215,33 @@
         <f aca="false">K22/SUMIF($A$14:$A$44,A22,$K$14:$K$44)*H22</f>
         <v>15.9707675531762</v>
       </c>
+      <c r="O22" s="31" t="n">
+        <f aca="false">물고기!E11</f>
+        <v>40</v>
+      </c>
+      <c r="P22" s="31" t="n">
+        <f aca="false">물고기!F11</f>
+        <v>100</v>
+      </c>
+      <c r="Q22" s="5" t="n">
+        <f aca="false">물고기!G11</f>
+        <v>400</v>
+      </c>
+      <c r="R22" s="33" t="n">
+        <f aca="false">물고기!I11</f>
+        <v>70</v>
+      </c>
+      <c r="S22" s="31" t="n">
+        <f aca="false">물고기!T11</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="C23" s="31" t="str">
         <f aca="false">물고기!B12</f>
@@ -5824,13 +6286,33 @@
         <f aca="false">K23/SUMIF($A$14:$A$44,A23,$K$14:$K$44)*H23</f>
         <v>19.4044825771091</v>
       </c>
+      <c r="O23" s="31" t="n">
+        <f aca="false">물고기!E12</f>
+        <v>80</v>
+      </c>
+      <c r="P23" s="31" t="n">
+        <f aca="false">물고기!F12</f>
+        <v>200</v>
+      </c>
+      <c r="Q23" s="5" t="n">
+        <f aca="false">물고기!G12</f>
+        <v>1800</v>
+      </c>
+      <c r="R23" s="33" t="n">
+        <f aca="false">물고기!I12</f>
+        <v>140</v>
+      </c>
+      <c r="S23" s="31" t="n">
+        <f aca="false">물고기!T12</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="C24" s="31" t="str">
         <f aca="false">물고기!B13</f>
@@ -5875,13 +6357,33 @@
         <f aca="false">K24/SUMIF($A$14:$A$44,A24,$K$14:$K$44)*H24</f>
         <v>2.96082372613453</v>
       </c>
+      <c r="O24" s="31" t="n">
+        <f aca="false">물고기!E13</f>
+        <v>8</v>
+      </c>
+      <c r="P24" s="31" t="n">
+        <f aca="false">물고기!F13</f>
+        <v>25</v>
+      </c>
+      <c r="Q24" s="5" t="n">
+        <f aca="false">물고기!G13</f>
+        <v>15</v>
+      </c>
+      <c r="R24" s="33" t="n">
+        <f aca="false">물고기!I13</f>
+        <v>16.5</v>
+      </c>
+      <c r="S24" s="31" t="n">
+        <f aca="false">물고기!T13</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="C25" s="31" t="str">
         <f aca="false">물고기!B14</f>
@@ -5926,13 +6428,33 @@
         <f aca="false">K25/SUMIF($A$14:$A$44,A25,$K$14:$K$44)*H25</f>
         <v>5.11996946985851</v>
       </c>
+      <c r="O25" s="31" t="n">
+        <f aca="false">물고기!E14</f>
+        <v>15</v>
+      </c>
+      <c r="P25" s="31" t="n">
+        <f aca="false">물고기!F14</f>
+        <v>40</v>
+      </c>
+      <c r="Q25" s="5" t="n">
+        <f aca="false">물고기!G14</f>
+        <v>35</v>
+      </c>
+      <c r="R25" s="33" t="n">
+        <f aca="false">물고기!I14</f>
+        <v>27.5</v>
+      </c>
+      <c r="S25" s="31" t="n">
+        <f aca="false">물고기!T14</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="C26" s="31" t="str">
         <f aca="false">물고기!B15</f>
@@ -5977,13 +6499,33 @@
         <f aca="false">K26/SUMIF($A$14:$A$44,A26,$K$14:$K$44)*H26</f>
         <v>10.0112808105512</v>
       </c>
+      <c r="O26" s="31" t="n">
+        <f aca="false">물고기!E15</f>
+        <v>25</v>
+      </c>
+      <c r="P26" s="31" t="n">
+        <f aca="false">물고기!F15</f>
+        <v>50</v>
+      </c>
+      <c r="Q26" s="5" t="n">
+        <f aca="false">물고기!G15</f>
+        <v>60</v>
+      </c>
+      <c r="R26" s="33" t="n">
+        <f aca="false">물고기!I15</f>
+        <v>37.5</v>
+      </c>
+      <c r="S26" s="31" t="n">
+        <f aca="false">물고기!T15</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="C27" s="31" t="str">
         <f aca="false">물고기!B16</f>
@@ -6028,13 +6570,33 @@
         <f aca="false">K27/SUMIF($A$14:$A$44,A27,$K$14:$K$44)*H27</f>
         <v>16.2496903241016</v>
       </c>
+      <c r="O27" s="31" t="n">
+        <f aca="false">물고기!E16</f>
+        <v>20</v>
+      </c>
+      <c r="P27" s="31" t="n">
+        <f aca="false">물고기!F16</f>
+        <v>50</v>
+      </c>
+      <c r="Q27" s="5" t="n">
+        <f aca="false">물고기!G16</f>
+        <v>150</v>
+      </c>
+      <c r="R27" s="33" t="n">
+        <f aca="false">물고기!I16</f>
+        <v>35</v>
+      </c>
+      <c r="S27" s="31" t="n">
+        <f aca="false">물고기!T16</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="C28" s="31" t="str">
         <f aca="false">물고기!B17</f>
@@ -6079,13 +6641,33 @@
         <f aca="false">K28/SUMIF($A$14:$A$44,A28,$K$14:$K$44)*H28</f>
         <v>44.051295220895</v>
       </c>
+      <c r="O28" s="31" t="n">
+        <f aca="false">물고기!E17</f>
+        <v>25</v>
+      </c>
+      <c r="P28" s="31" t="n">
+        <f aca="false">물고기!F17</f>
+        <v>60</v>
+      </c>
+      <c r="Q28" s="5" t="n">
+        <f aca="false">물고기!G17</f>
+        <v>450</v>
+      </c>
+      <c r="R28" s="33" t="n">
+        <f aca="false">물고기!I17</f>
+        <v>42.5</v>
+      </c>
+      <c r="S28" s="31" t="n">
+        <f aca="false">물고기!T17</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="C29" s="31" t="str">
         <f aca="false">물고기!B18</f>
@@ -6130,13 +6712,33 @@
         <f aca="false">K29/SUMIF($A$14:$A$44,A29,$K$14:$K$44)*H29</f>
         <v>39.6086201649976</v>
       </c>
+      <c r="O29" s="31" t="n">
+        <f aca="false">물고기!E18</f>
+        <v>40</v>
+      </c>
+      <c r="P29" s="31" t="n">
+        <f aca="false">물고기!F18</f>
+        <v>100</v>
+      </c>
+      <c r="Q29" s="5" t="n">
+        <f aca="false">물고기!G18</f>
+        <v>650</v>
+      </c>
+      <c r="R29" s="33" t="n">
+        <f aca="false">물고기!I18</f>
+        <v>70</v>
+      </c>
+      <c r="S29" s="31" t="n">
+        <f aca="false">물고기!T18</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="C30" s="31" t="str">
         <f aca="false">물고기!B19</f>
@@ -6181,13 +6783,33 @@
         <f aca="false">K30/SUMIF($A$14:$A$44,A30,$K$14:$K$44)*H30</f>
         <v>23.7867689719066</v>
       </c>
+      <c r="O30" s="31" t="n">
+        <f aca="false">물고기!E19</f>
+        <v>25</v>
+      </c>
+      <c r="P30" s="31" t="n">
+        <f aca="false">물고기!F19</f>
+        <v>55</v>
+      </c>
+      <c r="Q30" s="5" t="n">
+        <f aca="false">물고기!G19</f>
+        <v>550</v>
+      </c>
+      <c r="R30" s="33" t="n">
+        <f aca="false">물고기!I19</f>
+        <v>40</v>
+      </c>
+      <c r="S30" s="31" t="n">
+        <f aca="false">물고기!T19</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="C31" s="31" t="str">
         <f aca="false">물고기!B20</f>
@@ -6232,13 +6854,33 @@
         <f aca="false">K31/SUMIF($A$14:$A$44,A31,$K$14:$K$44)*H31</f>
         <v>26.5098393957261</v>
       </c>
+      <c r="O31" s="31" t="n">
+        <f aca="false">물고기!E20</f>
+        <v>30</v>
+      </c>
+      <c r="P31" s="31" t="n">
+        <f aca="false">물고기!F20</f>
+        <v>70</v>
+      </c>
+      <c r="Q31" s="5" t="n">
+        <f aca="false">물고기!G20</f>
+        <v>1600</v>
+      </c>
+      <c r="R31" s="33" t="n">
+        <f aca="false">물고기!I20</f>
+        <v>50</v>
+      </c>
+      <c r="S31" s="31" t="n">
+        <f aca="false">물고기!T20</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="C32" s="31" t="str">
         <f aca="false">물고기!B21</f>
@@ -6283,13 +6925,33 @@
         <f aca="false">K32/SUMIF($A$14:$A$44,A32,$K$14:$K$44)*H32</f>
         <v>32.6228464589079</v>
       </c>
+      <c r="O32" s="31" t="n">
+        <f aca="false">물고기!E21</f>
+        <v>60</v>
+      </c>
+      <c r="P32" s="31" t="n">
+        <f aca="false">물고기!F21</f>
+        <v>150</v>
+      </c>
+      <c r="Q32" s="5" t="n">
+        <f aca="false">물고기!G21</f>
+        <v>180</v>
+      </c>
+      <c r="R32" s="33" t="n">
+        <f aca="false">물고기!I21</f>
+        <v>105</v>
+      </c>
+      <c r="S32" s="31" t="n">
+        <f aca="false">물고기!T21</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="C33" s="31" t="str">
         <f aca="false">물고기!B22</f>
@@ -6334,13 +6996,33 @@
         <f aca="false">K33/SUMIF($A$14:$A$44,A33,$K$14:$K$44)*H33</f>
         <v>87.854863080623</v>
       </c>
+      <c r="O33" s="31" t="n">
+        <f aca="false">물고기!E22</f>
+        <v>35</v>
+      </c>
+      <c r="P33" s="31" t="n">
+        <f aca="false">물고기!F22</f>
+        <v>90</v>
+      </c>
+      <c r="Q33" s="5" t="n">
+        <f aca="false">물고기!G22</f>
+        <v>450</v>
+      </c>
+      <c r="R33" s="33" t="n">
+        <f aca="false">물고기!I22</f>
+        <v>62.5</v>
+      </c>
+      <c r="S33" s="31" t="n">
+        <f aca="false">물고기!T22</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="C34" s="31" t="str">
         <f aca="false">물고기!B23</f>
@@ -6385,13 +7067,33 @@
         <f aca="false">K34/SUMIF($A$14:$A$44,A34,$K$14:$K$44)*H34</f>
         <v>175.897880579644</v>
       </c>
+      <c r="O34" s="31" t="n">
+        <f aca="false">물고기!E23</f>
+        <v>30</v>
+      </c>
+      <c r="P34" s="31" t="n">
+        <f aca="false">물고기!F23</f>
+        <v>90</v>
+      </c>
+      <c r="Q34" s="5" t="n">
+        <f aca="false">물고기!G23</f>
+        <v>900</v>
+      </c>
+      <c r="R34" s="33" t="n">
+        <f aca="false">물고기!I23</f>
+        <v>60</v>
+      </c>
+      <c r="S34" s="31" t="n">
+        <f aca="false">물고기!T23</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="C35" s="31" t="str">
         <f aca="false">물고기!B24</f>
@@ -6436,13 +7138,33 @@
         <f aca="false">K35/SUMIF($A$14:$A$44,A35,$K$14:$K$44)*H35</f>
         <v>203.172715707247</v>
       </c>
+      <c r="O35" s="31" t="n">
+        <f aca="false">물고기!E24</f>
+        <v>50</v>
+      </c>
+      <c r="P35" s="31" t="n">
+        <f aca="false">물고기!F24</f>
+        <v>110</v>
+      </c>
+      <c r="Q35" s="5" t="n">
+        <f aca="false">물고기!G24</f>
+        <v>1400</v>
+      </c>
+      <c r="R35" s="33" t="n">
+        <f aca="false">물고기!I24</f>
+        <v>80</v>
+      </c>
+      <c r="S35" s="31" t="n">
+        <f aca="false">물고기!T24</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="C36" s="31" t="str">
         <f aca="false">물고기!B25</f>
@@ -6487,13 +7209,33 @@
         <f aca="false">K36/SUMIF($A$14:$A$44,A36,$K$14:$K$44)*H36</f>
         <v>195.144039323999</v>
       </c>
+      <c r="O36" s="31" t="n">
+        <f aca="false">물고기!E25</f>
+        <v>60</v>
+      </c>
+      <c r="P36" s="31" t="n">
+        <f aca="false">물고기!F25</f>
+        <v>140</v>
+      </c>
+      <c r="Q36" s="5" t="n">
+        <f aca="false">물고기!G25</f>
+        <v>2200</v>
+      </c>
+      <c r="R36" s="33" t="n">
+        <f aca="false">물고기!I25</f>
+        <v>100</v>
+      </c>
+      <c r="S36" s="31" t="n">
+        <f aca="false">물고기!T25</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="C37" s="31" t="str">
         <f aca="false">물고기!B26</f>
@@ -6538,13 +7280,33 @@
         <f aca="false">K37/SUMIF($A$14:$A$44,A37,$K$14:$K$44)*H37</f>
         <v>265.042927558541</v>
       </c>
+      <c r="O37" s="31" t="n">
+        <f aca="false">물고기!E26</f>
+        <v>100</v>
+      </c>
+      <c r="P37" s="31" t="n">
+        <f aca="false">물고기!F26</f>
+        <v>280</v>
+      </c>
+      <c r="Q37" s="5" t="n">
+        <f aca="false">물고기!G26</f>
+        <v>9000</v>
+      </c>
+      <c r="R37" s="33" t="n">
+        <f aca="false">물고기!I26</f>
+        <v>190</v>
+      </c>
+      <c r="S37" s="31" t="n">
+        <f aca="false">물고기!T26</f>
+        <v>4</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="C38" s="31" t="str">
         <f aca="false">물고기!B23</f>
@@ -6589,13 +7351,33 @@
         <f aca="false">K38/SUMIF($A$14:$A$44,A38,$K$14:$K$44)*H38</f>
         <v>152.41709788788</v>
       </c>
+      <c r="O38" s="31" t="n">
+        <f aca="false">물고기!E23</f>
+        <v>30</v>
+      </c>
+      <c r="P38" s="31" t="n">
+        <f aca="false">물고기!F23</f>
+        <v>90</v>
+      </c>
+      <c r="Q38" s="5" t="n">
+        <f aca="false">물고기!G23</f>
+        <v>900</v>
+      </c>
+      <c r="R38" s="33" t="n">
+        <f aca="false">물고기!I23</f>
+        <v>60</v>
+      </c>
+      <c r="S38" s="31" t="n">
+        <f aca="false">물고기!T23</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="C39" s="31" t="str">
         <f aca="false">물고기!B24</f>
@@ -6640,13 +7422,33 @@
         <f aca="false">K39/SUMIF($A$14:$A$44,A39,$K$14:$K$44)*H39</f>
         <v>182.822180052464</v>
       </c>
+      <c r="O39" s="31" t="n">
+        <f aca="false">물고기!E24</f>
+        <v>50</v>
+      </c>
+      <c r="P39" s="31" t="n">
+        <f aca="false">물고기!F24</f>
+        <v>110</v>
+      </c>
+      <c r="Q39" s="5" t="n">
+        <f aca="false">물고기!G24</f>
+        <v>1400</v>
+      </c>
+      <c r="R39" s="33" t="n">
+        <f aca="false">물고기!I24</f>
+        <v>80</v>
+      </c>
+      <c r="S39" s="31" t="n">
+        <f aca="false">물고기!T24</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="C40" s="31" t="str">
         <f aca="false">물고기!B25</f>
@@ -6691,13 +7493,33 @@
         <f aca="false">K40/SUMIF($A$14:$A$44,A40,$K$14:$K$44)*H40</f>
         <v>228.27699152441</v>
       </c>
+      <c r="O40" s="31" t="n">
+        <f aca="false">물고기!E25</f>
+        <v>60</v>
+      </c>
+      <c r="P40" s="31" t="n">
+        <f aca="false">물고기!F25</f>
+        <v>140</v>
+      </c>
+      <c r="Q40" s="5" t="n">
+        <f aca="false">물고기!G25</f>
+        <v>2200</v>
+      </c>
+      <c r="R40" s="33" t="n">
+        <f aca="false">물고기!I25</f>
+        <v>100</v>
+      </c>
+      <c r="S40" s="31" t="n">
+        <f aca="false">물고기!T25</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="C41" s="31" t="str">
         <f aca="false">물고기!B28</f>
@@ -6742,13 +7564,33 @@
         <f aca="false">K41/SUMIF($A$14:$A$44,A41,$K$14:$K$44)*H41</f>
         <v>317.400074948772</v>
       </c>
+      <c r="O41" s="31" t="n">
+        <f aca="false">물고기!E28</f>
+        <v>90</v>
+      </c>
+      <c r="P41" s="31" t="n">
+        <f aca="false">물고기!F28</f>
+        <v>180</v>
+      </c>
+      <c r="Q41" s="5" t="n">
+        <f aca="false">물고기!G28</f>
+        <v>1800</v>
+      </c>
+      <c r="R41" s="33" t="n">
+        <f aca="false">물고기!I28</f>
+        <v>135</v>
+      </c>
+      <c r="S41" s="31" t="n">
+        <f aca="false">물고기!T28</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="C42" s="31" t="str">
         <f aca="false">물고기!B27</f>
@@ -6793,13 +7635,33 @@
         <f aca="false">K42/SUMIF($A$14:$A$44,A42,$K$14:$K$44)*H42</f>
         <v>452.352779227973</v>
       </c>
+      <c r="O42" s="31" t="n">
+        <f aca="false">물고기!E27</f>
+        <v>30</v>
+      </c>
+      <c r="P42" s="31" t="n">
+        <f aca="false">물고기!F27</f>
+        <v>55</v>
+      </c>
+      <c r="Q42" s="5" t="n">
+        <f aca="false">물고기!G27</f>
+        <v>2500</v>
+      </c>
+      <c r="R42" s="33" t="n">
+        <f aca="false">물고기!I27</f>
+        <v>42.5</v>
+      </c>
+      <c r="S42" s="31" t="n">
+        <f aca="false">물고기!T27</f>
+        <v>4</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="C43" s="31" t="str">
         <f aca="false">물고기!B29</f>
@@ -6844,13 +7706,33 @@
         <f aca="false">K43/SUMIF($A$14:$A$44,A43,$K$14:$K$44)*H43</f>
         <v>418.98388435873</v>
       </c>
+      <c r="O43" s="31" t="n">
+        <f aca="false">물고기!E29</f>
+        <v>50</v>
+      </c>
+      <c r="P43" s="31" t="n">
+        <f aca="false">물고기!F29</f>
+        <v>120</v>
+      </c>
+      <c r="Q43" s="5" t="n">
+        <f aca="false">물고기!G29</f>
+        <v>6000</v>
+      </c>
+      <c r="R43" s="33" t="n">
+        <f aca="false">물고기!I29</f>
+        <v>85</v>
+      </c>
+      <c r="S43" s="31" t="n">
+        <f aca="false">물고기!T29</f>
+        <v>4</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="C44" s="31" t="str">
         <f aca="false">물고기!B30</f>
@@ -6894,6 +7776,26 @@
       <c r="N44" s="20" t="n">
         <f aca="false">K44/SUMIF($A$14:$A$44,A44,$K$14:$K$44)*H44</f>
         <v>352.585632958324</v>
+      </c>
+      <c r="O44" s="31" t="n">
+        <f aca="false">물고기!E30</f>
+        <v>100</v>
+      </c>
+      <c r="P44" s="31" t="n">
+        <f aca="false">물고기!F30</f>
+        <v>220</v>
+      </c>
+      <c r="Q44" s="5" t="n">
+        <f aca="false">물고기!G30</f>
+        <v>20000</v>
+      </c>
+      <c r="R44" s="33" t="n">
+        <f aca="false">물고기!I30</f>
+        <v>160</v>
+      </c>
+      <c r="S44" s="31" t="n">
+        <f aca="false">물고기!T30</f>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -6913,6 +7815,467 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:S10"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="11" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="14" style="0" width="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="20.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="N5" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="O5" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="P5" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="Q5" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="R5" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="S5" s="3" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="C6" s="12" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D6" s="20" t="n">
+        <f aca="false">SUM($C$6:C6)</f>
+        <v>5000</v>
+      </c>
+      <c r="E6" s="32" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="F6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="28" t="n">
+        <f aca="false">MAX(0.9,가정!$B$5-F6*가정!$B$6)</f>
+        <v>1.8</v>
+      </c>
+      <c r="H6" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="I6" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="J6" s="27" t="n">
+        <f aca="false">H6*I6/60</f>
+        <v>6</v>
+      </c>
+      <c r="K6" s="20" t="n">
+        <f aca="false">SUMPRODUCT((낚시터!$A$14:$A$44="강")*낚시터!$E$14:$E$44*(1+$F6*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E6*낚시터!$S$14:$S$44)*낚시터!$Q$14:$Q$44*(낚시터!$O$14:$O$44^2+2*낚시터!$O$14:$O$44*(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)/(1+$G6)+(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)^2/(1+2*$G6))/낚시터!$R$14:$R$44^2)/SUMPRODUCT((낚시터!$A$14:$A$44="강")*낚시터!$E$14:$E$44*(1+$F6*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E6*낚시터!$S$14:$S$44))</f>
+        <v>40.1249414961122</v>
+      </c>
+      <c r="L6" s="20" t="n">
+        <f aca="false">SUMPRODUCT((낚시터!$A$14:$A$44="방파제")*낚시터!$E$14:$E$44*(1+$F6*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E6*낚시터!$S$14:$S$44)*낚시터!$Q$14:$Q$44*(낚시터!$O$14:$O$44^2+2*낚시터!$O$14:$O$44*(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)/(1+$G6)+(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)^2/(1+2*$G6))/낚시터!$R$14:$R$44^2)/SUMPRODUCT((낚시터!$A$14:$A$44="방파제")*낚시터!$E$14:$E$44*(1+$F6*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E6*낚시터!$S$14:$S$44))</f>
+        <v>103.912533263905</v>
+      </c>
+      <c r="M6" s="20" t="n">
+        <f aca="false">SUMPRODUCT((낚시터!$A$14:$A$44="배낚시")*낚시터!$E$14:$E$44*(1+$F6*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E6*낚시터!$S$14:$S$44)*낚시터!$Q$14:$Q$44*(낚시터!$O$14:$O$44^2+2*낚시터!$O$14:$O$44*(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)/(1+$G6)+(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)^2/(1+2*$G6))/낚시터!$R$14:$R$44^2)/SUMPRODUCT((낚시터!$A$14:$A$44="배낚시")*낚시터!$E$14:$E$44*(1+$F6*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E6*낚시터!$S$14:$S$44))</f>
+        <v>669.037825681728</v>
+      </c>
+      <c r="N6" s="20" t="n">
+        <f aca="false">K6/$H6*60</f>
+        <v>26.7499609974081</v>
+      </c>
+      <c r="O6" s="20" t="n">
+        <f aca="false">L6/$H6*60</f>
+        <v>69.2750221759369</v>
+      </c>
+      <c r="P6" s="20" t="n">
+        <f aca="false">M6/$H6*60</f>
+        <v>446.025217121152</v>
+      </c>
+      <c r="Q6" s="24" t="n">
+        <f aca="false">C6/N6</f>
+        <v>186.916160381859</v>
+      </c>
+      <c r="R6" s="24" t="n">
+        <f aca="false">C6/O6</f>
+        <v>72.1760866030698</v>
+      </c>
+      <c r="S6" s="24" t="n">
+        <f aca="false">C6/P6</f>
+        <v>11.2101285041062</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>285</v>
+      </c>
+      <c r="C7" s="12" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D7" s="20" t="n">
+        <f aca="false">SUM($C$6:C7)</f>
+        <v>25000</v>
+      </c>
+      <c r="E7" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="21" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G7" s="28" t="n">
+        <f aca="false">MAX(0.9,가정!$B$5-F7*가정!$B$6)</f>
+        <v>1.74</v>
+      </c>
+      <c r="H7" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="I7" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J7" s="27" t="n">
+        <f aca="false">H7*I7/60</f>
+        <v>7.5</v>
+      </c>
+      <c r="K7" s="20" t="n">
+        <f aca="false">SUMPRODUCT((낚시터!$A$14:$A$44="강")*낚시터!$E$14:$E$44*(1+$F7*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E7*낚시터!$S$14:$S$44)*낚시터!$Q$14:$Q$44*(낚시터!$O$14:$O$44^2+2*낚시터!$O$14:$O$44*(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)/(1+$G7)+(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)^2/(1+2*$G7))/낚시터!$R$14:$R$44^2)/SUMPRODUCT((낚시터!$A$14:$A$44="강")*낚시터!$E$14:$E$44*(1+$F7*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E7*낚시터!$S$14:$S$44))</f>
+        <v>49.5180852401902</v>
+      </c>
+      <c r="L7" s="20" t="n">
+        <f aca="false">SUMPRODUCT((낚시터!$A$14:$A$44="방파제")*낚시터!$E$14:$E$44*(1+$F7*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E7*낚시터!$S$14:$S$44)*낚시터!$Q$14:$Q$44*(낚시터!$O$14:$O$44^2+2*낚시터!$O$14:$O$44*(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)/(1+$G7)+(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)^2/(1+2*$G7))/낚시터!$R$14:$R$44^2)/SUMPRODUCT((낚시터!$A$14:$A$44="방파제")*낚시터!$E$14:$E$44*(1+$F7*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E7*낚시터!$S$14:$S$44))</f>
+        <v>128.475845166968</v>
+      </c>
+      <c r="M7" s="20" t="n">
+        <f aca="false">SUMPRODUCT((낚시터!$A$14:$A$44="배낚시")*낚시터!$E$14:$E$44*(1+$F7*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E7*낚시터!$S$14:$S$44)*낚시터!$Q$14:$Q$44*(낚시터!$O$14:$O$44^2+2*낚시터!$O$14:$O$44*(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)/(1+$G7)+(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)^2/(1+2*$G7))/낚시터!$R$14:$R$44^2)/SUMPRODUCT((낚시터!$A$14:$A$44="배낚시")*낚시터!$E$14:$E$44*(1+$F7*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E7*낚시터!$S$14:$S$44))</f>
+        <v>789.785857921675</v>
+      </c>
+      <c r="N7" s="20" t="n">
+        <f aca="false">K7/$H7*60</f>
+        <v>39.6144681921522</v>
+      </c>
+      <c r="O7" s="20" t="n">
+        <f aca="false">L7/$H7*60</f>
+        <v>102.780676133575</v>
+      </c>
+      <c r="P7" s="20" t="n">
+        <f aca="false">M7/$H7*60</f>
+        <v>631.82868633734</v>
+      </c>
+      <c r="Q7" s="24" t="n">
+        <f aca="false">C7/N7</f>
+        <v>504.866048005211</v>
+      </c>
+      <c r="R7" s="24" t="n">
+        <f aca="false">C7/O7</f>
+        <v>194.589107139243</v>
+      </c>
+      <c r="S7" s="24" t="n">
+        <f aca="false">C7/P7</f>
+        <v>31.6541499816008</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>286</v>
+      </c>
+      <c r="C8" s="12" t="n">
+        <v>60000</v>
+      </c>
+      <c r="D8" s="20" t="n">
+        <f aca="false">SUM($C$6:C8)</f>
+        <v>85000</v>
+      </c>
+      <c r="E8" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F8" s="21" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G8" s="28" t="n">
+        <f aca="false">MAX(0.9,가정!$B$5-F8*가정!$B$6)</f>
+        <v>1.68</v>
+      </c>
+      <c r="H8" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="I8" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="J8" s="27" t="n">
+        <f aca="false">H8*I8/60</f>
+        <v>8</v>
+      </c>
+      <c r="K8" s="20" t="n">
+        <f aca="false">SUMPRODUCT((낚시터!$A$14:$A$44="강")*낚시터!$E$14:$E$44*(1+$F8*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E8*낚시터!$S$14:$S$44)*낚시터!$Q$14:$Q$44*(낚시터!$O$14:$O$44^2+2*낚시터!$O$14:$O$44*(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)/(1+$G8)+(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)^2/(1+2*$G8))/낚시터!$R$14:$R$44^2)/SUMPRODUCT((낚시터!$A$14:$A$44="강")*낚시터!$E$14:$E$44*(1+$F8*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E8*낚시터!$S$14:$S$44))</f>
+        <v>61.9406825153851</v>
+      </c>
+      <c r="L8" s="20" t="n">
+        <f aca="false">SUMPRODUCT((낚시터!$A$14:$A$44="방파제")*낚시터!$E$14:$E$44*(1+$F8*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E8*낚시터!$S$14:$S$44)*낚시터!$Q$14:$Q$44*(낚시터!$O$14:$O$44^2+2*낚시터!$O$14:$O$44*(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)/(1+$G8)+(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)^2/(1+2*$G8))/낚시터!$R$14:$R$44^2)/SUMPRODUCT((낚시터!$A$14:$A$44="방파제")*낚시터!$E$14:$E$44*(1+$F8*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E8*낚시터!$S$14:$S$44))</f>
+        <v>158.133562968333</v>
+      </c>
+      <c r="M8" s="20" t="n">
+        <f aca="false">SUMPRODUCT((낚시터!$A$14:$A$44="배낚시")*낚시터!$E$14:$E$44*(1+$F8*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E8*낚시터!$S$14:$S$44)*낚시터!$Q$14:$Q$44*(낚시터!$O$14:$O$44^2+2*낚시터!$O$14:$O$44*(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)/(1+$G8)+(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)^2/(1+2*$G8))/낚시터!$R$14:$R$44^2)/SUMPRODUCT((낚시터!$A$14:$A$44="배낚시")*낚시터!$E$14:$E$44*(1+$F8*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E8*낚시터!$S$14:$S$44))</f>
+        <v>922.671797924911</v>
+      </c>
+      <c r="N8" s="20" t="n">
+        <f aca="false">K8/$H8*60</f>
+        <v>61.9406825153851</v>
+      </c>
+      <c r="O8" s="20" t="n">
+        <f aca="false">L8/$H8*60</f>
+        <v>158.133562968333</v>
+      </c>
+      <c r="P8" s="20" t="n">
+        <f aca="false">M8/$H8*60</f>
+        <v>922.671797924911</v>
+      </c>
+      <c r="Q8" s="24" t="n">
+        <f aca="false">C8/N8</f>
+        <v>968.668693392214</v>
+      </c>
+      <c r="R8" s="24" t="n">
+        <f aca="false">C8/O8</f>
+        <v>379.426093194494</v>
+      </c>
+      <c r="S8" s="24" t="n">
+        <f aca="false">C8/P8</f>
+        <v>65.0285400886209</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>287</v>
+      </c>
+      <c r="C9" s="12" t="n">
+        <v>150000</v>
+      </c>
+      <c r="D9" s="20" t="n">
+        <f aca="false">SUM($C$6:C9)</f>
+        <v>235000</v>
+      </c>
+      <c r="E9" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="21" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G9" s="28" t="n">
+        <f aca="false">MAX(0.9,가정!$B$5-F9*가정!$B$6)</f>
+        <v>1.59</v>
+      </c>
+      <c r="H9" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="I9" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="J9" s="27" t="n">
+        <f aca="false">H9*I9/60</f>
+        <v>7.5</v>
+      </c>
+      <c r="K9" s="20" t="n">
+        <f aca="false">SUMPRODUCT((낚시터!$A$14:$A$44="강")*낚시터!$E$14:$E$44*(1+$F9*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E9*낚시터!$S$14:$S$44)*낚시터!$Q$14:$Q$44*(낚시터!$O$14:$O$44^2+2*낚시터!$O$14:$O$44*(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)/(1+$G9)+(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)^2/(1+2*$G9))/낚시터!$R$14:$R$44^2)/SUMPRODUCT((낚시터!$A$14:$A$44="강")*낚시터!$E$14:$E$44*(1+$F9*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E9*낚시터!$S$14:$S$44))</f>
+        <v>80.4270102664426</v>
+      </c>
+      <c r="L9" s="20" t="n">
+        <f aca="false">SUMPRODUCT((낚시터!$A$14:$A$44="방파제")*낚시터!$E$14:$E$44*(1+$F9*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E9*낚시터!$S$14:$S$44)*낚시터!$Q$14:$Q$44*(낚시터!$O$14:$O$44^2+2*낚시터!$O$14:$O$44*(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)/(1+$G9)+(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)^2/(1+2*$G9))/낚시터!$R$14:$R$44^2)/SUMPRODUCT((낚시터!$A$14:$A$44="방파제")*낚시터!$E$14:$E$44*(1+$F9*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E9*낚시터!$S$14:$S$44))</f>
+        <v>197.21479632833</v>
+      </c>
+      <c r="M9" s="20" t="n">
+        <f aca="false">SUMPRODUCT((낚시터!$A$14:$A$44="배낚시")*낚시터!$E$14:$E$44*(1+$F9*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E9*낚시터!$S$14:$S$44)*낚시터!$Q$14:$Q$44*(낚시터!$O$14:$O$44^2+2*낚시터!$O$14:$O$44*(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)/(1+$G9)+(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)^2/(1+2*$G9))/낚시터!$R$14:$R$44^2)/SUMPRODUCT((낚시터!$A$14:$A$44="배낚시")*낚시터!$E$14:$E$44*(1+$F9*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E9*낚시터!$S$14:$S$44))</f>
+        <v>1083.78606344074</v>
+      </c>
+      <c r="N9" s="20" t="n">
+        <f aca="false">K9/$H9*60</f>
+        <v>107.23601368859</v>
+      </c>
+      <c r="O9" s="20" t="n">
+        <f aca="false">L9/$H9*60</f>
+        <v>262.953061771107</v>
+      </c>
+      <c r="P9" s="20" t="n">
+        <f aca="false">M9/$H9*60</f>
+        <v>1445.04808458766</v>
+      </c>
+      <c r="Q9" s="24" t="n">
+        <f aca="false">C9/N9</f>
+        <v>1398.78381189733</v>
+      </c>
+      <c r="R9" s="24" t="n">
+        <f aca="false">C9/O9</f>
+        <v>570.44401380871</v>
+      </c>
+      <c r="S9" s="24" t="n">
+        <f aca="false">C9/P9</f>
+        <v>103.802774177444</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>288</v>
+      </c>
+      <c r="C10" s="12" t="n">
+        <v>400000</v>
+      </c>
+      <c r="D10" s="20" t="n">
+        <f aca="false">SUM($C$6:C10)</f>
+        <v>635000</v>
+      </c>
+      <c r="E10" s="32" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="F10" s="21" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G10" s="28" t="n">
+        <f aca="false">MAX(0.9,가정!$B$5-F10*가정!$B$6)</f>
+        <v>1.5</v>
+      </c>
+      <c r="H10" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="I10" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="J10" s="27" t="n">
+        <f aca="false">H10*I10/60</f>
+        <v>6</v>
+      </c>
+      <c r="K10" s="20" t="n">
+        <f aca="false">SUMPRODUCT((낚시터!$A$14:$A$44="강")*낚시터!$E$14:$E$44*(1+$F10*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E10*낚시터!$S$14:$S$44)*낚시터!$Q$14:$Q$44*(낚시터!$O$14:$O$44^2+2*낚시터!$O$14:$O$44*(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)/(1+$G10)+(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)^2/(1+2*$G10))/낚시터!$R$14:$R$44^2)/SUMPRODUCT((낚시터!$A$14:$A$44="강")*낚시터!$E$14:$E$44*(1+$F10*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E10*낚시터!$S$14:$S$44))</f>
+        <v>109.708620355131</v>
+      </c>
+      <c r="L10" s="20" t="n">
+        <f aca="false">SUMPRODUCT((낚시터!$A$14:$A$44="방파제")*낚시터!$E$14:$E$44*(1+$F10*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E10*낚시터!$S$14:$S$44)*낚시터!$Q$14:$Q$44*(낚시터!$O$14:$O$44^2+2*낚시터!$O$14:$O$44*(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)/(1+$G10)+(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)^2/(1+2*$G10))/낚시터!$R$14:$R$44^2)/SUMPRODUCT((낚시터!$A$14:$A$44="방파제")*낚시터!$E$14:$E$44*(1+$F10*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E10*낚시터!$S$14:$S$44))</f>
+        <v>249.554053224506</v>
+      </c>
+      <c r="M10" s="20" t="n">
+        <f aca="false">SUMPRODUCT((낚시터!$A$14:$A$44="배낚시")*낚시터!$E$14:$E$44*(1+$F10*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E10*낚시터!$S$14:$S$44)*낚시터!$Q$14:$Q$44*(낚시터!$O$14:$O$44^2+2*낚시터!$O$14:$O$44*(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)/(1+$G10)+(낚시터!$P$14:$P$44-낚시터!$O$14:$O$44)^2/(1+2*$G10))/낚시터!$R$14:$R$44^2)/SUMPRODUCT((낚시터!$A$14:$A$44="배낚시")*낚시터!$E$14:$E$44*(1+$F10*낚시터!$S$14:$S$44*가정!$B$7)*(1+가정!$B$27)^($E10*낚시터!$S$14:$S$44))</f>
+        <v>1284.16349788298</v>
+      </c>
+      <c r="N10" s="20" t="n">
+        <f aca="false">K10/$H10*60</f>
+        <v>219.417240710263</v>
+      </c>
+      <c r="O10" s="20" t="n">
+        <f aca="false">L10/$H10*60</f>
+        <v>499.108106449011</v>
+      </c>
+      <c r="P10" s="20" t="n">
+        <f aca="false">M10/$H10*60</f>
+        <v>2568.32699576596</v>
+      </c>
+      <c r="Q10" s="24" t="n">
+        <f aca="false">C10/N10</f>
+        <v>1823.01080218302</v>
+      </c>
+      <c r="R10" s="24" t="n">
+        <f aca="false">C10/O10</f>
+        <v>801.429579747497</v>
+      </c>
+      <c r="S10" s="24" t="n">
+        <f aca="false">C10/P10</f>
+        <v>155.743408319666</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:F9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -6926,132 +8289,132 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>258</v>
+        <v>289</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>259</v>
+        <v>290</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>260</v>
+        <v>291</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>261</v>
+        <v>292</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>262</v>
+        <v>293</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>263</v>
+        <v>294</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="B5" s="14" t="n">
         <v>3</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>264</v>
+        <v>295</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>265</v>
-      </c>
-      <c r="E5" s="33" t="n">
+        <v>296</v>
+      </c>
+      <c r="E5" s="34" t="n">
         <v>2</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>266</v>
+        <v>297</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="B6" s="14" t="n">
         <v>7</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>267</v>
+        <v>298</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>268</v>
+        <v>299</v>
       </c>
       <c r="E6" s="21" t="n">
         <v>0.1</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>269</v>
+        <v>300</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="B7" s="14" t="n">
         <v>8</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>270</v>
+        <v>301</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>271</v>
+        <v>302</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>0.3</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>272</v>
+        <v>303</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="B8" s="14" t="n">
         <v>6</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>273</v>
+        <v>304</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>274</v>
+        <v>305</v>
       </c>
       <c r="E8" s="21" t="n">
         <v>0.1</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>275</v>
+        <v>306</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="B9" s="14" t="n">
         <v>4</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>276</v>
+        <v>307</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>277</v>
-      </c>
-      <c r="E9" s="33" t="n">
+        <v>308</v>
+      </c>
+      <c r="E9" s="34" t="n">
         <v>30</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>278</v>
+        <v>309</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Weather events, auto-sell, progress-based quests, boss summon, shore landing
- Size medals pay 0.2/0.5/1x base price (was 2/5/15x)
- Weather events per 3-min window: fish schools, strong current (harder, x1.2 price), feeding, deep fog
- Hooked fish now land in front of the shore under the rod tip
- Quests follow the furthest unlocked stages and refresh unfinished ones on unlock; all-done bonus is 5 big-fish baits instead of a Busan ticket
- Nets about 15-20% cheaper
- Completed stage dex lets you summon that stage's boss (tap the boss panel or press B)
- Auto-sell for known fish up to a chosen grade that don't beat any record; also applies to nets
- Indoor/stream dex rewards: slower cast gauge, +5% sell price (keep net perks removed)
- Busan dex and stage card list all 7 fish that appear there
</commit_message>
<xml_diff>
--- a/bukangi-fishing-balance.xlsx
+++ b/bukangi-fishing-balance.xlsx
@@ -52,7 +52,23 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">. </t>
+          <t xml:space="preserve">(</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Noto Sans CJK SC"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">날씨 이벤트 없는 상태</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">). </t>
         </r>
         <r>
           <rPr>
@@ -123,6 +139,50 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">마리 기대가 정도</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B50" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Noto Sans CJK SC"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">예전엔 부산 이용권 </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">1</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Noto Sans CJK SC"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">장</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">. </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Noto Sans CJK SC"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">낚시터를 건너뛸 수 있어 대물 미끼로 바꿈</t>
         </r>
       </text>
     </comment>
@@ -523,7 +583,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="836" uniqueCount="525">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="867" uniqueCount="555">
   <si>
     <t xml:space="preserve">부캉이 낚시터 밸런스 요약</t>
   </si>
@@ -645,7 +705,10 @@
     <t xml:space="preserve">부산 도감 완성 시 +30초</t>
   </si>
   <si>
-    <t xml:space="preserve">살림망 칸 수 (실내 도감 완성 시)</t>
+    <t xml:space="preserve">살림망 칸 수</t>
+  </si>
+  <si>
+    <t xml:space="preserve">자동 판매가 생겨 도감 보상에서 뺌</t>
   </si>
   <si>
     <t xml:space="preserve">기본 대 적정 구간 (가장 쉬운 붕어)</t>
@@ -667,9 +730,6 @@
   </si>
   <si>
     <t xml:space="preserve">출처 / 설명</t>
-  </si>
-  <si>
-    <t xml:space="preserve">살림망 칸 수</t>
   </si>
   <si>
     <t xml:space="preserve">CONFIG.keepNetSize</t>
@@ -1757,7 +1817,7 @@
     <t xml:space="preserve">크기 메달</t>
   </si>
   <si>
-    <t xml:space="preserve">몸길이 범위의 몇 % 지점 이상이면 메달입니다. 처음 받는 단계마다 그 종 기준가 × 보상 배수를 받습니다(동→금을 한 번에 넘으면 셋 다).</t>
+    <t xml:space="preserve">몸길이 범위의 몇 % 지점 이상이면 메달입니다. 처음 받는 단계마다 그 종 기준가 × 보상 배수를 받습니다(동→금을 한 번에 넘으면 셋 다). 예전 2·5·15배에서 0.2·0.5·1배로 낮춤.</t>
   </si>
   <si>
     <t xml:space="preserve">메달</t>
@@ -1892,6 +1952,78 @@
     <t xml:space="preserve">비 / 맑음</t>
   </si>
   <si>
+    <t xml:space="preserve">날씨 이벤트 (날씨 구간마다, 낚시터마다 정해짐)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">구간마다 이벤트가 생길 확률</t>
+  </si>
+  <si>
+    <t xml:space="preserve">이벤트</t>
+  </si>
+  <si>
+    <t xml:space="preserve">생기는 날씨</t>
+  </si>
+  <si>
+    <t xml:space="preserve">출현 배수</t>
+  </si>
+  <si>
+    <t xml:space="preserve">난이도 +</t>
+  </si>
+  <si>
+    <t xml:space="preserve">판매가 배수</t>
+  </si>
+  <si>
+    <t xml:space="preserve">입질 대기 배수</t>
+  </si>
+  <si>
+    <t xml:space="preserve">좋은 물고기 보정</t>
+  </si>
+  <si>
+    <t xml:space="preserve">물고기 떼</t>
+  </si>
+  <si>
+    <t xml:space="preserve">맑음, 비, 안개, 눈보라</t>
+  </si>
+  <si>
+    <t xml:space="preserve">떼가 몰려왔어요 · 그 물고기 출현 3배</t>
+  </si>
+  <si>
+    <t xml:space="preserve">거센 물살</t>
+  </si>
+  <si>
+    <t xml:space="preserve">비, 눈보라</t>
+  </si>
+  <si>
+    <t xml:space="preserve">물고기 힘이 세져 잡기 어렵지만 판매가 ×1.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">먹이 활동</t>
+  </si>
+  <si>
+    <t xml:space="preserve">맑음</t>
+  </si>
+  <si>
+    <t xml:space="preserve">입질이 훨씬 빨라져요</t>
+  </si>
+  <si>
+    <t xml:space="preserve">안개 속 대물</t>
+  </si>
+  <si>
+    <t xml:space="preserve">안개</t>
+  </si>
+  <si>
+    <t xml:space="preserve">좋은 물고기가 늘지만 입질이 느려요</t>
+  </si>
+  <si>
+    <t xml:space="preserve">맑을 때 이벤트별 확률 (물고기 떼·먹이 활동)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">비·눈보라일 때 거센 물살 확률</t>
+  </si>
+  <si>
+    <t xml:space="preserve">안개일 때 안개 속 대물 확률</t>
+  </si>
+  <si>
     <t xml:space="preserve">수족관 · 특수 미끼 · 낚시 대회 · 환생 · 의뢰 · 희귀 변종</t>
   </si>
   <si>
@@ -2020,13 +2152,10 @@
     <t xml:space="preserve">환생 레벨</t>
   </si>
   <si>
-    <t xml:space="preserve">판매가 배수</t>
-  </si>
-  <si>
     <t xml:space="preserve">보스 기척 1마리당</t>
   </si>
   <si>
-    <t xml:space="preserve">오늘의 의뢰 (하루 3개, 열린 맵 중 가장 뒤 맵 기준)</t>
+    <t xml:space="preserve">오늘의 의뢰 (하루 3개, 연 낚시터 중 가장 먼 2곳 기준. 새 낚시터를 열면 못 끝낸 의뢰가 바뀜)</t>
   </si>
   <si>
     <t xml:space="preserve">보상 배수 최소·최대</t>
@@ -2035,7 +2164,10 @@
     <t xml:space="preserve">판매 의뢰 목표 = 1마리 기대가 ×</t>
   </si>
   <si>
-    <t xml:space="preserve">세 개 모두 완료 보너스 (부산 이용권)</t>
+    <t xml:space="preserve">의뢰에 쓰는 최근 낚시터 수</t>
+  </si>
+  <si>
+    <t xml:space="preserve">세 개 모두 완료 보너스 (대물 미끼 횟수)</t>
   </si>
   <si>
     <t xml:space="preserve">가장 뒤 맵</t>
@@ -2071,10 +2203,22 @@
     <t xml:space="preserve">황금 미끼 +5일 때 (안개면 2배)</t>
   </si>
   <si>
+    <t xml:space="preserve">자동 판매</t>
+  </si>
+  <si>
+    <t xml:space="preserve">처음 설정 (이 등급까지 자동 판매)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">조건</t>
+  </si>
+  <si>
+    <t xml:space="preserve">이미 잡아 본 종류 · 고른 등급 이하 · 그 종류의 최대 크기·최고가·최고 등급·메달을 넘지 않음 · 변종·보스 아님</t>
+  </si>
+  <si>
     <t xml:space="preserve">도감 완성 보상</t>
   </si>
   <si>
-    <t xml:space="preserve">낚시터의 물고기를 모두 한 번 이상 잡으면 받는 작은 편의 효과입니다. 부산은 부산 전용 어종 기준입니다.</t>
+    <t xml:space="preserve">낚시터의 물고기를 모두 한 번 이상 잡으면 받는 작은 편의 효과입니다. 부산은 나오는 7종(전용 4종 + 참돔·방어·부시리) 기준입니다.</t>
   </si>
   <si>
     <t xml:space="preserve">채워야 할 종 수</t>
@@ -2089,16 +2233,22 @@
     <t xml:space="preserve">게임에서 쓰이는 곳</t>
   </si>
   <si>
-    <t xml:space="preserve">살림망 +2칸</t>
-  </si>
-  <si>
-    <t xml:space="preserve">net</t>
-  </si>
-  <si>
-    <t xml:space="preserve">살림망 칸 수에 더함</t>
-  </si>
-  <si>
-    <t xml:space="preserve">살림망 +1칸</t>
+    <t xml:space="preserve">캐스팅 게이지 15% 느려짐</t>
+  </si>
+  <si>
+    <t xml:space="preserve">castSlow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">캐스팅 게이지 속도에 (1−수치)를 곱함</t>
+  </si>
+  <si>
+    <t xml:space="preserve">판매가 +5%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sell</t>
+  </si>
+  <si>
+    <t xml:space="preserve">판매가에 더함 (환생 보너스와 합산)</t>
   </si>
   <si>
     <t xml:space="preserve">챔질 판정 10% 넓어짐</t>
@@ -3093,7 +3243,7 @@
       </c>
       <c r="B28" s="5" t="n">
         <f aca="false">그물!D10</f>
-        <v>635000</v>
+        <v>535000</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>34</v>
@@ -3146,26 +3296,28 @@
         <v>40</v>
       </c>
       <c r="B33" s="7" t="n">
-        <f aca="false">가정!$B$4+'도감 보상'!E5</f>
-        <v>17</v>
-      </c>
-      <c r="C33" s="4"/>
+        <f aca="false">가정!$B$4</f>
+        <v>15</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B34" s="8" t="n">
         <f aca="false">물고기!R5</f>
         <v>0.24495</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B35" s="8" t="n">
         <f aca="false">물고기!R51</f>
@@ -3175,7 +3327,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B36" s="8" t="n">
         <f aca="false">물고기!S51</f>
@@ -3199,12 +3351,15 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="44"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3578,6 +3733,176 @@
       <c r="G27" s="36" t="n">
         <f aca="false">D27/B27</f>
         <v>1.03349031920461</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="30" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="4" t="s">
+        <v>442</v>
+      </c>
+      <c r="B30" s="21" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="3" t="s">
+        <v>443</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>444</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>446</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>448</v>
+      </c>
+      <c r="G31" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="H31" s="3" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="11" t="s">
+        <v>450</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="C32" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D32" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="4" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="11" t="s">
+        <v>453</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>454</v>
+      </c>
+      <c r="C33" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="22" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E33" s="22" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F33" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="4" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="11" t="s">
+        <v>456</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>457</v>
+      </c>
+      <c r="C34" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="22" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G34" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="11" t="s">
+        <v>459</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>460</v>
+      </c>
+      <c r="C35" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" s="22" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="G35" s="22" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4" t="s">
+        <v>462</v>
+      </c>
+      <c r="B36" s="29" t="n">
+        <f aca="false">B30/2</f>
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="4" t="s">
+        <v>463</v>
+      </c>
+      <c r="B37" s="29" t="n">
+        <f aca="false">B30/2</f>
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="4" t="s">
+        <v>464</v>
+      </c>
+      <c r="B38" s="29" t="n">
+        <f aca="false">B30/2</f>
+        <v>0.25</v>
       </c>
     </row>
   </sheetData>
@@ -3597,7 +3922,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G65"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="36"/>
@@ -3609,17 +3934,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="20.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>441</v>
+        <v>465</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="30" t="s">
-        <v>442</v>
+        <v>466</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>443</v>
+        <v>467</v>
       </c>
       <c r="B4" s="21" t="n">
         <v>0.1</v>
@@ -3627,7 +3952,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>444</v>
+        <v>468</v>
       </c>
       <c r="B5" s="9" t="n">
         <v>24</v>
@@ -3635,7 +3960,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>445</v>
+        <v>469</v>
       </c>
       <c r="B6" s="12" t="n">
         <v>2000</v>
@@ -3643,30 +3968,30 @@
     </row>
     <row r="8" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>446</v>
+        <v>470</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>447</v>
+        <v>471</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>128</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>448</v>
+        <v>472</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>449</v>
+        <v>473</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>450</v>
+        <v>474</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>451</v>
+        <v>475</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>452</v>
+        <v>476</v>
       </c>
       <c r="B9" s="12" t="n">
         <v>20000</v>
@@ -3693,7 +4018,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>453</v>
+        <v>477</v>
       </c>
       <c r="B10" s="12" t="n">
         <v>60000</v>
@@ -3720,7 +4045,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>454</v>
+        <v>478</v>
       </c>
       <c r="B11" s="12" t="n">
         <v>150000</v>
@@ -3747,7 +4072,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>455</v>
+        <v>479</v>
       </c>
       <c r="B12" s="12" t="n">
         <v>400000</v>
@@ -3774,7 +4099,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>456</v>
+        <v>480</v>
       </c>
       <c r="B13" s="12" t="n">
         <v>1000000</v>
@@ -3801,7 +4126,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="30" t="s">
-        <v>457</v>
+        <v>481</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3809,21 +4134,21 @@
         <v>178</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>458</v>
+        <v>482</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>459</v>
+        <v>483</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>460</v>
+        <v>484</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>461</v>
+        <v>485</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>462</v>
+        <v>486</v>
       </c>
       <c r="B17" s="12" t="n">
         <v>3000</v>
@@ -3836,12 +4161,12 @@
         <v>300</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>463</v>
+        <v>487</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>464</v>
+        <v>488</v>
       </c>
       <c r="B18" s="12" t="n">
         <v>8000</v>
@@ -3854,12 +4179,12 @@
         <v>800</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>465</v>
+        <v>489</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>466</v>
+        <v>490</v>
       </c>
       <c r="B19" s="12" t="n">
         <v>15000</v>
@@ -3872,17 +4197,17 @@
         <v>15000</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>467</v>
+        <v>491</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="30" t="s">
-        <v>468</v>
+        <v>492</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>469</v>
+        <v>493</v>
       </c>
       <c r="B22" s="9" t="n">
         <v>180</v>
@@ -3890,7 +4215,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>470</v>
+        <v>494</v>
       </c>
       <c r="B23" s="9" t="n">
         <v>10</v>
@@ -3898,7 +4223,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>471</v>
+        <v>495</v>
       </c>
       <c r="B24" s="32" t="n">
         <v>6</v>
@@ -3918,19 +4243,19 @@
         <v>312</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>472</v>
+        <v>496</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>473</v>
+        <v>497</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>474</v>
+        <v>498</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>475</v>
+        <v>499</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>476</v>
+        <v>500</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3955,7 +4280,7 @@
         <v>345</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>477</v>
+        <v>501</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3980,7 +4305,7 @@
         <v>705</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>477</v>
+        <v>501</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4005,7 +4330,7 @@
         <v>1830</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>477</v>
+        <v>501</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4030,7 +4355,7 @@
         <v>4035</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>477</v>
+        <v>501</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4055,7 +4380,7 @@
         <v>11370</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>477</v>
+        <v>501</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4080,7 +4405,7 @@
         <v>18930</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>477</v>
+        <v>501</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4105,17 +4430,17 @@
         <v>30135</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>477</v>
+        <v>501</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="30" t="s">
-        <v>478</v>
+        <v>502</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>479</v>
+        <v>503</v>
       </c>
       <c r="B36" s="21" t="n">
         <v>0.1</v>
@@ -4123,7 +4448,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>480</v>
+        <v>504</v>
       </c>
       <c r="B37" s="21" t="n">
         <v>0.1</v>
@@ -4131,7 +4456,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>481</v>
+        <v>505</v>
       </c>
       <c r="B38" s="12" t="n">
         <v>150</v>
@@ -4139,13 +4464,13 @@
     </row>
     <row r="39" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>482</v>
+        <v>506</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>483</v>
+        <v>447</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>484</v>
+        <v>507</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4215,12 +4540,12 @@
     </row>
     <row r="46" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="30" t="s">
-        <v>485</v>
+        <v>508</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="4" t="s">
-        <v>486</v>
+        <v>509</v>
       </c>
       <c r="B47" s="9" t="n">
         <v>10</v>
@@ -4231,7 +4556,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>487</v>
+        <v>510</v>
       </c>
       <c r="B48" s="9" t="n">
         <v>25</v>
@@ -4239,168 +4564,168 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="4" t="s">
-        <v>488</v>
+        <v>511</v>
       </c>
       <c r="B49" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="3" t="s">
-        <v>489</v>
-      </c>
-      <c r="B50" s="3" t="s">
-        <v>490</v>
-      </c>
-      <c r="C50" s="3" t="s">
-        <v>491</v>
-      </c>
-      <c r="D50" s="3" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="31" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="4" t="s">
+        <v>512</v>
+      </c>
+      <c r="B50" s="9" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="3" t="s">
+        <v>513</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>514</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="31" t="str">
         <f aca="false">낚시터!B6</f>
         <v>하천</v>
       </c>
-      <c r="B51" s="20" t="n">
+      <c r="B52" s="20" t="n">
         <f aca="false">낚시터!F6*$B$47</f>
         <v>229.060014687636</v>
       </c>
-      <c r="C51" s="20" t="n">
+      <c r="C52" s="20" t="n">
         <f aca="false">낚시터!F6*$C$47</f>
         <v>366.496023500217</v>
       </c>
-      <c r="D51" s="20" t="n">
+      <c r="D52" s="20" t="n">
         <f aca="false">낚시터!F6*$B$48</f>
         <v>572.650036719089</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="31" t="str">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="31" t="str">
         <f aca="false">낚시터!B7</f>
         <v>강</v>
       </c>
-      <c r="B52" s="20" t="n">
+      <c r="B53" s="20" t="n">
         <f aca="false">낚시터!F7*$B$47</f>
         <v>470.148669809363</v>
       </c>
-      <c r="C52" s="20" t="n">
+      <c r="C53" s="20" t="n">
         <f aca="false">낚시터!F7*$C$47</f>
         <v>752.237871694981</v>
       </c>
-      <c r="D52" s="20" t="n">
+      <c r="D53" s="20" t="n">
         <f aca="false">낚시터!F7*$B$48</f>
         <v>1175.37167452341</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="31" t="str">
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="31" t="str">
         <f aca="false">낚시터!B8</f>
         <v>방파제</v>
       </c>
-      <c r="B53" s="20" t="n">
+      <c r="B54" s="20" t="n">
         <f aca="false">낚시터!F8*$B$47</f>
         <v>1222.21537481253</v>
       </c>
-      <c r="C53" s="20" t="n">
+      <c r="C54" s="20" t="n">
         <f aca="false">낚시터!F8*$C$47</f>
         <v>1955.54459970004</v>
       </c>
-      <c r="D53" s="20" t="n">
+      <c r="D54" s="20" t="n">
         <f aca="false">낚시터!F8*$B$48</f>
         <v>3055.53843703132</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="31" t="str">
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="31" t="str">
         <f aca="false">낚시터!B9</f>
         <v>독도</v>
       </c>
-      <c r="B54" s="20" t="n">
+      <c r="B55" s="20" t="n">
         <f aca="false">낚시터!F9*$B$47</f>
         <v>2694.29188313713</v>
       </c>
-      <c r="C54" s="20" t="n">
+      <c r="C55" s="20" t="n">
         <f aca="false">낚시터!F9*$C$47</f>
         <v>4310.8670130194</v>
       </c>
-      <c r="D54" s="20" t="n">
+      <c r="D55" s="20" t="n">
         <f aca="false">낚시터!F9*$B$48</f>
         <v>6735.72970784282</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="31" t="str">
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="31" t="str">
         <f aca="false">낚시터!B10</f>
         <v>배낚시</v>
       </c>
-      <c r="B55" s="20" t="n">
+      <c r="B56" s="20" t="n">
         <f aca="false">낚시터!F10*$B$47</f>
         <v>7582.69279988315</v>
       </c>
-      <c r="C55" s="20" t="n">
+      <c r="C56" s="20" t="n">
         <f aca="false">낚시터!F10*$C$47</f>
         <v>12132.308479813</v>
       </c>
-      <c r="D55" s="20" t="n">
+      <c r="D56" s="20" t="n">
         <f aca="false">낚시터!F10*$B$48</f>
         <v>18956.7319997079</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="31" t="str">
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="31" t="str">
         <f aca="false">낚시터!B11</f>
         <v>아마존</v>
       </c>
-      <c r="B56" s="20" t="n">
+      <c r="B57" s="20" t="n">
         <f aca="false">낚시터!F11*$B$47</f>
         <v>12618.3027138793</v>
       </c>
-      <c r="C56" s="20" t="n">
+      <c r="C57" s="20" t="n">
         <f aca="false">낚시터!F11*$C$47</f>
         <v>20189.2843422068</v>
       </c>
-      <c r="D56" s="20" t="n">
+      <c r="D57" s="20" t="n">
         <f aca="false">낚시터!F11*$B$48</f>
         <v>31545.7567846982</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="31" t="str">
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="31" t="str">
         <f aca="false">낚시터!B12</f>
         <v>알래스카</v>
       </c>
-      <c r="B57" s="20" t="n">
+      <c r="B58" s="20" t="n">
         <f aca="false">낚시터!F12*$B$47</f>
         <v>20088.3703106896</v>
       </c>
-      <c r="C57" s="20" t="n">
+      <c r="C58" s="20" t="n">
         <f aca="false">낚시터!F12*$C$47</f>
         <v>32141.3924971033</v>
       </c>
-      <c r="D57" s="20" t="n">
+      <c r="D58" s="20" t="n">
         <f aca="false">낚시터!F12*$B$48</f>
         <v>50220.9257767239</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="30" t="s">
-        <v>493</v>
-      </c>
-    </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="4" t="s">
-        <v>494</v>
-      </c>
-      <c r="B60" s="10" t="n">
-        <v>0.01</v>
+      <c r="A60" s="30" t="s">
+        <v>517</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="4" t="s">
-        <v>495</v>
+        <v>518</v>
       </c>
       <c r="B61" s="10" t="n">
         <v>0.01</v>
@@ -4408,42 +4733,75 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="4" t="s">
-        <v>496</v>
-      </c>
-      <c r="B62" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="C62" s="37" t="n">
-        <v>5</v>
+        <v>519</v>
+      </c>
+      <c r="B62" s="10" t="n">
+        <v>0.01</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="4" t="s">
-        <v>497</v>
+        <v>520</v>
       </c>
       <c r="B63" s="21" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="C63" s="37" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="4" t="s">
-        <v>498</v>
-      </c>
-      <c r="B64" s="29" t="n">
-        <f aca="false">$B$60</f>
-        <v>0.01</v>
+        <v>521</v>
+      </c>
+      <c r="B64" s="21" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C64" s="37" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="4" t="s">
-        <v>499</v>
+        <v>522</v>
       </c>
       <c r="B65" s="29" t="n">
-        <f aca="false">$B$60+1.3*$B$61</f>
+        <f aca="false">$B$61</f>
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="4" t="s">
+        <v>523</v>
+      </c>
+      <c r="B66" s="29" t="n">
+        <f aca="false">$B$61+1.3*$B$62</f>
         <v>0.023</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="30" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="4" t="s">
+        <v>525</v>
+      </c>
+      <c r="B69" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C69" s="4" t="str">
+        <f aca="false">IF(B69&lt;0,"끔",INDEX(등급!$A$4:$A$8,B69+1))</f>
+        <v>고급</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="4" t="s">
+        <v>526</v>
+      </c>
+      <c r="B70" s="4" t="s">
+        <v>527</v>
       </c>
     </row>
   </sheetData>
@@ -4476,12 +4834,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>500</v>
+        <v>528</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>501</v>
+        <v>529</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4489,19 +4847,19 @@
         <v>312</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>502</v>
+        <v>530</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>503</v>
+        <v>531</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>504</v>
+        <v>532</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>129</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>505</v>
+        <v>533</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4512,16 +4870,16 @@
         <v>3</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>506</v>
+        <v>534</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>507</v>
-      </c>
-      <c r="E5" s="35" t="n">
-        <v>2</v>
+        <v>535</v>
+      </c>
+      <c r="E5" s="21" t="n">
+        <v>0.15</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>508</v>
+        <v>536</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4532,16 +4890,16 @@
         <v>6</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>509</v>
+        <v>537</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>507</v>
-      </c>
-      <c r="E6" s="35" t="n">
-        <v>1</v>
+        <v>538</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>0.05</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>508</v>
+        <v>539</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4552,16 +4910,16 @@
         <v>7</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>510</v>
+        <v>540</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>511</v>
+        <v>541</v>
       </c>
       <c r="E7" s="21" t="n">
         <v>0.1</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>512</v>
+        <v>542</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4572,16 +4930,16 @@
         <v>8</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>513</v>
+        <v>543</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>514</v>
+        <v>544</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>0.3</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>515</v>
+        <v>545</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4592,16 +4950,16 @@
         <v>7</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>516</v>
+        <v>546</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>511</v>
+        <v>541</v>
       </c>
       <c r="E9" s="21" t="n">
         <v>0.05</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>512</v>
+        <v>542</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4612,16 +4970,16 @@
         <v>6</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>517</v>
+        <v>547</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>518</v>
+        <v>548</v>
       </c>
       <c r="E10" s="21" t="n">
         <v>0.1</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>519</v>
+        <v>549</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4632,16 +4990,16 @@
         <v>6</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>520</v>
+        <v>550</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>514</v>
+        <v>544</v>
       </c>
       <c r="E11" s="32" t="n">
         <v>0.2</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>515</v>
+        <v>545</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4652,36 +5010,36 @@
         <v>7</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>521</v>
+        <v>551</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>518</v>
+        <v>548</v>
       </c>
       <c r="E12" s="21" t="n">
         <v>0.05</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>519</v>
+        <v>549</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>195</v>
+        <v>338</v>
       </c>
       <c r="B13" s="14" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>522</v>
+        <v>552</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>523</v>
+        <v>553</v>
       </c>
       <c r="E13" s="35" t="n">
         <v>30</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>524</v>
+        <v>554</v>
       </c>
     </row>
   </sheetData>
@@ -4710,12 +5068,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="20.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4726,12 +5084,12 @@
         <v>3</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="B4" s="9" t="n">
         <v>15</v>
@@ -5108,7 +5466,7 @@
         <v>110</v>
       </c>
       <c r="D4" s="14" t="n">
-        <f aca="false">COUNTIF(물고기!$O$5:$O$40,A4)</f>
+        <f aca="false">COUNTIF(물고기!$O$5:$O$200,A4)</f>
         <v>7</v>
       </c>
     </row>
@@ -5123,7 +5481,7 @@
         <v>112</v>
       </c>
       <c r="D5" s="14" t="n">
-        <f aca="false">COUNTIF(물고기!$O$5:$O$40,A5)</f>
+        <f aca="false">COUNTIF(물고기!$O$5:$O$200,A5)</f>
         <v>5</v>
       </c>
     </row>
@@ -5138,7 +5496,7 @@
         <v>114</v>
       </c>
       <c r="D6" s="14" t="n">
-        <f aca="false">COUNTIF(물고기!$O$5:$O$40,A6)</f>
+        <f aca="false">COUNTIF(물고기!$O$5:$O$200,A6)</f>
         <v>7</v>
       </c>
     </row>
@@ -5153,8 +5511,8 @@
         <v>116</v>
       </c>
       <c r="D7" s="14" t="n">
-        <f aca="false">COUNTIF(물고기!$O$5:$O$40,A7)</f>
-        <v>7</v>
+        <f aca="false">COUNTIF(물고기!$O$5:$O$200,A7)</f>
+        <v>8</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5168,8 +5526,8 @@
         <v>118</v>
       </c>
       <c r="D8" s="14" t="n">
-        <f aca="false">COUNTIF(물고기!$O$5:$O$40,A8)</f>
-        <v>10</v>
+        <f aca="false">COUNTIF(물고기!$O$5:$O$200,A8)</f>
+        <v>20</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14435,11 +14793,11 @@
         <v>369</v>
       </c>
       <c r="C6" s="12" t="n">
-        <v>5000</v>
+        <v>4000</v>
       </c>
       <c r="D6" s="20" t="n">
         <f aca="false">SUM($C$6:C6)</f>
-        <v>5000</v>
+        <v>4000</v>
       </c>
       <c r="E6" s="32" t="n">
         <v>-0.5</v>
@@ -14487,15 +14845,15 @@
       </c>
       <c r="Q6" s="24" t="n">
         <f aca="false">C6/N6</f>
-        <v>186.916160381859</v>
+        <v>149.532928305487</v>
       </c>
       <c r="R6" s="24" t="n">
         <f aca="false">C6/O6</f>
-        <v>11.2101285041062</v>
+        <v>8.96810280328499</v>
       </c>
       <c r="S6" s="24" t="n">
         <f aca="false">C6/P6</f>
-        <v>3.85917359405891</v>
+        <v>3.08733887524713</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14506,11 +14864,11 @@
         <v>370</v>
       </c>
       <c r="C7" s="12" t="n">
-        <v>20000</v>
+        <v>16000</v>
       </c>
       <c r="D7" s="20" t="n">
         <f aca="false">SUM($C$6:C7)</f>
-        <v>25000</v>
+        <v>20000</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>0</v>
@@ -14558,15 +14916,15 @@
       </c>
       <c r="Q7" s="24" t="n">
         <f aca="false">C7/N7</f>
-        <v>504.866048005211</v>
+        <v>403.892838404169</v>
       </c>
       <c r="R7" s="24" t="n">
         <f aca="false">C7/O7</f>
-        <v>31.6541499816008</v>
+        <v>25.3233199852807</v>
       </c>
       <c r="S7" s="24" t="n">
         <f aca="false">C7/P7</f>
-        <v>12.2090187392485</v>
+        <v>9.7672149913988</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14577,11 +14935,11 @@
         <v>371</v>
       </c>
       <c r="C8" s="12" t="n">
-        <v>60000</v>
+        <v>50000</v>
       </c>
       <c r="D8" s="20" t="n">
         <f aca="false">SUM($C$6:C8)</f>
-        <v>85000</v>
+        <v>70000</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>0.5</v>
@@ -14629,15 +14987,15 @@
       </c>
       <c r="Q8" s="24" t="n">
         <f aca="false">C8/N8</f>
-        <v>968.668693392214</v>
+        <v>807.223911160178</v>
       </c>
       <c r="R8" s="24" t="n">
         <f aca="false">C8/O8</f>
-        <v>65.0285400886209</v>
+        <v>54.1904500738508</v>
       </c>
       <c r="S8" s="24" t="n">
         <f aca="false">C8/P8</f>
-        <v>27.7558582189626</v>
+        <v>23.1298818491355</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14648,11 +15006,11 @@
         <v>372</v>
       </c>
       <c r="C9" s="12" t="n">
-        <v>150000</v>
+        <v>125000</v>
       </c>
       <c r="D9" s="20" t="n">
         <f aca="false">SUM($C$6:C9)</f>
-        <v>235000</v>
+        <v>195000</v>
       </c>
       <c r="E9" s="32" t="n">
         <v>1</v>
@@ -14700,15 +15058,15 @@
       </c>
       <c r="Q9" s="24" t="n">
         <f aca="false">C9/N9</f>
-        <v>1398.78381189733</v>
+        <v>1165.65317658111</v>
       </c>
       <c r="R9" s="24" t="n">
         <f aca="false">C9/O9</f>
-        <v>103.802774177444</v>
+        <v>86.5023118145364</v>
       </c>
       <c r="S9" s="24" t="n">
         <f aca="false">C9/P9</f>
-        <v>48.766583127312</v>
+        <v>40.63881927276</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14719,11 +15077,11 @@
         <v>373</v>
       </c>
       <c r="C10" s="12" t="n">
-        <v>400000</v>
+        <v>340000</v>
       </c>
       <c r="D10" s="20" t="n">
         <f aca="false">SUM($C$6:C10)</f>
-        <v>635000</v>
+        <v>535000</v>
       </c>
       <c r="E10" s="32" t="n">
         <v>1.6</v>
@@ -14771,15 +15129,15 @@
       </c>
       <c r="Q10" s="24" t="n">
         <f aca="false">C10/N10</f>
-        <v>1823.01080218302</v>
+        <v>1549.55918185557</v>
       </c>
       <c r="R10" s="24" t="n">
         <f aca="false">C10/O10</f>
-        <v>155.743408319666</v>
+        <v>132.381897071716</v>
       </c>
       <c r="S10" s="24" t="n">
         <f aca="false">C10/P10</f>
-        <v>80.4687637863487</v>
+        <v>68.3984492183964</v>
       </c>
     </row>
   </sheetData>
@@ -15312,8 +15670,8 @@
       <c r="B5" s="21" t="n">
         <v>0.7</v>
       </c>
-      <c r="C5" s="9" t="n">
-        <v>2</v>
+      <c r="C5" s="32" t="n">
+        <v>0.2</v>
       </c>
       <c r="D5" s="29" t="n">
         <f aca="false">1-B5^(1/가정!$B$5)</f>
@@ -15331,8 +15689,8 @@
       <c r="B6" s="21" t="n">
         <v>0.85</v>
       </c>
-      <c r="C6" s="9" t="n">
-        <v>5</v>
+      <c r="C6" s="32" t="n">
+        <v>0.5</v>
       </c>
       <c r="D6" s="29" t="n">
         <f aca="false">1-B6^(1/가정!$B$5)</f>
@@ -15350,8 +15708,8 @@
       <c r="B7" s="21" t="n">
         <v>0.95</v>
       </c>
-      <c r="C7" s="9" t="n">
-        <v>15</v>
+      <c r="C7" s="32" t="n">
+        <v>1</v>
       </c>
       <c r="D7" s="29" t="n">
         <f aca="false">1-B7^(1/가정!$B$5)</f>
@@ -15419,7 +15777,7 @@
       </c>
       <c r="H10" s="20" t="n">
         <f aca="false">D10*SUM($C$5:$C$7)</f>
-        <v>264</v>
+        <v>20.4</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15453,7 +15811,7 @@
       </c>
       <c r="H11" s="20" t="n">
         <f aca="false">D11*SUM($C$5:$C$7)</f>
-        <v>660</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15487,7 +15845,7 @@
       </c>
       <c r="H12" s="20" t="n">
         <f aca="false">D12*SUM($C$5:$C$7)</f>
-        <v>1320</v>
+        <v>102</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15521,7 +15879,7 @@
       </c>
       <c r="H13" s="20" t="n">
         <f aca="false">D13*SUM($C$5:$C$7)</f>
-        <v>132</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15555,7 +15913,7 @@
       </c>
       <c r="H14" s="20" t="n">
         <f aca="false">D14*SUM($C$5:$C$7)</f>
-        <v>1540</v>
+        <v>119</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15589,7 +15947,7 @@
       </c>
       <c r="H15" s="20" t="n">
         <f aca="false">D15*SUM($C$5:$C$7)</f>
-        <v>3520</v>
+        <v>272</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15623,7 +15981,7 @@
       </c>
       <c r="H16" s="20" t="n">
         <f aca="false">D16*SUM($C$5:$C$7)</f>
-        <v>8800</v>
+        <v>680</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15657,7 +16015,7 @@
       </c>
       <c r="H17" s="20" t="n">
         <f aca="false">D17*SUM($C$5:$C$7)</f>
-        <v>39600</v>
+        <v>3060</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15691,7 +16049,7 @@
       </c>
       <c r="H18" s="20" t="n">
         <f aca="false">D18*SUM($C$5:$C$7)</f>
-        <v>330</v>
+        <v>25.5</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15725,7 +16083,7 @@
       </c>
       <c r="H19" s="20" t="n">
         <f aca="false">D19*SUM($C$5:$C$7)</f>
-        <v>770</v>
+        <v>59.5</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15759,7 +16117,7 @@
       </c>
       <c r="H20" s="20" t="n">
         <f aca="false">D20*SUM($C$5:$C$7)</f>
-        <v>1320</v>
+        <v>102</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15793,7 +16151,7 @@
       </c>
       <c r="H21" s="20" t="n">
         <f aca="false">D21*SUM($C$5:$C$7)</f>
-        <v>3300</v>
+        <v>255</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15827,7 +16185,7 @@
       </c>
       <c r="H22" s="20" t="n">
         <f aca="false">D22*SUM($C$5:$C$7)</f>
-        <v>9900</v>
+        <v>765</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15861,7 +16219,7 @@
       </c>
       <c r="H23" s="20" t="n">
         <f aca="false">D23*SUM($C$5:$C$7)</f>
-        <v>14300</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15895,7 +16253,7 @@
       </c>
       <c r="H24" s="20" t="n">
         <f aca="false">D24*SUM($C$5:$C$7)</f>
-        <v>12100</v>
+        <v>935</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15929,7 +16287,7 @@
       </c>
       <c r="H25" s="20" t="n">
         <f aca="false">D25*SUM($C$5:$C$7)</f>
-        <v>35200</v>
+        <v>2720</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15963,7 +16321,7 @@
       </c>
       <c r="H26" s="20" t="n">
         <f aca="false">D26*SUM($C$5:$C$7)</f>
-        <v>3960</v>
+        <v>306</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15997,7 +16355,7 @@
       </c>
       <c r="H27" s="20" t="n">
         <f aca="false">D27*SUM($C$5:$C$7)</f>
-        <v>9900</v>
+        <v>765</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16031,7 +16389,7 @@
       </c>
       <c r="H28" s="20" t="n">
         <f aca="false">D28*SUM($C$5:$C$7)</f>
-        <v>19800</v>
+        <v>1530</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16065,7 +16423,7 @@
       </c>
       <c r="H29" s="20" t="n">
         <f aca="false">D29*SUM($C$5:$C$7)</f>
-        <v>30800</v>
+        <v>2380</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16099,7 +16457,7 @@
       </c>
       <c r="H30" s="20" t="n">
         <f aca="false">D30*SUM($C$5:$C$7)</f>
-        <v>48400</v>
+        <v>3740</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16133,7 +16491,7 @@
       </c>
       <c r="H31" s="20" t="n">
         <f aca="false">D31*SUM($C$5:$C$7)</f>
-        <v>198000</v>
+        <v>15300</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16167,7 +16525,7 @@
       </c>
       <c r="H32" s="20" t="n">
         <f aca="false">D32*SUM($C$5:$C$7)</f>
-        <v>176</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16201,7 +16559,7 @@
       </c>
       <c r="H33" s="20" t="n">
         <f aca="false">D33*SUM($C$5:$C$7)</f>
-        <v>264</v>
+        <v>20.4</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16235,7 +16593,7 @@
       </c>
       <c r="H34" s="20" t="n">
         <f aca="false">D34*SUM($C$5:$C$7)</f>
-        <v>550</v>
+        <v>42.5</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16269,7 +16627,7 @@
       </c>
       <c r="H35" s="20" t="n">
         <f aca="false">D35*SUM($C$5:$C$7)</f>
-        <v>1540</v>
+        <v>119</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16303,7 +16661,7 @@
       </c>
       <c r="H36" s="20" t="n">
         <f aca="false">D36*SUM($C$5:$C$7)</f>
-        <v>3300</v>
+        <v>255</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16337,7 +16695,7 @@
       </c>
       <c r="H37" s="20" t="n">
         <f aca="false">D37*SUM($C$5:$C$7)</f>
-        <v>2640</v>
+        <v>204</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16371,7 +16729,7 @@
       </c>
       <c r="H38" s="20" t="n">
         <f aca="false">D38*SUM($C$5:$C$7)</f>
-        <v>3960</v>
+        <v>306</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16405,7 +16763,7 @@
       </c>
       <c r="H39" s="20" t="n">
         <f aca="false">D39*SUM($C$5:$C$7)</f>
-        <v>39600</v>
+        <v>3060</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16439,7 +16797,7 @@
       </c>
       <c r="H40" s="20" t="n">
         <f aca="false">D40*SUM($C$5:$C$7)</f>
-        <v>6600</v>
+        <v>510</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16473,7 +16831,7 @@
       </c>
       <c r="H41" s="20" t="n">
         <f aca="false">D41*SUM($C$5:$C$7)</f>
-        <v>15400</v>
+        <v>1190</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16507,7 +16865,7 @@
       </c>
       <c r="H42" s="20" t="n">
         <f aca="false">D42*SUM($C$5:$C$7)</f>
-        <v>33000</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16541,7 +16899,7 @@
       </c>
       <c r="H43" s="20" t="n">
         <f aca="false">D43*SUM($C$5:$C$7)</f>
-        <v>57200</v>
+        <v>4420</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16575,7 +16933,7 @@
       </c>
       <c r="H44" s="20" t="n">
         <f aca="false">D44*SUM($C$5:$C$7)</f>
-        <v>61600</v>
+        <v>4760</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16609,7 +16967,7 @@
       </c>
       <c r="H45" s="20" t="n">
         <f aca="false">D45*SUM($C$5:$C$7)</f>
-        <v>352000</v>
+        <v>27200</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16643,7 +17001,7 @@
       </c>
       <c r="H46" s="20" t="n">
         <f aca="false">D46*SUM($C$5:$C$7)</f>
-        <v>22000</v>
+        <v>1700</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16677,7 +17035,7 @@
       </c>
       <c r="H47" s="20" t="n">
         <f aca="false">D47*SUM($C$5:$C$7)</f>
-        <v>39600</v>
+        <v>3060</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16711,7 +17069,7 @@
       </c>
       <c r="H48" s="20" t="n">
         <f aca="false">D48*SUM($C$5:$C$7)</f>
-        <v>52800</v>
+        <v>4080</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16745,7 +17103,7 @@
       </c>
       <c r="H49" s="20" t="n">
         <f aca="false">D49*SUM($C$5:$C$7)</f>
-        <v>44000</v>
+        <v>3400</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16779,7 +17137,7 @@
       </c>
       <c r="H50" s="20" t="n">
         <f aca="false">D50*SUM($C$5:$C$7)</f>
-        <v>77000</v>
+        <v>5950</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16813,7 +17171,7 @@
       </c>
       <c r="H51" s="20" t="n">
         <f aca="false">D51*SUM($C$5:$C$7)</f>
-        <v>110000</v>
+        <v>8500</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16847,7 +17205,7 @@
       </c>
       <c r="H52" s="20" t="n">
         <f aca="false">D52*SUM($C$5:$C$7)</f>
-        <v>308000</v>
+        <v>23800</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16881,7 +17239,7 @@
       </c>
       <c r="H53" s="20" t="n">
         <f aca="false">D53*SUM($C$5:$C$7)</f>
-        <v>55000</v>
+        <v>4250</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16915,7 +17273,7 @@
       </c>
       <c r="H54" s="20" t="n">
         <f aca="false">D54*SUM($C$5:$C$7)</f>
-        <v>39600</v>
+        <v>3060</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16949,7 +17307,7 @@
       </c>
       <c r="H55" s="20" t="n">
         <f aca="false">D55*SUM($C$5:$C$7)</f>
-        <v>132000</v>
+        <v>10200</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16983,7 +17341,7 @@
       </c>
       <c r="H56" s="20" t="n">
         <f aca="false">D56*SUM($C$5:$C$7)</f>
-        <v>440000</v>
+        <v>34000</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16992,7 +17350,7 @@
       </c>
       <c r="H57" s="20" t="n">
         <f aca="false">SUM(H10:H56)</f>
-        <v>2341746</v>
+        <v>180953.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix Dokdo flag and cliff surf, Korean-layout shortcuts, cheaper quests, boss cancel, no tap-to-cast
- Dokdo: flag, building and lighthouse sit on the island slope; cliff gets a single foam wash instead of dotted streaks; sun glints moved off the cliff
- Shortcuts W/S/B/Space/1/2 also work with Korean input (ㅈ/ㄴ/ㅠ) and IME key events
- Quest rewards 4-7x expected catch value (was 10-16x); existing unclaimed quests scaled down
- Summoned boss can be cancelled before casting (tap panel again or B)
- Tapping the scene no longer casts, hooks or reels; only skips travel/landing
</commit_message>
<xml_diff>
--- a/bukangi-fishing-balance.xlsx
+++ b/bukangi-fishing-balance.xlsx
@@ -4548,10 +4548,10 @@
         <v>509</v>
       </c>
       <c r="B47" s="9" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="C47" s="9" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4599,11 +4599,11 @@
       </c>
       <c r="B52" s="20" t="n">
         <f aca="false">낚시터!F6*$B$47</f>
-        <v>229.060014687636</v>
+        <v>91.6240058750543</v>
       </c>
       <c r="C52" s="20" t="n">
         <f aca="false">낚시터!F6*$C$47</f>
-        <v>366.496023500217</v>
+        <v>160.342010281345</v>
       </c>
       <c r="D52" s="20" t="n">
         <f aca="false">낚시터!F6*$B$48</f>
@@ -4617,11 +4617,11 @@
       </c>
       <c r="B53" s="20" t="n">
         <f aca="false">낚시터!F7*$B$47</f>
-        <v>470.148669809363</v>
+        <v>188.059467923745</v>
       </c>
       <c r="C53" s="20" t="n">
         <f aca="false">낚시터!F7*$C$47</f>
-        <v>752.237871694981</v>
+        <v>329.104068866554</v>
       </c>
       <c r="D53" s="20" t="n">
         <f aca="false">낚시터!F7*$B$48</f>
@@ -4635,11 +4635,11 @@
       </c>
       <c r="B54" s="20" t="n">
         <f aca="false">낚시터!F8*$B$47</f>
-        <v>1222.21537481253</v>
+        <v>488.886149925011</v>
       </c>
       <c r="C54" s="20" t="n">
         <f aca="false">낚시터!F8*$C$47</f>
-        <v>1955.54459970004</v>
+        <v>855.550762368769</v>
       </c>
       <c r="D54" s="20" t="n">
         <f aca="false">낚시터!F8*$B$48</f>
@@ -4653,11 +4653,11 @@
       </c>
       <c r="B55" s="20" t="n">
         <f aca="false">낚시터!F9*$B$47</f>
-        <v>2694.29188313713</v>
+        <v>1077.71675325485</v>
       </c>
       <c r="C55" s="20" t="n">
         <f aca="false">낚시터!F9*$C$47</f>
-        <v>4310.8670130194</v>
+        <v>1886.00431819599</v>
       </c>
       <c r="D55" s="20" t="n">
         <f aca="false">낚시터!F9*$B$48</f>
@@ -4671,11 +4671,11 @@
       </c>
       <c r="B56" s="20" t="n">
         <f aca="false">낚시터!F10*$B$47</f>
-        <v>7582.69279988315</v>
+        <v>3033.07711995326</v>
       </c>
       <c r="C56" s="20" t="n">
         <f aca="false">낚시터!F10*$C$47</f>
-        <v>12132.308479813</v>
+        <v>5307.88495991821</v>
       </c>
       <c r="D56" s="20" t="n">
         <f aca="false">낚시터!F10*$B$48</f>
@@ -4689,11 +4689,11 @@
       </c>
       <c r="B57" s="20" t="n">
         <f aca="false">낚시터!F11*$B$47</f>
-        <v>12618.3027138793</v>
+        <v>5047.32108555171</v>
       </c>
       <c r="C57" s="20" t="n">
         <f aca="false">낚시터!F11*$C$47</f>
-        <v>20189.2843422068</v>
+        <v>8832.81189971549</v>
       </c>
       <c r="D57" s="20" t="n">
         <f aca="false">낚시터!F11*$B$48</f>
@@ -4707,11 +4707,11 @@
       </c>
       <c r="B58" s="20" t="n">
         <f aca="false">낚시터!F12*$B$47</f>
-        <v>20088.3703106896</v>
+        <v>8035.34812427582</v>
       </c>
       <c r="C58" s="20" t="n">
         <f aca="false">낚시터!F12*$C$47</f>
-        <v>32141.3924971033</v>
+        <v>14061.8592174827</v>
       </c>
       <c r="D58" s="20" t="n">
         <f aca="false">낚시터!F12*$B$48</f>

</xml_diff>

<commit_message>
Ease boss fights: lower difficulty (stream-river most) and give bosses the matching-method bonus with either method
</commit_message>
<xml_diff>
--- a/bukangi-fishing-balance.xlsx
+++ b/bukangi-fishing-balance.xlsx
@@ -15278,7 +15278,7 @@
         <v>30</v>
       </c>
       <c r="H7" s="22" t="n">
-        <v>0.74</v>
+        <v>0.62</v>
       </c>
       <c r="I7" s="27" t="n">
         <f aca="false">(D7+E7)/2</f>
@@ -15298,11 +15298,11 @@
       </c>
       <c r="M7" s="28" t="n">
         <f aca="false">0.08*H7^2*1.5</f>
-        <v>0.065712</v>
+        <v>0.046128</v>
       </c>
       <c r="N7" s="28" t="n">
         <f aca="false">0.28*H7^2*1.5</f>
-        <v>0.229992</v>
+        <v>0.161448</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15329,7 +15329,7 @@
         <v>30</v>
       </c>
       <c r="H8" s="22" t="n">
-        <v>0.8</v>
+        <v>0.66</v>
       </c>
       <c r="I8" s="27" t="n">
         <f aca="false">(D8+E8)/2</f>
@@ -15349,11 +15349,11 @@
       </c>
       <c r="M8" s="28" t="n">
         <f aca="false">0.08*H8^2*1.5</f>
-        <v>0.0768</v>
+        <v>0.052272</v>
       </c>
       <c r="N8" s="28" t="n">
         <f aca="false">0.28*H8^2*1.5</f>
-        <v>0.2688</v>
+        <v>0.182952</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15380,7 +15380,7 @@
         <v>30</v>
       </c>
       <c r="H9" s="22" t="n">
-        <v>0.86</v>
+        <v>0.74</v>
       </c>
       <c r="I9" s="27" t="n">
         <f aca="false">(D9+E9)/2</f>
@@ -15400,11 +15400,11 @@
       </c>
       <c r="M9" s="28" t="n">
         <f aca="false">0.08*H9^2*1.5</f>
-        <v>0.088752</v>
+        <v>0.065712</v>
       </c>
       <c r="N9" s="28" t="n">
         <f aca="false">0.28*H9^2*1.5</f>
-        <v>0.310632</v>
+        <v>0.229992</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15431,7 +15431,7 @@
         <v>30</v>
       </c>
       <c r="H10" s="22" t="n">
-        <v>0.9</v>
+        <v>0.84</v>
       </c>
       <c r="I10" s="27" t="n">
         <f aca="false">(D10+E10)/2</f>
@@ -15451,11 +15451,11 @@
       </c>
       <c r="M10" s="28" t="n">
         <f aca="false">0.08*H10^2*1.5</f>
-        <v>0.0972</v>
+        <v>0.084672</v>
       </c>
       <c r="N10" s="28" t="n">
         <f aca="false">0.28*H10^2*1.5</f>
-        <v>0.3402</v>
+        <v>0.296352</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15482,7 +15482,7 @@
         <v>30</v>
       </c>
       <c r="H11" s="22" t="n">
-        <v>0.94</v>
+        <v>0.91</v>
       </c>
       <c r="I11" s="27" t="n">
         <f aca="false">(D11+E11)/2</f>
@@ -15502,11 +15502,11 @@
       </c>
       <c r="M11" s="28" t="n">
         <f aca="false">0.08*H11^2*1.5</f>
-        <v>0.106032</v>
+        <v>0.099372</v>
       </c>
       <c r="N11" s="28" t="n">
         <f aca="false">0.28*H11^2*1.5</f>
-        <v>0.371112</v>
+        <v>0.347802</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15533,7 +15533,7 @@
         <v>30</v>
       </c>
       <c r="H12" s="22" t="n">
-        <v>0.98</v>
+        <v>0.96</v>
       </c>
       <c r="I12" s="27" t="n">
         <f aca="false">(D12+E12)/2</f>
@@ -15553,11 +15553,11 @@
       </c>
       <c r="M12" s="28" t="n">
         <f aca="false">0.08*H12^2*1.5</f>
-        <v>0.115248</v>
+        <v>0.110592</v>
       </c>
       <c r="N12" s="28" t="n">
         <f aca="false">0.28*H12^2*1.5</f>
-        <v>0.403368</v>
+        <v>0.387072</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15584,7 +15584,7 @@
         <v>30</v>
       </c>
       <c r="H13" s="22" t="n">
-        <v>1</v>
+        <v>0.99</v>
       </c>
       <c r="I13" s="27" t="n">
         <f aca="false">(D13+E13)/2</f>
@@ -15604,11 +15604,11 @@
       </c>
       <c r="M13" s="28" t="n">
         <f aca="false">0.08*H13^2*1.5</f>
-        <v>0.12</v>
+        <v>0.117612</v>
       </c>
       <c r="N13" s="28" t="n">
         <f aca="false">0.28*H13^2*1.5</f>
-        <v>0.42</v>
+        <v>0.411642</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Boss dives rarer and shorter: every ~8s/6s (was 4.5s/3.2s), 1.1s long (was 1.6s), stronger pull, 2.5s grace after a phase change
</commit_message>
<xml_diff>
--- a/bukangi-fishing-balance.xlsx
+++ b/bukangi-fishing-balance.xlsx
@@ -15301,8 +15301,8 @@
         <v>0.046128</v>
       </c>
       <c r="N7" s="28" t="n">
-        <f aca="false">0.28*H7^2*1.5</f>
-        <v>0.161448</v>
+        <f aca="false">0.38*H7^2*1.5</f>
+        <v>0.219108</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15352,8 +15352,8 @@
         <v>0.052272</v>
       </c>
       <c r="N8" s="28" t="n">
-        <f aca="false">0.28*H8^2*1.5</f>
-        <v>0.182952</v>
+        <f aca="false">0.38*H8^2*1.5</f>
+        <v>0.248292</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15403,8 +15403,8 @@
         <v>0.065712</v>
       </c>
       <c r="N9" s="28" t="n">
-        <f aca="false">0.28*H9^2*1.5</f>
-        <v>0.229992</v>
+        <f aca="false">0.38*H9^2*1.5</f>
+        <v>0.312132</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15454,8 +15454,8 @@
         <v>0.084672</v>
       </c>
       <c r="N10" s="28" t="n">
-        <f aca="false">0.28*H10^2*1.5</f>
-        <v>0.296352</v>
+        <f aca="false">0.38*H10^2*1.5</f>
+        <v>0.402192</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15505,8 +15505,8 @@
         <v>0.099372</v>
       </c>
       <c r="N11" s="28" t="n">
-        <f aca="false">0.28*H11^2*1.5</f>
-        <v>0.347802</v>
+        <f aca="false">0.38*H11^2*1.5</f>
+        <v>0.472017</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15556,8 +15556,8 @@
         <v>0.110592</v>
       </c>
       <c r="N12" s="28" t="n">
-        <f aca="false">0.28*H12^2*1.5</f>
-        <v>0.387072</v>
+        <f aca="false">0.38*H12^2*1.5</f>
+        <v>0.525312</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15607,8 +15607,8 @@
         <v>0.117612</v>
       </c>
       <c r="N13" s="28" t="n">
-        <f aca="false">0.28*H13^2*1.5</f>
-        <v>0.411642</v>
+        <f aca="false">0.38*H13^2*1.5</f>
+        <v>0.558657</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Prestige: replace boss-meter bonus with wider tension zone (+0.02/lv) and more burst absorb (+4%/lv), capped at 5 levels
</commit_message>
<xml_diff>
--- a/bukangi-fishing-balance.xlsx
+++ b/bukangi-fishing-balance.xlsx
@@ -142,7 +142,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B50" authorId="0">
+    <comment ref="B52" authorId="0">
       <text>
         <r>
           <rPr>
@@ -583,7 +583,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="867" uniqueCount="555">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="871" uniqueCount="559">
   <si>
     <t xml:space="preserve">부캉이 낚시터 밸런스 요약</t>
   </si>
@@ -2143,7 +2143,13 @@
     <t xml:space="preserve">레벨당 판매가 보너스</t>
   </si>
   <si>
-    <t xml:space="preserve">레벨당 보스 기척 보너스</t>
+    <t xml:space="preserve">레벨당 장력 초록 구간 (낚싯대 구간에 더함)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">레벨당 돌진 흡수 (릴낚시 들기)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">구간·흡수가 쌓이는 최대 레벨</t>
   </si>
   <si>
     <t xml:space="preserve">환생 후 시작 금액 (원)</t>
@@ -2152,7 +2158,14 @@
     <t xml:space="preserve">환생 레벨</t>
   </si>
   <si>
-    <t xml:space="preserve">보스 기척 1마리당</t>
+    <t xml:space="preserve">초록 구간 추가</t>
+  </si>
+  <si>
+    <t xml:space="preserve">돌진 흡수 추가</t>
+  </si>
+  <si>
+    <t xml:space="preserve">최고 낚싯대 구간
+(전설의 장대 +5)</t>
   </si>
   <si>
     <t xml:space="preserve">오늘의 의뢰 (하루 3개, 연 낚시터 중 가장 먼 2곳 기준. 새 낚시터를 열면 못 끝낸 의뢰가 바뀜)</t>
@@ -3922,7 +3935,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G72"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="36"/>
@@ -4450,358 +4463,420 @@
       <c r="A37" s="4" t="s">
         <v>504</v>
       </c>
-      <c r="B37" s="21" t="n">
-        <v>0.1</v>
+      <c r="B37" s="22" t="n">
+        <v>0.02</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
         <v>505</v>
       </c>
-      <c r="B38" s="12" t="n">
+      <c r="B38" s="21" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="4" t="s">
+        <v>506</v>
+      </c>
+      <c r="B39" s="9" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="4" t="s">
+        <v>507</v>
+      </c>
+      <c r="B40" s="12" t="n">
         <v>150</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="3" t="s">
-        <v>506</v>
-      </c>
-      <c r="B39" s="3" t="s">
+    <row r="41" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="3" t="s">
+        <v>508</v>
+      </c>
+      <c r="B41" s="3" t="s">
         <v>447</v>
       </c>
-      <c r="C39" s="3" t="s">
-        <v>507</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="B40" s="28" t="n">
-        <f aca="false">1+A40*$B$36</f>
-        <v>1.1</v>
-      </c>
-      <c r="C40" s="28" t="n">
-        <f aca="false">1+A40*$B$37</f>
-        <v>1.1</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="B41" s="28" t="n">
-        <f aca="false">1+A41*$B$36</f>
-        <v>1.2</v>
-      </c>
-      <c r="C41" s="28" t="n">
-        <f aca="false">1+A41*$B$37</f>
-        <v>1.2</v>
+      <c r="C41" s="3" t="s">
+        <v>509</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>510</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>511</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B42" s="28" t="n">
         <f aca="false">1+A42*$B$36</f>
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="C42" s="28" t="n">
-        <f aca="false">1+A42*$B$37</f>
-        <v>1.3</v>
+        <f aca="false">MIN(A42,$B$39)*$B$37</f>
+        <v>0.02</v>
+      </c>
+      <c r="D42" s="36" t="n">
+        <f aca="false">MIN(A42,$B$39)*$B$38</f>
+        <v>0.04</v>
+      </c>
+      <c r="E42" s="28" t="n">
+        <f aca="false">0.51+C42</f>
+        <v>0.53</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B43" s="28" t="n">
         <f aca="false">1+A43*$B$36</f>
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="C43" s="28" t="n">
-        <f aca="false">1+A43*$B$37</f>
-        <v>1.4</v>
+        <f aca="false">MIN(A43,$B$39)*$B$37</f>
+        <v>0.04</v>
+      </c>
+      <c r="D43" s="36" t="n">
+        <f aca="false">MIN(A43,$B$39)*$B$38</f>
+        <v>0.08</v>
+      </c>
+      <c r="E43" s="28" t="n">
+        <f aca="false">0.51+C43</f>
+        <v>0.55</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="14" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B44" s="28" t="n">
         <f aca="false">1+A44*$B$36</f>
+        <v>1.3</v>
+      </c>
+      <c r="C44" s="28" t="n">
+        <f aca="false">MIN(A44,$B$39)*$B$37</f>
+        <v>0.06</v>
+      </c>
+      <c r="D44" s="36" t="n">
+        <f aca="false">MIN(A44,$B$39)*$B$38</f>
+        <v>0.12</v>
+      </c>
+      <c r="E44" s="28" t="n">
+        <f aca="false">0.51+C44</f>
+        <v>0.57</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="B45" s="28" t="n">
+        <f aca="false">1+A45*$B$36</f>
+        <v>1.4</v>
+      </c>
+      <c r="C45" s="28" t="n">
+        <f aca="false">MIN(A45,$B$39)*$B$37</f>
+        <v>0.08</v>
+      </c>
+      <c r="D45" s="36" t="n">
+        <f aca="false">MIN(A45,$B$39)*$B$38</f>
+        <v>0.16</v>
+      </c>
+      <c r="E45" s="28" t="n">
+        <f aca="false">0.51+C45</f>
+        <v>0.59</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="B46" s="28" t="n">
+        <f aca="false">1+A46*$B$36</f>
         <v>1.5</v>
       </c>
-      <c r="C44" s="28" t="n">
-        <f aca="false">1+A44*$B$37</f>
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="30" t="s">
-        <v>508</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="4" t="s">
-        <v>509</v>
-      </c>
-      <c r="B47" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="C47" s="9" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="4" t="s">
-        <v>510</v>
-      </c>
-      <c r="B48" s="9" t="n">
-        <v>25</v>
+      <c r="C46" s="28" t="n">
+        <f aca="false">MIN(A46,$B$39)*$B$37</f>
+        <v>0.1</v>
+      </c>
+      <c r="D46" s="36" t="n">
+        <f aca="false">MIN(A46,$B$39)*$B$38</f>
+        <v>0.2</v>
+      </c>
+      <c r="E46" s="28" t="n">
+        <f aca="false">0.51+C46</f>
+        <v>0.61</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="30" t="s">
+        <v>512</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="4" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="B49" s="9" t="n">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="C49" s="9" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="4" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="B50" s="9" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="4" t="s">
+        <v>515</v>
+      </c>
+      <c r="B51" s="9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="4" t="s">
+        <v>516</v>
+      </c>
+      <c r="B52" s="9" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="3" t="s">
-        <v>513</v>
-      </c>
-      <c r="B51" s="3" t="s">
-        <v>514</v>
-      </c>
-      <c r="C51" s="3" t="s">
-        <v>515</v>
-      </c>
-      <c r="D51" s="3" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="31" t="str">
+    <row r="53" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="3" t="s">
+        <v>517</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>518</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>519</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="31" t="str">
         <f aca="false">낚시터!B6</f>
         <v>하천</v>
       </c>
-      <c r="B52" s="20" t="n">
-        <f aca="false">낚시터!F6*$B$47</f>
+      <c r="B54" s="20" t="n">
+        <f aca="false">낚시터!F6*$B$49</f>
         <v>91.6240058750543</v>
       </c>
-      <c r="C52" s="20" t="n">
-        <f aca="false">낚시터!F6*$C$47</f>
+      <c r="C54" s="20" t="n">
+        <f aca="false">낚시터!F6*$C$49</f>
         <v>160.342010281345</v>
       </c>
-      <c r="D52" s="20" t="n">
-        <f aca="false">낚시터!F6*$B$48</f>
+      <c r="D54" s="20" t="n">
+        <f aca="false">낚시터!F6*$B$50</f>
         <v>572.650036719089</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="31" t="str">
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="31" t="str">
         <f aca="false">낚시터!B7</f>
         <v>강</v>
       </c>
-      <c r="B53" s="20" t="n">
-        <f aca="false">낚시터!F7*$B$47</f>
+      <c r="B55" s="20" t="n">
+        <f aca="false">낚시터!F7*$B$49</f>
         <v>188.059467923745</v>
       </c>
-      <c r="C53" s="20" t="n">
-        <f aca="false">낚시터!F7*$C$47</f>
+      <c r="C55" s="20" t="n">
+        <f aca="false">낚시터!F7*$C$49</f>
         <v>329.104068866554</v>
       </c>
-      <c r="D53" s="20" t="n">
-        <f aca="false">낚시터!F7*$B$48</f>
+      <c r="D55" s="20" t="n">
+        <f aca="false">낚시터!F7*$B$50</f>
         <v>1175.37167452341</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="31" t="str">
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="31" t="str">
         <f aca="false">낚시터!B8</f>
         <v>방파제</v>
       </c>
-      <c r="B54" s="20" t="n">
-        <f aca="false">낚시터!F8*$B$47</f>
+      <c r="B56" s="20" t="n">
+        <f aca="false">낚시터!F8*$B$49</f>
         <v>488.886149925011</v>
       </c>
-      <c r="C54" s="20" t="n">
-        <f aca="false">낚시터!F8*$C$47</f>
+      <c r="C56" s="20" t="n">
+        <f aca="false">낚시터!F8*$C$49</f>
         <v>855.550762368769</v>
       </c>
-      <c r="D54" s="20" t="n">
-        <f aca="false">낚시터!F8*$B$48</f>
+      <c r="D56" s="20" t="n">
+        <f aca="false">낚시터!F8*$B$50</f>
         <v>3055.53843703132</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="31" t="str">
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="31" t="str">
         <f aca="false">낚시터!B9</f>
         <v>독도</v>
       </c>
-      <c r="B55" s="20" t="n">
-        <f aca="false">낚시터!F9*$B$47</f>
+      <c r="B57" s="20" t="n">
+        <f aca="false">낚시터!F9*$B$49</f>
         <v>1077.71675325485</v>
       </c>
-      <c r="C55" s="20" t="n">
-        <f aca="false">낚시터!F9*$C$47</f>
+      <c r="C57" s="20" t="n">
+        <f aca="false">낚시터!F9*$C$49</f>
         <v>1886.00431819599</v>
       </c>
-      <c r="D55" s="20" t="n">
-        <f aca="false">낚시터!F9*$B$48</f>
+      <c r="D57" s="20" t="n">
+        <f aca="false">낚시터!F9*$B$50</f>
         <v>6735.72970784282</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="31" t="str">
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="31" t="str">
         <f aca="false">낚시터!B10</f>
         <v>배낚시</v>
       </c>
-      <c r="B56" s="20" t="n">
-        <f aca="false">낚시터!F10*$B$47</f>
+      <c r="B58" s="20" t="n">
+        <f aca="false">낚시터!F10*$B$49</f>
         <v>3033.07711995326</v>
       </c>
-      <c r="C56" s="20" t="n">
-        <f aca="false">낚시터!F10*$C$47</f>
+      <c r="C58" s="20" t="n">
+        <f aca="false">낚시터!F10*$C$49</f>
         <v>5307.88495991821</v>
       </c>
-      <c r="D56" s="20" t="n">
-        <f aca="false">낚시터!F10*$B$48</f>
+      <c r="D58" s="20" t="n">
+        <f aca="false">낚시터!F10*$B$50</f>
         <v>18956.7319997079</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="31" t="str">
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="31" t="str">
         <f aca="false">낚시터!B11</f>
         <v>아마존</v>
       </c>
-      <c r="B57" s="20" t="n">
-        <f aca="false">낚시터!F11*$B$47</f>
+      <c r="B59" s="20" t="n">
+        <f aca="false">낚시터!F11*$B$49</f>
         <v>5047.32108555171</v>
       </c>
-      <c r="C57" s="20" t="n">
-        <f aca="false">낚시터!F11*$C$47</f>
+      <c r="C59" s="20" t="n">
+        <f aca="false">낚시터!F11*$C$49</f>
         <v>8832.81189971549</v>
       </c>
-      <c r="D57" s="20" t="n">
-        <f aca="false">낚시터!F11*$B$48</f>
+      <c r="D59" s="20" t="n">
+        <f aca="false">낚시터!F11*$B$50</f>
         <v>31545.7567846982</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="31" t="str">
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="31" t="str">
         <f aca="false">낚시터!B12</f>
         <v>알래스카</v>
       </c>
-      <c r="B58" s="20" t="n">
-        <f aca="false">낚시터!F12*$B$47</f>
+      <c r="B60" s="20" t="n">
+        <f aca="false">낚시터!F12*$B$49</f>
         <v>8035.34812427582</v>
       </c>
-      <c r="C58" s="20" t="n">
-        <f aca="false">낚시터!F12*$C$47</f>
+      <c r="C60" s="20" t="n">
+        <f aca="false">낚시터!F12*$C$49</f>
         <v>14061.8592174827</v>
       </c>
-      <c r="D58" s="20" t="n">
-        <f aca="false">낚시터!F12*$B$48</f>
+      <c r="D60" s="20" t="n">
+        <f aca="false">낚시터!F12*$B$50</f>
         <v>50220.9257767239</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="30" t="s">
-        <v>517</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="4" t="s">
-        <v>518</v>
-      </c>
-      <c r="B61" s="10" t="n">
-        <v>0.01</v>
-      </c>
-    </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="4" t="s">
-        <v>519</v>
-      </c>
-      <c r="B62" s="10" t="n">
-        <v>0.01</v>
+      <c r="A62" s="30" t="s">
+        <v>521</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="4" t="s">
-        <v>520</v>
-      </c>
-      <c r="B63" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="C63" s="37" t="n">
-        <v>5</v>
+        <v>522</v>
+      </c>
+      <c r="B63" s="10" t="n">
+        <v>0.01</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="4" t="s">
-        <v>521</v>
-      </c>
-      <c r="B64" s="21" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="C64" s="37" t="n">
-        <v>3</v>
+        <v>523</v>
+      </c>
+      <c r="B64" s="10" t="n">
+        <v>0.01</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="4" t="s">
-        <v>522</v>
-      </c>
-      <c r="B65" s="29" t="n">
-        <f aca="false">$B$61</f>
-        <v>0.01</v>
+        <v>524</v>
+      </c>
+      <c r="B65" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C65" s="37" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="4" t="s">
-        <v>523</v>
-      </c>
-      <c r="B66" s="29" t="n">
-        <f aca="false">$B$61+1.3*$B$62</f>
+        <v>525</v>
+      </c>
+      <c r="B66" s="21" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C66" s="37" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="4" t="s">
+        <v>526</v>
+      </c>
+      <c r="B67" s="29" t="n">
+        <f aca="false">$B$63</f>
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="4" t="s">
+        <v>527</v>
+      </c>
+      <c r="B68" s="29" t="n">
+        <f aca="false">$B$63+1.3*$B$64</f>
         <v>0.023</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="30" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="4" t="s">
-        <v>525</v>
-      </c>
-      <c r="B69" s="9" t="n">
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="30" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="4" t="s">
+        <v>529</v>
+      </c>
+      <c r="B71" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="C69" s="4" t="str">
-        <f aca="false">IF(B69&lt;0,"끔",INDEX(등급!$A$4:$A$8,B69+1))</f>
+      <c r="C71" s="4" t="str">
+        <f aca="false">IF(B71&lt;0,"끔",INDEX(등급!$A$4:$A$8,B71+1))</f>
         <v>고급</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="4" t="s">
-        <v>526</v>
-      </c>
-      <c r="B70" s="4" t="s">
-        <v>527</v>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="4" t="s">
+        <v>530</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>531</v>
       </c>
     </row>
   </sheetData>
@@ -4834,12 +4909,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>529</v>
+        <v>533</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4847,19 +4922,19 @@
         <v>312</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>530</v>
+        <v>534</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>531</v>
+        <v>535</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>532</v>
+        <v>536</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>129</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>533</v>
+        <v>537</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4870,16 +4945,16 @@
         <v>3</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>534</v>
+        <v>538</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="E5" s="21" t="n">
         <v>0.15</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>536</v>
+        <v>540</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4890,16 +4965,16 @@
         <v>6</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>537</v>
+        <v>541</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="E6" s="21" t="n">
         <v>0.05</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>539</v>
+        <v>543</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4910,16 +4985,16 @@
         <v>7</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>540</v>
+        <v>544</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>541</v>
+        <v>545</v>
       </c>
       <c r="E7" s="21" t="n">
         <v>0.1</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>542</v>
+        <v>546</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4930,16 +5005,16 @@
         <v>8</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>544</v>
+        <v>548</v>
       </c>
       <c r="E8" s="32" t="n">
         <v>0.3</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>545</v>
+        <v>549</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4950,16 +5025,16 @@
         <v>7</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>546</v>
+        <v>550</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>541</v>
+        <v>545</v>
       </c>
       <c r="E9" s="21" t="n">
         <v>0.05</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>542</v>
+        <v>546</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4970,16 +5045,16 @@
         <v>6</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>547</v>
+        <v>551</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>548</v>
+        <v>552</v>
       </c>
       <c r="E10" s="21" t="n">
         <v>0.1</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>549</v>
+        <v>553</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4990,16 +5065,16 @@
         <v>6</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>550</v>
+        <v>554</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>544</v>
+        <v>548</v>
       </c>
       <c r="E11" s="32" t="n">
         <v>0.2</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>545</v>
+        <v>549</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5010,16 +5085,16 @@
         <v>7</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>551</v>
+        <v>555</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>548</v>
+        <v>552</v>
       </c>
       <c r="E12" s="21" t="n">
         <v>0.05</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>549</v>
+        <v>553</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5030,16 +5105,16 @@
         <v>7</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>552</v>
+        <v>556</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>553</v>
+        <v>557</v>
       </c>
       <c r="E13" s="35" t="n">
         <v>30</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
     </row>
   </sheetData>

</xml_diff>